<commit_message>
Update news 2026-07-14 17:34
</commit_message>
<xml_diff>
--- a/Noticias_Calcario_20260714.xlsx
+++ b/Noticias_Calcario_20260714.xlsx
@@ -2888,7 +2888,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Alta do enxofre afeta produção e gera demissões em Araxá - G1</t>
+          <t>Alta do enxofre provoca crise na produção de fertilizantes em Minas Gerais - G1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPdDlyUTJPY3lkTzRodWhvRVhRTjB1RHlEX2lGcWJxcHFQQlRjamRIY0VIYnhjWlVXVjFWQmtYOTQtSGhsU0NYbGZmSjVYX0Z0NVJXdEVfNzM2OHQwQl9uRG5oUElfbUtjblNEMl9VWWJQUTdoTEVFYkhnZWxNTFpHR1NOVm9TTU12eE1xR3pjak95YkFzWHpNN3ZKUmFvdjZEaFk3MkwxNXhMb1NLSTFaUDdJUlk5MWlpdW1OYnNuMkhZYzQ1cDQtRkd6cnMza0xNbHRQRHg3ZW5NbmVENjNaeUpQN1JOVUnSAfYBQVVfeXFMT1B5bkdkT0s0YXRtRzF5RS1pNDFXQTlLZHhrQnVZbU5RM3V2R2J2UW81a3NQOE8zd1VBcmtFbUNiRnlPaDA3LTlIT25DZ3dhOE9wRksxRXE5eEJaV2xLSVZ4OFowMFN5SzF3OU4tajdDdjFfVEFvZTFXVDl2dmdQZHVHd1drUjdOOVc4TlhDZmhhT0h6RmlWQ1M2ckxJMGxPWXZFVUl5WnJudzJIM2NoWkhUa3ptb1pGVUszN0RjRGN2TjN4aExoV202enh1OEdYOWJRdmhhTldhcFAxeHFydnFPU2VFXzdCblVIYmJnSWoxOXRCaEpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxQYnY2QmNpaXc4aHRDMDFLUmxTNzhRME9pNWhac1psdWtNMXMwSHJsN3oxeUJqNXZtOHVNWUNaQnNjOUJaLWRhbF91M05Sa3VIM3dsTjM2X2VLSS03ZTlPWFF4T2xLMUdzTlZLdk9tblk1WHRZUWtGT3BmUktDODYzMU1VUTEtbVc3N0VTelc4ZUROZDBkX2xZeFlma01wMjV3WHBISVdRQ0lwYmFseFA5d1ZnNXdFMVpRUk9zeHJpbEUzQ1Y0MUdpbXdiTnlSZ3o2ekJfbnZOYlNJU29nU2FaclhFR1ZqUmFx0gH3AUFVX3lxTE1sQjBVb2UzRGxTdGVBTXd6Y0lwX0pBUmYtOXIxYmU3b2EtLUtLYklfS3FHcHp3VklkU0xtdjlwMHAxYzJtNmcwNHkzOUd6TFBZZVkxa1VWVmJBRFZKLXFSLUpxQnc5al8ySjRJQkNFUnpWRXlmbTctMlp4SXd4OUJSai00ZGxocEd6dUVZbE8zZ0JXaDJ2SEllampRdER2aF9IRlBoMDZ4SHZ4UXhqT1RVYVV5ekFOSTVyUkgxQ0RJNzQ2N2ZfQThQR182WUVGQ2ZVNHBKOUtuVktNNG5LTVBnX2tUbGNHNzhOQkpuMEhjR2RBTHJYVkk?oc=5</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Alta do enxofre provoca crise na produção de fertilizantes em Minas Gerais - G1</t>
+          <t>Alta do enxofre afeta produção e gera demissões em Araxá - G1</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxQYnY2QmNpaXc4aHRDMDFLUmxTNzhRME9pNWhac1psdWtNMXMwSHJsN3oxeUJqNXZtOHVNWUNaQnNjOUJaLWRhbF91M05Sa3VIM3dsTjM2X2VLSS03ZTlPWFF4T2xLMUdzTlZLdk9tblk1WHRZUWtGT3BmUktDODYzMU1VUTEtbVc3N0VTelc4ZUROZDBkX2xZeFlma01wMjV3WHBISVdRQ0lwYmFseFA5d1ZnNXdFMVpRUk9zeHJpbEUzQ1Y0MUdpbXdiTnlSZ3o2ekJfbnZOYlNJU29nU2FaclhFR1ZqUmFx0gH3AUFVX3lxTE1sQjBVb2UzRGxTdGVBTXd6Y0lwX0pBUmYtOXIxYmU3b2EtLUtLYklfS3FHcHp3VklkU0xtdjlwMHAxYzJtNmcwNHkzOUd6TFBZZVkxa1VWVmJBRFZKLXFSLUpxQnc5al8ySjRJQkNFUnpWRXlmbTctMlp4SXd4OUJSai00ZGxocEd6dUVZbE8zZ0JXaDJ2SEllampRdER2aF9IRlBoMDZ4SHZ4UXhqT1RVYVV5ekFOSTVyUkgxQ0RJNzQ2N2ZfQThQR182WUVGQ2ZVNHBKOUtuVktNNG5LTVBnX2tUbGNHNzhOQkpuMEhjR2RBTHJYVkk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPdDlyUTJPY3lkTzRodWhvRVhRTjB1RHlEX2lGcWJxcHFQQlRjamRIY0VIYnhjWlVXVjFWQmtYOTQtSGhsU0NYbGZmSjVYX0Z0NVJXdEVfNzM2OHQwQl9uRG5oUElfbUtjblNEMl9VWWJQUTdoTEVFYkhnZWxNTFpHR1NOVm9TTU12eE1xR3pjak95YkFzWHpNN3ZKUmFvdjZEaFk3MkwxNXhMb1NLSTFaUDdJUlk5MWlpdW1OYnNuMkhZYzQ1cDQtRkd6cnMza0xNbHRQRHg3ZW5NbmVENjNaeUpQN1JOVUnSAfYBQVVfeXFMT1B5bkdkT0s0YXRtRzF5RS1pNDFXQTlLZHhrQnVZbU5RM3V2R2J2UW81a3NQOE8zd1VBcmtFbUNiRnlPaDA3LTlIT25DZ3dhOE9wRksxRXE5eEJaV2xLSVZ4OFowMFN5SzF3OU4tajdDdjFfVEFvZTFXVDl2dmdQZHVHd1drUjdOOVc4TlhDZmhhT0h6RmlWQ1M2ckxJMGxPWXZFVUl5WnJudzJIM2NoWkhUa3ptb1pGVUszN0RjRGN2TjN4aExoV202enh1OEdYOWJRdmhhTldhcFAxeHFydnFPU2VFXzdCblVIYmJnSWoxOXRCaEpB?oc=5</t>
         </is>
       </c>
     </row>
@@ -3103,12 +3103,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Mosaic enfrenta pressão após Casa Branca suspender tarifas sobre Marrocos - Investing.com Brasil - Finanças, Câmbio e Investimentos</t>
+          <t>Mercado de fertilizantes amplia movimento de baixa com recuo da ureia, MAP e cloreto de potássio - Notícias Agrícolas</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3118,19 +3118,19 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQU1JyUHczQlZyM01aNnp4dHJSLWNUNHRvU3FfY0ZYWHRNUkVpRkM1V3VOcVZhME1Kb2Q1a0ZwUXNzUDNDeDBKSUhGdVoxOUxCUjZkb2pKOFI5OC1aUGdQbVVRSGY4RjRfZVJZV0xxSXd0U3o1VmtGeHAxYl94eHVQOFlMQm5nRk1qX0g3MW5YUWdnV0JlTGVvZy1ibDI1OFhoVmt0RmZiaFRRTDBLMW1lNl8tM1U0LVVRVV9ESURZcGhuMThaeWpFcDQ1blR0ZzA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQcWo1blNvbFFwUzl4S0hfaW9sSklENjRLa1M4UzNSNXg5aFd0aWNQUjFhLTNmRDYxZWk1Mlp5WXdRNjZNd1RveGNDbkNsa0o5R1dRM1RTMGFpVUhHYzk3Qms5a09jOVdEX1A0cjZVWmU3SHQ1d29zbHZYeTI4MWpRS19mUFVadUpwY2NQMjJwTzZGMk9HTW82OHVzZHhtbHVQcFpseG83Z2xQUGlKb29NbkxVNHZWQ29SeTVQN01meGFlVV9ZSW9UaVU1azdIOFh6V0JhcktVVzJDblRKNGNYQTNKWnBzVGhRR25xdy1MRTZWMzdlV0J2eNIB_gFBVV95cUxOMWY5TFpKa0RFNVpidGRSdFBOeUczUDduTWxqLUpMWmg4cUxra2N6RF91bTd4MHBlMmluQXNBTE9PTi03WlFRQWNCdUU5NTZaNXV3UTVhclgtaUtva1gxYjZncmtES3V3LVFQcHpCLXoydmtXSXZwOFlfSDhYOUVmbEpETEQ2SkM4cHgyTHBBUTZxUExpTkEtYm5FTjJGLTFJSXBnQzBNNWZmd3M1N2hiRUw0OTNNVU9ra2hJRnIweXR1ZnZfN0RjM2d0c21TRTlteC1rMzA0a2Q2TnlORTFOUEJaRG03Nk1sNkVYNnhtSTJCMm5YWnZ6ZmZjRlo1QQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Mercado de fertilizantes amplia movimento de baixa com recuo da ureia, MAP e cloreto de potássio - Notícias Agrícolas</t>
+          <t>Mosaic enfrenta pressão após Casa Branca suspender tarifas sobre Marrocos - Investing.com Brasil - Finanças, Câmbio e Investimentos</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQcWo1blNvbFFwUzl4S0hfaW9sSklENjRLa1M4UzNSNXg5aFd0aWNQUjFhLTNmRDYxZWk1Mlp5WXdRNjZNd1RveGNDbkNsa0o5R1dRM1RTMGFpVUhHYzk3Qms5a09jOVdEX1A0cjZVWmU3SHQ1d29zbHZYeTI4MWpRS19mUFVadUpwY2NQMjJwTzZGMk9HTW82OHVzZHhtbHVQcFpseG83Z2xQUGlKb29NbkxVNHZWQ29SeTVQN01meGFlVV9ZSW9UaVU1azdIOFh6V0JhcktVVzJDblRKNGNYQTNKWnBzVGhRR25xdy1MRTZWMzdlV0J2eNIB_gFBVV95cUxOMWY5TFpKa0RFNVpidGRSdFBOeUczUDduTWxqLUpMWmg4cUxra2N6RF91bTd4MHBlMmluQXNBTE9PTi03WlFRQWNCdUU5NTZaNXV3UTVhclgtaUtva1gxYjZncmtES3V3LVFQcHpCLXoydmtXSXZwOFlfSDhYOUVmbEpETEQ2SkM4cHgyTHBBUTZxUExpTkEtYm5FTjJGLTFJSXBnQzBNNWZmd3M1N2hiRUw0OTNNVU9ra2hJRnIweXR1ZnZfN0RjM2d0c21TRTlteC1rMzA0a2Q2TnlORTFOUEJaRG03Nk1sNkVYNnhtSTJCMm5YWnZ6ZmZjRlo1QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQU1JyUHczQlZyM01aNnp4dHJSLWNUNHRvU3FfY0ZYWHRNUkVpRkM1V3VOcVZhME1Kb2Q1a0ZwUXNzUDNDeDBKSUhGdVoxOUxCUjZkb2pKOFI5OC1aUGdQbVVRSGY4RjRfZVJZV0xxSXd0U3o1VmtGeHAxYl94eHVQOFlMQm5nRk1qX0g3MW5YUWdnV0JlTGVvZy1ibDI1OFhoVmt0RmZiaFRRTDBLMW1lNl8tM1U0LVVRVV9ESURZcGhuMThaeWpFcDQ1blR0ZzA?oc=5</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Martin Marietta anuncia aquisição da Lhoist North America por US$ 13,5 bilhões - Investing.com Brasil - Finanças, Câmbio e Investimentos</t>
+          <t>Martin Marietta confirma acordo de US$ 13,5 bilhões pela Lhoist North America - Investing.com Brasil - Finanças, Câmbio e Investimentos</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNYXg3YkM0VFFac3BVN0QwMmZqYm9rQW9XM1ppUzRJTl85Y3FkMEhHSFY1Q0NON2pxTE9uTUNob0N1bkw5bFA5Y002X1VVTzdLT1JmdDFGUk16cDBJaEc1eFdLdlZwNWYtZXFxVnVjUnA5QlhWaGhFZmJUalBLQXpJZFF2TmpmVjZfZFM4THVXQndEUUlZYnI4X3FLY1VoQ2tNY1NyNFVZVkpaSmdxanJwQTVxcGJCNmxtOTBOZklvY3JlbzQtM2NMX0NRZmY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNYUJCZDhUVml3MGVqMUw2QllsRmVrTF90WjJCYjhGUEtuVlVpc2hRNzJ6UzhJaDd3a1lnU0MtYnFGUGU4SmxNb1Jwc0hpZnJubUpVQ1U3UjhGYkk2a2VtRFg0Vl9mYWt4aXIxYV9xZF9SM29OcFhPdUJaVWVMQlcxcERTay1YODdGaVNMT2owWWdYeWNEWW5KbHk1Q19sTllKMng2T1lNNTBTZFAxRW5nV1pid2tZNnRzejJCc3M3SURsdGFXQnJGazhZRQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Martin Marietta confirma acordo de US$ 13,5 bilhões pela Lhoist North America - Investing.com Brasil - Finanças, Câmbio e Investimentos</t>
+          <t>Martin Marietta anuncia aquisição da Lhoist North America por US$ 13,5 bilhões - Investing.com Brasil - Finanças, Câmbio e Investimentos</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3206,19 +3206,19 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNYUJCZDhUVml3MGVqMUw2QllsRmVrTF90WjJCYjhGUEtuVlVpc2hRNzJ6UzhJaDd3a1lnU0MtYnFGUGU4SmxNb1Jwc0hpZnJubUpVQ1U3UjhGYkk2a2VtRFg0Vl9mYWt4aXIxYV9xZF9SM29OcFhPdUJaVWVMQlcxcERTay1YODdGaVNMT2owWWdYeWNEWW5KbHk1Q19sTllKMng2T1lNNTBTZFAxRW5nV1pid2tZNnRzejJCc3M3SURsdGFXQnJGazhZRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNYXg3YkM0VFFac3BVN0QwMmZqYm9rQW9XM1ppUzRJTl85Y3FkMEhHSFY1Q0NON2pxTE9uTUNob0N1bkw5bFA5Y002X1VVTzdLT1JmdDFGUk16cDBJaEc1eFdLdlZwNWYtZXFxVnVjUnA5QlhWaGhFZmJUalBLQXpJZFF2TmpmVjZfZFM4THVXQndEUUlZYnI4X3FLY1VoQ2tNY1NyNFVZVkpaSmdxanJwQTVxcGJCNmxtOTBOZklvY3JlbzQtM2NMX0NRZmY?oc=5</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Lhoist</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Com foco em data centers, Martin Marietta acerta compra de fornecedora de minerais por US$ 13,5 bi - Valor Econômico</t>
+          <t>Ureia, MAP e potássio registram queda no Brasil - Agrolink</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxOQmNERDdXd2o0VlYxZXE2aDRFUV90bEdkWTd6ZUwyNjhJMDZBV20xbWxWZ2V6VGVtZG83VHFjSnVDU3ppbUZpTm1tY3NSWUNmRFhxeW5VaEp2SHp3c1BjVkxQZXBNZEhrd2RUdHVKZUNFTHlHZFliODlHMHp4c3lMbXhVUkhqWjltOFRzUVlJMU9Da0RIZnk2Y3B6bUVTelRSZ2tUT0c1aFVZamlSTERiX2ZIa1puUnVrUlQ1aDhtRW1uLVBZZ0NSSU91RGpPY243OWVLOXp3TGNjU0pKR015dFQ2RGI1dDdO0gH3AUFVX3lxTE1jZVlGVWNwdWlxX2lGVGpRTnRPUXJJNTJWbXJTcXRjb3lQQVFNT3A5TVhPM2xpSmRNOVZKZmFFR3Y5eEJnRlRNX0taNmppMTdVT1dBeDRKVjQ2TzNPZHR0OEhBRWlmM3VBaWcwQjVzSDZmM1hVNmJTcVVRR1VGYzkxY2trZ3FXMjNpNzlnUkRxLXB6UG0xbVBFZmU5MVVIa3FVZkdSMFFwaGhBeGZna01zOVNwUGFKMXpQdkstaWhud1RxVEJXUXVFdmt1bXdjNHF3azh6Vi0zSG1tbzE0aHQwaUFUNjNwdXVRNUdOaWlJeFVXTmZTSXM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQckZkR0twcU1KM1hzRlBoYnlKaEVXbERoOEJfSk5zLVJHSlFXc2pVS0hqRlQ0djV0b2o5NDY0azg3REJLbnBlaVJ2VWZ6Y2lzaVF4STlrWlh4TDcteXBGN29xWDdTc0hmU1pROF9UZ2d4UlR0bGFtNjd6UzZqakxCeGlHTEZRTUVReHllcG5NOFV4OFRXZ05YZTIySlg?oc=5</t>
         </is>
       </c>
     </row>
@@ -3279,12 +3279,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Lhoist</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Ureia, MAP e potássio registram queda no Brasil - Agrolink</t>
+          <t>Com foco em data centers, Martin Marietta acerta compra de fornecedora de minerais por US$ 13,5 bi - Valor Econômico</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQckZkR0twcU1KM1hzRlBoYnlKaEVXbERoOEJfSk5zLVJHSlFXc2pVS0hqRlQ0djV0b2o5NDY0azg3REJLbnBlaVJ2VWZ6Y2lzaVF4STlrWlh4TDcteXBGN29xWDdTc0hmU1pROF9UZ2d4UlR0bGFtNjd6UzZqakxCeGlHTEZRTUVReHllcG5NOFV4OFRXZ05YZTIySlg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxOQmNERDdXd2o0VlYxZXE2aDRFUV90bEdkWTd6ZUwyNjhJMDZBV20xbWxWZ2V6VGVtZG83VHFjSnVDU3ppbUZpTm1tY3NSWUNmRFhxeW5VaEp2SHp3c1BjVkxQZXBNZEhrd2RUdHVKZUNFTHlHZFliODlHMHp4c3lMbXhVUkhqWjltOFRzUVlJMU9Da0RIZnk2Y3B6bUVTelRSZ2tUT0c1aFVZamlSTERiX2ZIa1puUnVrUlQ1aDhtRW1uLVBZZ0NSSU91RGpPY243OWVLOXp3TGNjU0pKR015dFQ2RGI1dDdO0gH3AUFVX3lxTE1jZVlGVWNwdWlxX2lGVGpRTnRPUXJJNTJWbXJTcXRjb3lQQVFNT3A5TVhPM2xpSmRNOVZKZmFFR3Y5eEJnRlRNX0taNmppMTdVT1dBeDRKVjQ2TzNPZHR0OEhBRWlmM3VBaWcwQjVzSDZmM1hVNmJTcVVRR1VGYzkxY2trZ3FXMjNpNzlnUkRxLXB6UG0xbVBFZmU5MVVIa3FVZkdSMFFwaGhBeGZna01zOVNwUGFKMXpQdkstaWhud1RxVEJXUXVFdmt1bXdjNHF3azh6Vi0zSG1tbzE0aHQwaUFUNjNwdXVRNUdOaWlJeFVXTmZTSXM?oc=5</t>
         </is>
       </c>
     </row>
@@ -3323,12 +3323,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Com pouco enxofre, indústria de fertilizante já teme paralisações - Globo Rural</t>
+          <t>Justiça condena herdeira a devolver R$ 4,9 milhões a "gigante do calcário" em MT - FOLHAMAX</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3338,19 +3338,19 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNWDFOU0tpUTJqVVQxcEVDUmRCQXB2Sm95SXJwZlIyVkNxVmMxM3FpY0xVbnZxR3IyZkNFZE9NS3VOenZGYjVZcEUxN3hWOVJkNG51SGNhemc1TVQ4YWlLNEE1SFl6eVNjaWtZVnltMG4wU2VYTEZCMFI3Y21mZVBjNTBvSHE5eXlGR0dkQzFCVG5LTTBzOWdXRnJhM1dSV2hiQkJhNFFzajhwRTdlSXVzWV9MTDZiZ3RMSW9jbmxZYW_SAc8BQVVfeXFMT0l2YXdPMW5WTVN1OHFpQWNBekR5R0dKX1Y4WkY5dEtVbFdKVHJDMm9hV1lTY2FsQnFsVG92d2RuM0V1cGNCUmhYZHZjdzFzVlNkckxKaDhnVm9PUVNYRnJBaEt4WG5NVDloSWhLbEFZQmdXSWhqdFNzRU1ySDBHdmRYUlZZTDd0UzI3d3lzSm5ZRTM0Y2NCWnVMaU9WWElKa0pBZjlPUk5yS1ZhLV9Nd3FDRHVxMVF2bUVTWFprQTYwc2hpa3YtRzhKVi1hQUtr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOQ0E2ZGFseTRjVFBDMmV6ZGxHTDdZektMM09pNTZuSGppV3R0eFhSM1lZcWRrSElmeS1MMEhHQWlFTnNWT3dJcDJLeVJrMlFaN2FkLUhadFd2NFhob3hpUE5YLTNZblItdS1pbDExUlZFMS0wSDV3VV9DUmxyZUllYmVXU2ZWQXprNHU0TF9IcnhsR3BySWMzWmx4MWJoclFGa2p6dmZKWGhtVkwwNTVtdW9YOTZSZDBFQmc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Justiça condena herdeira a devolver R$ 4,9 milhões a "gigante do calcário" em MT - FOLHAMAX</t>
+          <t>Embarques de fertilizantes crescem após acordo no estreito de Ormuz - CNN Brasil</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOQ0E2ZGFseTRjVFBDMmV6ZGxHTDdZektMM09pNTZuSGppV3R0eFhSM1lZcWRrSElmeS1MMEhHQWlFTnNWT3dJcDJLeVJrMlFaN2FkLUhadFd2NFhob3hpUE5YLTNZblItdS1pbDExUlZFMS0wSDV3VV9DUmxyZUllYmVXU2ZWQXprNHU0TF9IcnhsR3BySWMzWmx4MWJoclFGa2p6dmZKWGhtVkwwNTVtdW9YOTZSZDBFQmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOcENnZnlBVWF1ZEVFeElfLU56Y1RaZ2ZiQkdOck1KdnJkbzUwa1Z3dUo3aTItQmJrRjNKVVZKLW9NNHdhSE9FejZXb3ZiMDZZSTBGdk16SmZ2ckd1UHB2TXlNYnFZc1c2V0hlaXF4ZEpRT1pWcktSM055QXBtS3d2bVMtU1BFWkRkQmt6alZiYWFldVR0ZWp1N2hGMjRFLUlnMkxNTA?oc=5</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Embarques de fertilizantes crescem após acordo no estreito de Ormuz - CNN Brasil</t>
+          <t>Com pouco enxofre, indústria de fertilizante já teme paralisações - Globo Rural</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3382,19 +3382,19 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOcENnZnlBVWF1ZEVFeElfLU56Y1RaZ2ZiQkdOck1KdnJkbzUwa1Z3dUo3aTItQmJrRjNKVVZKLW9NNHdhSE9FejZXb3ZiMDZZSTBGdk16SmZ2ckd1UHB2TXlNYnFZc1c2V0hlaXF4ZEpRT1pWcktSM055QXBtS3d2bVMtU1BFWkRkQmt6alZiYWFldVR0ZWp1N2hGMjRFLUlnMkxNTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNWDFOU0tpUTJqVVQxcEVDUmRCQXB2Sm95SXJwZlIyVkNxVmMxM3FpY0xVbnZxR3IyZkNFZE9NS3VOenZGYjVZcEUxN3hWOVJkNG51SGNhemc1TVQ4YWlLNEE1SFl6eVNjaWtZVnltMG4wU2VYTEZCMFI3Y21mZVBjNTBvSHE5eXlGR0dkQzFCVG5LTTBzOWdXRnJhM1dSV2hiQkJhNFFzajhwRTdlSXVzWV9MTDZiZ3RMSW9jbmxZYW_SAc8BQVVfeXFMT0l2YXdPMW5WTVN1OHFpQWNBekR5R0dKX1Y4WkY5dEtVbFdKVHJDMm9hV1lTY2FsQnFsVG92d2RuM0V1cGNCUmhYZHZjdzFzVlNkckxKaDhnVm9PUVNYRnJBaEt4WG5NVDloSWhLbEFZQmdXSWhqdFNzRU1ySDBHdmRYUlZZTDd0UzI3d3lzSm5ZRTM0Y2NCWnVMaU9WWElKa0pBZjlPUk5yS1ZhLV9Nd3FDRHVxMVF2bUVTWFprQTYwc2hpa3YtRzhKVi1hQUtr?oc=5</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Brazilian Farmers Delay Input Purchases as They Await Debt Relief Bill, Mosaic Says - The AgriBiz</t>
+          <t>Terremotos na Venezuela, menor importação de ureia pelo Brasil e prêmios da soja no BR em destaque - Notícias Agrícolas</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3404,19 +3404,19 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQN2xNaUxQMDVWZl9tOVF1UFA3SG9QaHdTVndkU2Z3ci1Dazl6cElWRmV1NjVDMzVyY1Z1ckh1S2kydnFleVQ0YXpnOExKdlpBVkFPMk1xUWJodkpjODgyMzB3Q1lSdmN1Rm04SG1yb3hLbnhjb21fdUFoeFFoN0d6d3YzSHVfMmZWcF9WMHBKV2RRTUR6Z1VuRTRKM21CdTctOGh6VDdQSHhaQ0xhZV9xd1c0dU9wVkZIQ2U3c21weWtCdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxNS0R0cnpLaTNtU3c2TXZ5bDVkMWlEazJIeHktbEE4RmFjNktPeU1wb1FtUWxmZHExMmFZaXQ3aXJJWW1qMkliSjAtYUxEc3NwclNOMnI1YTNQRnlJTko1aXN4T2M5bXpNZ1R6QTNsSTgyUmZWcU1YUEZWRlc5NS1YcXVKMjBoUzdJSUpuT01wTXFOUy12Nm80c01zcFdqSkNhMFB1Wmt2ZDA4SjFwemJiTTZrV0lxTGJsd25pUXBjcGNlM1VTTnpOemo2dXpHVV90d1Y0STFNdGdoR3ZlZzVDdWxtUTRtZHAwbnkwT1ctWF9NWEppcjRJOGZTeUktbE1wNHlN0gGIAkFVX3lxTE5zUE5IamQ0ZjNxWDNXQVpLcmZuekp1VzRTNEVVZW9yMm5NVFV4M2tTekFOc1dHLVVaQkh3ZngxZ19hdDhpbk1YcGliRkFqOVhrYlVpWWdISzFiNHBkNE5qZnZOUjhBY3FrVDhzbmtpNXBnZThtMjE0di1TS19ZZVdmZHpEVG05eFZVU2xLVHdBbFFkSUdwSzlMNzBpSzlOa1VBX1JheWRxcXJiYUN5a2Qyd1JqQno0SjhxazdsYjhXeWt0THR6eFJPa1ZjZXoxVFpqbkZGdUxMRWN3d3BsOGkwUnlkUVRQcUU3OWJnMVRTV0Y0dVRRcEVpLWhuMDhmT09OdUlxaFpxaQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Terremotos na Venezuela, menor importação de ureia pelo Brasil e prêmios da soja no BR em destaque - Notícias Agrícolas</t>
+          <t>Brazilian Farmers Delay Input Purchases as They Await Debt Relief Bill, Mosaic Says - The AgriBiz</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxNS0R0cnpLaTNtU3c2TXZ5bDVkMWlEazJIeHktbEE4RmFjNktPeU1wb1FtUWxmZHExMmFZaXQ3aXJJWW1qMkliSjAtYUxEc3NwclNOMnI1YTNQRnlJTko1aXN4T2M5bXpNZ1R6QTNsSTgyUmZWcU1YUEZWRlc5NS1YcXVKMjBoUzdJSUpuT01wTXFOUy12Nm80c01zcFdqSkNhMFB1Wmt2ZDA4SjFwemJiTTZrV0lxTGJsd25pUXBjcGNlM1VTTnpOemo2dXpHVV90d1Y0STFNdGdoR3ZlZzVDdWxtUTRtZHAwbnkwT1ctWF9NWEppcjRJOGZTeUktbE1wNHlN0gGIAkFVX3lxTE5zUE5IamQ0ZjNxWDNXQVpLcmZuekp1VzRTNEVVZW9yMm5NVFV4M2tTekFOc1dHLVVaQkh3ZngxZ19hdDhpbk1YcGliRkFqOVhrYlVpWWdISzFiNHBkNE5qZnZOUjhBY3FrVDhzbmtpNXBnZThtMjE0di1TS19ZZVdmZHpEVG05eFZVU2xLVHdBbFFkSUdwSzlMNzBpSzlOa1VBX1JheWRxcXJiYUN5a2Qyd1JqQno0SjhxazdsYjhXeWt0THR6eFJPa1ZjZXoxVFpqbkZGdUxMRWN3d3BsOGkwUnlkUVRQcUU3OWJnMVRTV0Y0dVRRcEVpLWhuMDhmT09OdUlxaFpxaQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQN2xNaUxQMDVWZl9tOVF1UFA3SG9QaHdTVndkU2Z3ci1Dazl6cElWRmV1NjVDMzVyY1Z1ckh1S2kydnFleVQ0YXpnOExKdlpBVkFPMk1xUWJodkpjODgyMzB3Q1lSdmN1Rm04SG1yb3hLbnhjb21fdUFoeFFoN0d6d3YzSHVfMmZWcF9WMHBKV2RRTUR6Z1VuRTRKM21CdTctOGh6VDdQSHhaQ0xhZV9xd1c0dU9wVkZIQ2U3c21weWtCdw?oc=5</t>
         </is>
       </c>
     </row>
@@ -3455,12 +3455,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Indústria de fertilizante negocia subsídio ao enxofre para enfrentar alta de preços - AgFeed</t>
+          <t>Arqueólogos encontram mosaico de deus do rio na Turquia - Aventuras na História</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3470,19 +3470,19 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxONnhnQWZIM0h0SjNPU1JoQzZoMXgzY0FmdmRZYVVCZXVvZHp3RkxVUnhyelJWa3gzUWJQM1dEQ1I3VWUzUTFyMktmVU0wMnlOLUdaV2tjZ1lkRHhIMDdUX3lKWWtLZ3Y3R1ppa3UtRDBlejJhMVIxYUwyRVU1VFVFSk5td0JWYnRIdkRSTk5YMWVnT1c3V093Mml4YjRmSllxN0JmVlhiWmN3R0VlRzJybmZRM283QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNdFM4Yk1jUU5RMURVMTViQklhT2I4SW1jWUxTRVI0azJDM2lmMGtrWThNNGNKTE5HcWFabEV5MUVNU2lSc2NIYkhmbm5xcWZieXAxRmRpN1BPWXlscGtIZmZyZHREWkhQc21scEQ0d3ZobjB6eER4TVNMMHpfVUNMUGRVY3lFNnRRRGVhLUxVd0l0OXBRT3RKWjdtMENVcm5RRURBZ2EyVlNXTkc2UlpjdWozMVRXMWdyVW5j?oc=5</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Importação de ureia no Brasil atinge menor nível em dez anos, diz Rabobank - Globo Rural</t>
+          <t>1a fabrica de bateria de litio-enxofre do mundo - CPG Click Petróleo e Gás</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3492,19 +3492,19 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPNjdCU2M2dTdMN2NKU3hKVC1jWkFPTjFBd0RDZHd0X0U3OU1sYVNhWjRWdzVtaGM5UHNTOXgtcWpzWHFWVTJoNy1oMzBvekR4NW5GbVZTX1NmYmZLTlU4d1lRaXZJZGNrUTYtSlo3cllmekJjUWV1TU1YVnNocTQ4VkZkaXRqZkstNGY1WHBVZ0pvV1ozSHlsaUtDNGJPRDNHUXBMRnZ3LUIxcGNnTWxYU21ycWt5ZEtaR0g1SmZrRl9VMmVNanQxaGxJbTPSAdsBQVVfeXFMUHhsM2xrQVJIUnpfbjFCWEFDTThmUFJOZFR2dEtGdnNwWDhRLXV1WVdxeU10YXZtd1lHMnZ4VVd1cUVzR29sY29hMENsc1FUYVN1VVIwUjcyTzlhRE10RVkydWl3NTB2MF9SOFVNbGhXUEhCd2NJSFdSeTBmc2dac1NoN0tpREYtS29tb3ZuZ0lrdmlsV0NUMUFNR1NoeXV6WFpQNmpUZ3FvRkJBdE5vNzY3MTdjdk1kb0RuTE5xU2w1b1FxR2x4YzZrd2MtekgwTzJhUHBnN3UtWjd3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxQYnFCT1R2NWVCa3c3bkgyc0ZNdEJCeTkzVkN1SEZ5TXZUektSTzJabG1YaFFBdGY3dnZmQ3E1U0JBc1oxT3FuQmJ0WWZyUUYxZ2x0QW1DenRLd0FQd1d2WThZQkxLZy12bmVCT2duU2haV0ZJdUd4YXVaNkZqclBqdWNEa1UxZDJlZlF4Tk9nSHhmTVdTT0RqTHBrcTFiQlBhTTV3NG84elFoem5LVmlmU0x4WFV5QUd5YlRHQjk1VUVHQzNwaUxZQThXVjFwa2Yzc09SUUdSS3BIU1FQYUVMVlZCWFlHNjN2MThZOEhXRnVBSTg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Arqueólogos encontram mosaico de deus do rio na Turquia - Aventuras na História</t>
+          <t>Importação de ureia pelo Brasil tem queda brusca; ouça o comentário - Globo Rural</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNdFM4Yk1jUU5RMURVMTViQklhT2I4SW1jWUxTRVI0azJDM2lmMGtrWThNNGNKTE5HcWFabEV5MUVNU2lSc2NIYkhmbm5xcWZieXAxRmRpN1BPWXlscGtIZmZyZHREWkhQc21scEQ0d3ZobjB6eER4TVNMMHpfVUNMUGRVY3lFNnRRRGVhLUxVd0l0OXBRT3RKWjdtMENVcm5RRURBZ2EyVlNXTkc2UlpjdWozMVRXMWdyVW5j?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOSGNOWlZSaHBzRUJkY0ZyWnZkOXo4WlRoLWhOYWUxOXNnUkZJZi1YbXlPRktTT1EzZUdydnM3bkFoc243VmtkdllCYVZibnNyb2Q4d0VESVlXamN6OFRyOEQ2XzUyQmg0RGIwbmoyd05tdy1lVUQxV2gwZ3RxT2dpLUlqb3JtVlpmMEdBc0NNYjVsX1ZPZl9DQXVPLTdCSi0ydWRUbVhJZEJleHVOYjhpY29rbWl4amhWdVdGbXF0b3M3Ynd6OFF4SzRxSTbSAdsBQVVfeXFMUE5CZDBKenFqQ3RwamdaNzFjb2ZuSC16ekZSMTFaQVg2S2RFdG1DcTlCai1oRm1halpORjdhc3h1UUE5YzNmT013aGJVTElUX1UzcHdyNTdFc0xQSzR2OTBLNVViR1N4VHB5alpOUC1JdENHS2VOc2ZWLUlYR1hveExIYVdEam5TazZpX3F0bjBtYXlyUFhmcW9lX1hUMW1RNHRxTEJ1YVoyOGFyX0NlNEJ5S3dsanVFY3F2akxfM19oRGhqLXgxc0ppTFRMNzU4aWt2MnJOQkI3N3Yw?oc=5</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Importação de ureia pelo Brasil tem queda brusca; ouça o comentário - Globo Rural</t>
+          <t>Importação de ureia no Brasil atinge menor nível em dez anos, diz Rabobank - Globo Rural</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOSGNOWlZSaHBzRUJkY0ZyWnZkOXo4WlRoLWhOYWUxOXNnUkZJZi1YbXlPRktTT1EzZUdydnM3bkFoc243VmtkdllCYVZibnNyb2Q4d0VESVlXamN6OFRyOEQ2XzUyQmg0RGIwbmoyd05tdy1lVUQxV2gwZ3RxT2dpLUlqb3JtVlpmMEdBc0NNYjVsX1ZPZl9DQXVPLTdCSi0ydWRUbVhJZEJleHVOYjhpY29rbWl4amhWdVdGbXF0b3M3Ynd6OFF4SzRxSTbSAdsBQVVfeXFMUE5CZDBKenFqQ3RwamdaNzFjb2ZuSC16ekZSMTFaQVg2S2RFdG1DcTlCai1oRm1halpORjdhc3h1UUE5YzNmT013aGJVTElUX1UzcHdyNTdFc0xQSzR2OTBLNVViR1N4VHB5alpOUC1JdENHS2VOc2ZWLUlYR1hveExIYVdEam5TazZpX3F0bjBtYXlyUFhmcW9lX1hUMW1RNHRxTEJ1YVoyOGFyX0NlNEJ5S3dsanVFY3F2akxfM19oRGhqLXgxc0ppTFRMNzU4aWt2MnJOQkI3N3Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPNjdCU2M2dTdMN2NKU3hKVC1jWkFPTjFBd0RDZHd0X0U3OU1sYVNhWjRWdzVtaGM5UHNTOXgtcWpzWHFWVTJoNy1oMzBvekR4NW5GbVZTX1NmYmZLTlU4d1lRaXZJZGNrUTYtSlo3cllmekJjUWV1TU1YVnNocTQ4VkZkaXRqZkstNGY1WHBVZ0pvV1ozSHlsaUtDNGJPRDNHUXBMRnZ3LUIxcGNnTWxYU21ycWt5ZEtaR0g1SmZrRl9VMmVNanQxaGxJbTPSAdsBQVVfeXFMUHhsM2xrQVJIUnpfbjFCWEFDTThmUFJOZFR2dEtGdnNwWDhRLXV1WVdxeU10YXZtd1lHMnZ4VVd1cUVzR29sY29hMENsc1FUYVN1VVIwUjcyTzlhRE10RVkydWl3NTB2MF9SOFVNbGhXUEhCd2NJSFdSeTBmc2dac1NoN0tpREYtS29tb3ZuZ0lrdmlsV0NUMUFNR1NoeXV6WFpQNmpUZ3FvRkJBdE5vNzY3MTdjdk1kb0RuTE5xU2w1b1FxR2x4YzZrd2MtekgwTzJhUHBnN3UtWjd3?oc=5</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>1a fabrica de bateria de litio-enxofre do mundo - CPG Click Petróleo e Gás</t>
+          <t>Indústria de fertilizante negocia subsídio ao enxofre para enfrentar alta de preços - AgFeed</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxQYnFCT1R2NWVCa3c3bkgyc0ZNdEJCeTkzVkN1SEZ5TXZUektSTzJabG1YaFFBdGY3dnZmQ3E1U0JBc1oxT3FuQmJ0WWZyUUYxZ2x0QW1DenRLd0FQd1d2WThZQkxLZy12bmVCT2duU2haV0ZJdUd4YXVaNkZqclBqdWNEa1UxZDJlZlF4Tk9nSHhmTVdTT0RqTHBrcTFiQlBhTTV3NG84elFoem5LVmlmU0x4WFV5QUd5YlRHQjk1VUVHQzNwaUxZQThXVjFwa2Yzc09SUUdSS3BIU1FQYUVMVlZCWFlHNjN2MThZOEhXRnVBSTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxONnhnQWZIM0h0SjNPU1JoQzZoMXgzY0FmdmRZYVVCZXVvZHp3RkxVUnhyelJWa3gzUWJQM1dEQ1I3VWUzUTFyMktmVU0wMnlOLUdaV2tjZ1lkRHhIMDdUX3lKWWtLZ3Y3R1ppa3UtRDBlejJhMVIxYUwyRVU1VFVFSk5td0JWYnRIdkRSTk5YMWVnT1c3V093Mml4YjRmSllxN0JmVlhiWmN3R0VlRzJybmZRM283QQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Risco de desabastecimento de fertilizantes diminui, mas produtores continuam "ariscos" na hora das compras, diz Mosaic - AgFeed</t>
+          <t>Expectativa pelo PL da renegociação de dívidas emperra o varejo agrícola, diz Mosaic - The AgriBiz</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxOTDBlYlkzZWxfeVJJZ1RBTmVqclRXV1ZYcDYzV3hxR21VNDV5NkpRRXV3XzdmOVlCNFpXMXFJazJvTWllaFpfVTNObGE5S0JKQklsZUhZMi1GTE9QZG15TklEdUdaUUVmbXdxTmI0emNCdnVmNVFCWkJCN3NnY3FwcmozSzdzUjV2bzhoaElESnlPcVRmbzJXWlpiUkhGSmR2N29IbFE2N2xvMXNRZkV2WTg3aEc2czRWcGN3M2xGLUxtN1pLZTBPa0pjS0xBakVMTGRvMlFQWWg2anB1b1pR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxNN3A0WWpXR1M2UEhQQlhXUk5GbGFhMXlFVzZtczVnSW9wYzMxeFROWEpUU2tsb2xmSTQyUFdDTS1oa1BoU01GNy14OElqaGlEVXhNSTRkczhTSmdiUEQ1TGdXMUQtMHVFWHhPa2p3cHluYnhpUWhMNHRrcXl5SFI1dGtyN0hKeFd5b3dVcHNLc2cyMkRycFRGWnJLT2NGZWlLRXNwY0N3X0FCWWJseE9xcEF4a2xncHFUb3lSb2tMUFJMWk5JOXh1Q0tQSG13MEhfVlNBb0h4OXYtWEpQNjFrS3JYQmd4aW1M?oc=5</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Expectativa pelo PL da renegociação de dívidas emperra o varejo agrícola, diz Mosaic - The AgriBiz</t>
+          <t>Risco de desabastecimento de fertilizantes diminui, mas produtores continuam "ariscos" na hora das compras, diz Mosaic - AgFeed</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxNN3A0WWpXR1M2UEhQQlhXUk5GbGFhMXlFVzZtczVnSW9wYzMxeFROWEpUU2tsb2xmSTQyUFdDTS1oa1BoU01GNy14OElqaGlEVXhNSTRkczhTSmdiUEQ1TGdXMUQtMHVFWHhPa2p3cHluYnhpUWhMNHRrcXl5SFI1dGtyN0hKeFd5b3dVcHNLc2cyMkRycFRGWnJLT2NGZWlLRXNwY0N3X0FCWWJseE9xcEF4a2xncHFUb3lSb2tMUFJMWk5JOXh1Q0tQSG13MEhfVlNBb0h4OXYtWEpQNjFrS3JYQmd4aW1M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxOTDBlYlkzZWxfeVJJZ1RBTmVqclRXV1ZYcDYzV3hxR21VNDV5NkpRRXV3XzdmOVlCNFpXMXFJazJvTWllaFpfVTNObGE5S0JKQklsZUhZMi1GTE9QZG15TklEdUdaUUVmbXdxTmI0emNCdnVmNVFCWkJCN3NnY3FwcmozSzdzUjV2bzhoaElESnlPcVRmbzJXWlpiUkhGSmR2N29IbFE2N2xvMXNRZkV2WTg3aEc2czRWcGN3M2xGLUxtN1pLZTBPa0pjS0xBakVMTGRvMlFQWWg2anB1b1pR?oc=5</t>
         </is>
       </c>
     </row>
@@ -3741,12 +3741,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Ureia despenca e volta aos níveis pré-guerra - Agrolink</t>
+          <t>Visconde supera Monerá e é campeão da Copa do Calcário 2026 - Serra News</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQSGNkVDd3UG5tUk1aMHVUdk5yMFZIZUlONTROU0VoR21mSGJTakEzX2hQeUtYWXlfQUFHeXZNZWw1d3AwLXQwSE92YXFuRTFhb1pROG5aeDR1aTF6cU85eTdMelBxNnpob2FtUnZQQWJvWlBEbWNWMDNLUlVuMmN2OEFUVTVkeFNFSU1OTGdYZGNCMkZxdVFCVg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQdDBrMzFVejA0SWNzMERWbzFwVWNVSm5XZ2lWd1lTQzlqX3BBX09mRFcwZV9Qa2l1WUxNekNKSFZHNFJrekl6TnEzWE9IWW1hb2xVTS1XSzRwOU1rdEtFdzRzWk1SNEdOVTN6VzE1ZTN1Vk9aLWttaFBldUU1Qm1EUFhn?oc=5</t>
         </is>
       </c>
     </row>
@@ -3785,12 +3785,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Visconde supera Monerá e é campeão da Copa do Calcário 2026 - Serra News</t>
+          <t>Ureia despenca e volta aos níveis pré-guerra - Agrolink</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3800,19 +3800,19 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQdDBrMzFVejA0SWNzMERWbzFwVWNVSm5XZ2lWd1lTQzlqX3BBX09mRFcwZV9Qa2l1WUxNekNKSFZHNFJrekl6TnEzWE9IWW1hb2xVTS1XSzRwOU1rdEtFdzRzWk1SNEdOVTN6VzE1ZTN1Vk9aLWttaFBldUU1Qm1EUFhn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQSGNkVDd3UG5tUk1aMHVUdk5yMFZIZUlONTROU0VoR21mSGJTakEzX2hQeUtYWXlfQUFHeXZNZWw1d3AwLXQwSE92YXFuRTFhb1pROG5aeDR1aTF6cU85eTdMelBxNnpob2FtUnZQQWJvWlBEbWNWMDNLUlVuMmN2OEFUVTVkeFNFSU1OTGdYZGNCMkZxdVFCVg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Preço futuro da ureia: perspectiva após fim do conflito com Irã - Farmnews</t>
+          <t>Mosaico de antigo 'deus do rio' é encontrado na Turquia - Globo</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3822,19 +3822,19 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNb1dTZU45Ulg5NzZPTUFZT0JnV2swWVJkTERUb1hDMy1faHZ6RHFsdzJXWHNCeERXdW1iNl9MYXV1WlhjVWtNWlJDV2xWWXJIelJjTHFETjgtbkZaWXBSVndiTXJpWW1SaXBnN242ZGlBX01jWGlvUVgyTUNXS0RsOFg1WU82c2U3T2FvOHZQMUZoRWRnZkhTbklsSi15TWtz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOLTdXYW1GZW4ybGRZM2Q1OU5WWFNYNEVENXNhVDZBTG9LanM0YnM2NGlZQnAxbThZeWs0a0lOdVgyVkRfN3JQaEI4RHY1Y3BLa1lobmFuN1VvTGg5SUFiT2VvMkNxMHJDdjdyRTJGWm1HZWxpRlZNajdmQmg0WERVTGlyeW80U2g0WDctOGY0X0Vsblg5RVVLdmtFanU2bkVaaWNEQjhCdE1MWlg1cmpOZ05RQXZMcXPSAcYBQVVfeXFMUGFBczRwMXpFN0tOdm1GWWlid0hBYjV4bEFQbWRMeUEzS0hFTzZiNTdvVUI2QW5SaGg1OUY2cXV2Q1ltellaSEk1V3BHUHBzeTMwSmZJZTUxZ2FEN1UxNTVQWjY1eVBaOHFkblBqTWc3VDJWdXpzRGo0QUI1TVdYYk9MdE1uSGwxSHFnQktpX2VZYzlwT1FWT2Jub1U5dWdHWHlWRlhDZHU0ck51SmZKVjBqREhaa0JVcnFsN2tMN0dlLU0welJ3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Mosaico de antigo 'deus do rio' é encontrado na Turquia - Globo</t>
+          <t>Principais exportadores de ureia para o Brasil em 2026, até abril - Farmnews</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOLTdXYW1GZW4ybGRZM2Q1OU5WWFNYNEVENXNhVDZBTG9LanM0YnM2NGlZQnAxbThZeWs0a0lOdVgyVkRfN3JQaEI4RHY1Y3BLa1lobmFuN1VvTGg5SUFiT2VvMkNxMHJDdjdyRTJGWm1HZWxpRlZNajdmQmg0WERVTGlyeW80U2g0WDctOGY0X0Vsblg5RVVLdmtFanU2bkVaaWNEQjhCdE1MWlg1cmpOZ05RQXZMcXPSAcYBQVVfeXFMUGFBczRwMXpFN0tOdm1GWWlid0hBYjV4bEFQbWRMeUEzS0hFTzZiNTdvVUI2QW5SaGg1OUY2cXV2Q1ltellaSEk1V3BHUHBzeTMwSmZJZTUxZ2FEN1UxNTVQWjY1eVBaOHFkblBqTWc3VDJWdXpzRGo0QUI1TVdYYk9MdE1uSGwxSHFnQktpX2VZYzlwT1FWT2Jub1U5dWdHWHlWRlhDZHU0ck51SmZKVjBqREhaa0JVcnFsN2tMN0dlLU0welJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPQkZnLXNRb0ZVWkxHckFMZVE4c3paNXJDcnU2SlZYbDA3bkRDYzlVOFJMVUxuS1hwVW5GWjJEVzZVTTMtT3hPd1J3X2FBR1hsZ2lHZjU4TmRYUGxZVVRlcFp3djlHNkhUZUNWUGpUS2hsTFczTUlLLXN5Mjl6R0JId21Pb0p2V3FzTEVfQ1JhTm00b25fZzFJVGhfMHM1QQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Principais exportadores de ureia para o Brasil em 2026, até abril - Farmnews</t>
+          <t>Preço futuro da ureia: perspectiva após fim do conflito com Irã - Farmnews</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPQkZnLXNRb0ZVWkxHckFMZVE4c3paNXJDcnU2SlZYbDA3bkRDYzlVOFJMVUxuS1hwVW5GWjJEVzZVTTMtT3hPd1J3X2FBR1hsZ2lHZjU4TmRYUGxZVVRlcFp3djlHNkhUZUNWUGpUS2hsTFczTUlLLXN5Mjl6R0JId21Pb0p2V3FzTEVfQ1JhTm00b25fZzFJVGhfMHM1QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNb1dTZU45Ulg5NzZPTUFZT0JnV2swWVJkTERUb1hDMy1faHZ6RHFsdzJXWHNCeERXdW1iNl9MYXV1WlhjVWtNWlJDV2xWWXJIelJjTHFETjgtbkZaWXBSVndiTXJpWW1SaXBnN242ZGlBX01jWGlvUVgyTUNXS0RsOFg1WU82c2U3T2FvOHZQMUZoRWRnZkhTbklsSi15TWtz?oc=5</t>
         </is>
       </c>
     </row>
@@ -3895,12 +3895,12 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>cal agricola</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Sistema FAEP lamenta decisão da ANTT que impede o cultivo agrícola na faixa de domínio - Minuto Rural</t>
+          <t>Um pedido de socorro para os fertilizantes | Radar Econômico - VEJA</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3910,19 +3910,19 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPaHp3NnFKcU5hLURNY2RlTW1XWHc4WnFkWkZQRlVxQ0RfaEpTdGlaMlFIbTF4M0pNMEs1dnpZOGNjdUFuckRlMUlUV1BmN1puMkFkMHZ0SEVQbm1kMVRKLXVLYWs1dHJtTDhBN3ptbU40NjB1NGxDcU1xUTV4bTlLc1g4T19CNDVrQVkxd0lQQmZiTmluRGhrN1hWbGc4bm1leHNod0NQdld3T29tWmc2MmwyZzBoN19IT0hZdU53VzVrY0J1N2phOG8xMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNXzNyRkc3R1RCQVRpMzZlZGRtN1J6bkJtZl9YRzBFN2JkdElMc01CN2lyaWVOanRNekgybzJrNnhwMHdZV3pDTUZEY2lkMno5dHNPZ3pCSlM2QTROUlJuSFo3cWpxQzR3cGhLUzJYRmY2SXFobEdOTGpfdEhVTS1Jc0IxMGJ0TllQMFNrVnNFa0QwZlRfTGw4?oc=5</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Um pedido de socorro para os fertilizantes | Radar Econômico - VEJA</t>
+          <t>O recuo estratégico da Mosaic no Brasil - VEJA</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3932,19 +3932,19 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNXzNyRkc3R1RCQVRpMzZlZGRtN1J6bkJtZl9YRzBFN2JkdElMc01CN2lyaWVOanRNekgybzJrNnhwMHdZV3pDTUZEY2lkMno5dHNPZ3pCSlM2QTROUlJuSFo3cWpxQzR3cGhLUzJYRmY2SXFobEdOTGpfdEhVTS1Jc0IxMGJ0TllQMFNrVnNFa0QwZlRfTGw4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNcWNOZnE5TE9kN3JvVzA4eThSNEV3NFVQanBMcm1WdVd5YUhoa2N1UFlTMTNvUXQtNDhoX05LeGlGRlBLNzBfeGI1VnNJV3M0NklZLTBhNXJEY0FwV0YzMjg3Vm5iQzJ5OFV0UkRqbThiTjhmQ1ExX2V3MnFJbEM2c1RZUkd2QS13YWxwS0w4Z2stNms?oc=5</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>cal agricola</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>O recuo estratégico da Mosaic no Brasil - VEJA</t>
+          <t>Sistema FAEP lamenta decisão da ANTT que impede o cultivo agrícola na faixa de domínio - Minuto Rural</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNcWNOZnE5TE9kN3JvVzA4eThSNEV3NFVQanBMcm1WdVd5YUhoa2N1UFlTMTNvUXQtNDhoX05LeGlGRlBLNzBfeGI1VnNJV3M0NklZLTBhNXJEY0FwV0YzMjg3Vm5iQzJ5OFV0UkRqbThiTjhmQ1ExX2V3MnFJbEM2c1RZUkd2QS13YWxwS0w4Z2stNms?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPaHp3NnFKcU5hLURNY2RlTW1XWHc4WnFkWkZQRlVxQ0RfaEpTdGlaMlFIbTF4M0pNMEs1dnpZOGNjdUFuckRlMUlUV1BmN1puMkFkMHZ0SEVQbm1kMVRKLXVLYWs1dHJtTDhBN3ptbU40NjB1NGxDcU1xUTV4bTlLc1g4T19CNDVrQVkxd0lQQmZiTmluRGhrN1hWbGc4bm1leHNod0NQdld3T29tWmc2MmwyZzBoN19IT0hZdU53VzVrY0J1N2phOG8xMA?oc=5</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>ProSolos: Capão Bonito do Sul distribui calcário para 25 produtores rurais - Tua Rádio</t>
+          <t>Viter, da Votorantim Cimentos, entra no mercado de foliares e investe R$ 300 milhões na “mistura” - AgFeed</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPczJPU19lVkVaMG8wVGZGVEpQbjQyb3pYbmY2VGhUNW1GVW9lazlCaEtONGlDR3ZpSHFxVWMwaGoyNXhzcTRBLXREWkVKZUQtNF9TRXFWY1pnYXIwS3RfNVBkaTJIbFh5blVtaEZuRWhDRzU3dW5ETDZ5RXBEZU5KZzR5NW9OMTluT0dHaGU5OC0taUI5Y2FzXzZLdlZkb2tjdnMwS2ZXTXZDMnBJT05xTEFXNFl0VXBpRTlFWVA5ZFFja2xCdGpPSExFNDJsdGVjbUVaYnNhYmFsSGZkbVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPUWJ5VkZXQTJ4VjNNaWw2R2xKZ3BtLUYwazI4QzVZeGJzUnlESXFvcXFreEdDQVZnT0ZnMS1LMzhfWE1zTVoyRGp4ODlDdHppdFU2N3R4Y1RSM2k0WFN5OU51c2hHZzJfZldiWnlMaXJTM0w3dF8xTmZGM0FnSi10VXFTT3EtakJVR2dJUno5NzNiWHhpWHl2V0hBR0ZEQUtoaTlyWndNMjdMZEdVRHpIbF96aXVJZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Viter, da Votorantim Cimentos, entra no mercado de foliares e investe R$ 300 milhões na “mistura” - AgFeed</t>
+          <t>ProSolos: Capão Bonito do Sul distribui calcário para 25 produtores rurais - Tua Rádio</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3998,7 +3998,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPUWJ5VkZXQTJ4VjNNaWw2R2xKZ3BtLUYwazI4QzVZeGJzUnlESXFvcXFreEdDQVZnT0ZnMS1LMzhfWE1zTVoyRGp4ODlDdHppdFU2N3R4Y1RSM2k0WFN5OU51c2hHZzJfZldiWnlMaXJTM0w3dF8xTmZGM0FnSi10VXFTT3EtakJVR2dJUno5NzNiWHhpWHl2V0hBR0ZEQUtoaTlyWndNMjdMZEdVRHpIbF96aXVJZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPczJPU19lVkVaMG8wVGZGVEpQbjQyb3pYbmY2VGhUNW1GVW9lazlCaEtONGlDR3ZpSHFxVWMwaGoyNXhzcTRBLXREWkVKZUQtNF9TRXFWY1pnYXIwS3RfNVBkaTJIbFh5blVtaEZuRWhDRzU3dW5ETDZ5RXBEZU5KZzR5NW9OMTluT0dHaGU5OC0taUI5Y2FzXzZLdlZkb2tjdnMwS2ZXTXZDMnBJT05xTEFXNFl0VXBpRTlFWVA5ZFFja2xCdGpPSExFNDJsdGVjbUVaYnNhYmFsSGZkbVE?oc=5</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Importação de ureia pelo Brasil despenca em maio: dados de 2018 a 2026 - Farmnews</t>
+          <t>Ureia cai mais de 40% e volta ao nível pré-crise com avanço de acordo entre EUA e Irã - Notícias Agrícolas</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOc2dmVzJBa0tyZGQ3T3dCOFlFZjhkQXg0SmFjUmltT3RmbVlKSDlfYm1vOHNDMG5kdTdDalcyQ3dmTTlyY00taHRwTVhRSE54ZUdjdEZNWVEwYkRmRV9JS0FOY0xIQ01ISUF3VHA5ZmVZVS1XdlA2Mzk1UUNEbHFuT1VyUFhYSWZlU2lVay0wYUl1WmFzaEg5VmpKaGw1OTFHdWlHdDBGWlpqUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOMGREaHlncEZNM3ZPbjY2Mkdjcmp3b0xIYnNyd0ZrQ0ZIU1VOd1Z1SzlZRXRWYnJVSW9YN25rTVI2dV9BbkpxQ3ExTnJET2laeDJxSEJhTlFmbVR1NjJLVGVXMlRwN1pONGprSFhTeHVfeHFhaTh3LU91dml3ZnBkU19QMDRWeTlvVmZVOFBzTkpYRWNXVzgtS3ljUXVRYkVRSFlnX2VrWHQyWl83RUxZaFBNZFNkTEJsMmdIVW5EaWJ1QzFsbEhTNG1Ia2ZaVWItOG5vMndxaVlZMElfM3NmZXUwX2U0bmRVdEHSAe8BQVVfeXFMUHU1T0d6VUZOVnNHME1ySkpyV2NsbmtiTHBjZjIwVHJjRHBXRUR2R1pleTZjT1FBZi1CbUhxNnFTUUJUZ0xBZTZ5NG1KWUUzcnVpMHZSNkYzWG9NcGI2OEpuOFdCSllRYTlVa2hXMEpnRjUwTTV5NTlmQ21FOVhEQTFVZm5wdEU0akc2V0hNdV9JbFNCSGxlWW1DN3lFa0xIRmxSdldQR1BwYmJ5RDRzMW5kek1NNllsZ0I1VDB5WEhTNktSNGdqb1RkV0xWZ1NadlBPbmx3dXh1aUNHcVRTWk1Sbmw0NnFJbmk5R3JlYmM?oc=5</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Ureia cai mais de 40% e volta ao nível pré-crise com avanço de acordo entre EUA e Irã - Notícias Agrícolas</t>
+          <t>Importação de ureia pelo Brasil despenca em maio: dados de 2018 a 2026 - Farmnews</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4152,19 +4152,19 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOMGREaHlncEZNM3ZPbjY2Mkdjcmp3b0xIYnNyd0ZrQ0ZIU1VOd1Z1SzlZRXRWYnJVSW9YN25rTVI2dV9BbkpxQ3ExTnJET2laeDJxSEJhTlFmbVR1NjJLVGVXMlRwN1pONGprSFhTeHVfeHFhaTh3LU91dml3ZnBkU19QMDRWeTlvVmZVOFBzTkpYRWNXVzgtS3ljUXVRYkVRSFlnX2VrWHQyWl83RUxZaFBNZFNkTEJsMmdIVW5EaWJ1QzFsbEhTNG1Ia2ZaVWItOG5vMndxaVlZMElfM3NmZXUwX2U0bmRVdEHSAe8BQVVfeXFMUHU1T0d6VUZOVnNHME1ySkpyV2NsbmtiTHBjZjIwVHJjRHBXRUR2R1pleTZjT1FBZi1CbUhxNnFTUUJUZ0xBZTZ5NG1KWUUzcnVpMHZSNkYzWG9NcGI2OEpuOFdCSllRYTlVa2hXMEpnRjUwTTV5NTlmQ21FOVhEQTFVZm5wdEU0akc2V0hNdV9JbFNCSGxlWW1DN3lFa0xIRmxSdldQR1BwYmJ5RDRzMW5kek1NNllsZ0I1VDB5WEhTNktSNGdqb1RkV0xWZ1NadlBPbmx3dXh1aUNHcVRTWk1Sbmw0NnFJbmk5R3JlYmM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOc2dmVzJBa0tyZGQ3T3dCOFlFZjhkQXg0SmFjUmltT3RmbVlKSDlfYm1vOHNDMG5kdTdDalcyQ3dmTTlyY00taHRwTVhRSE54ZUdjdEZNWVEwYkRmRV9JS0FOY0xIQ01ISUF3VHA5ZmVZVS1XdlA2Mzk1UUNEbHFuT1VyUFhYSWZlU2lVay0wYUl1WmFzaEg5VmpKaGw1OTFHdWlHdDBGWlpqUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Ureia volta ao preço pré-guerra, mas vendas ainda não reagem - CNN Brasil</t>
+          <t>Visconde sai na frente na decisão da Copa do Calcário - FERJ</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOT2J4STBfU3p3enNZSHhWZjZxcVc2YUp3VDlhanpJMHI4dWVpREtfanF3dWFiV1hiSWN2NWxmMFJqQk1FY0w3Rm43OWVfSlpFS3J5SWM3ZzZnbXJQa25hWVMxYmNCd2QwalBGa2dQenc1NmZVZHJ3U0NxRUxqay1nTHdlMTFGNDR3RUxwRWs4cnAwWF9TVGNlWXc5ZDdiSldlUzFKdzhTRGQ4bTN3ckVpNFV5cHhmX2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOUDdiZWgzRUVPQVFSZEl0d2hfbTVoMmtSR0k3UTRBMjlVTEFqS1F2cHZrRXpVZ3VtbVExb3R2ckx1TWZ4T3ZPWEQ5c2l3bVRWcU4yNXQ2cXphcVpyaTl5a0xPcEhqRW1Yc3Jyb3VVeDB1dTJlamttamhEN3pJZ2plcDBxb3JUcGl1UG9vdUNYMTc?oc=5</t>
         </is>
       </c>
     </row>
@@ -4203,12 +4203,12 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Sibelco</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Visconde sai na frente na decisão da Copa do Calcário - FERJ</t>
+          <t>Rio Maior organizou Gala Empresarial do concelho - O Mirante</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4218,19 +4218,19 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOUDdiZWgzRUVPQVFSZEl0d2hfbTVoMmtSR0k3UTRBMjlVTEFqS1F2cHZrRXpVZ3VtbVExb3R2ckx1TWZ4T3ZPWEQ5c2l3bVRWcU4yNXQ2cXphcVpyaTl5a0xPcEhqRW1Yc3Jyb3VVeDB1dTJlamttamhEN3pJZ2plcDBxb3JUcGl1UG9vdUNYMTc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPYmIwcks0U205THc0UF80M2tqOTBpZWY1VWhZMFZzUUE2UEt2bmFLcTBsQ1g4YjRBRjBmRUZiN25XQVdCNDdldTdiZC10VTdBSzY3YjJiTFo5TXdaNjVVNkZUMTZSQ1g4MU1XX2s0azMwd0hNTFlDTktFVktWSWtrWUpPTjFQZEhoUzU3M3NzaXpQMVVaajZoYWhPRHNtLUhf?oc=5</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Sibelco</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Rio Maior organizou Gala Empresarial do concelho - O Mirante</t>
+          <t>Ureia volta ao preço pré-guerra, mas vendas ainda não reagem - CNN Brasil</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPYmIwcks0U205THc0UF80M2tqOTBpZWY1VWhZMFZzUUE2UEt2bmFLcTBsQ1g4YjRBRjBmRUZiN25XQVdCNDdldTdiZC10VTdBSzY3YjJiTFo5TXdaNjVVNkZUMTZSQ1g4MU1XX2s0azMwd0hNTFlDTktFVktWSWtrWUpPTjFQZEhoUzU3M3NzaXpQMVVaajZoYWhPRHNtLUhf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOT2J4STBfU3p3enNZSHhWZjZxcVc2YUp3VDlhanpJMHI4dWVpREtfanF3dWFiV1hiSWN2NWxmMFJqQk1FY0w3Rm43OWVfSlpFS3J5SWM3ZzZnbXJQa25hWVMxYmNCd2QwalBGa2dQenc1NmZVZHJ3U0NxRUxqay1nTHdlMTFGNDR3RUxwRWs4cnAwWF9TVGNlWXc5ZDdiSldlUzFKdzhTRGQ4bTN3ckVpNFV5cHhmX2c?oc=5</t>
         </is>
       </c>
     </row>
@@ -4467,12 +4467,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Visconde e Monerá estão na decisão da Copa do Calcário - FERJ</t>
+          <t>Ureia cai 32%, mas compras seguem lentas - Agrolink</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNdTE4ODV2amJMQVVTaUd3bXdPa1psaE91azdMNDIwTHJSd3NDdDRMZEstX3pzWHBmdXlhd2d0dXphTlNYelc2T19zVTRJVVJmWktXRDlac2Q0RVoxeWQ1TTl3R2NnVkRHNS1pWTljYm8xSjRzY1JrUV82SldFNEFsRkp5MjBDdjdSQnhNRF9ibmxDUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQN0l5anBLTS11NTdjc3huWTJtZWhGSkgzLUNRcEdwODFMeFpSRTBfZEdka3ctczB3c29GSjNvY24xbzRVOGVnS2xXRGRoRm1YR0k0bkQxb3RxV0I3ZDF6WlpLRjBzbEM4M2Z4ODZJQ2swSkV3X2xYLW1LRDQxc1pyX1B4MGhGNHBhbjlURDhxdlBhUnM?oc=5</t>
         </is>
       </c>
     </row>
@@ -4511,12 +4511,12 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Lhoist</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Monerá e Visconde são os grandes finalistas da Copa do Calcário - jornaldaregiao.com</t>
+          <t>Empresas ampliam vagas e buscam talentos - Portal UAI</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -4526,19 +4526,19 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOb2tvdUhDbG0yZzRQc0dxa0l1eS14YzVtQjdEdV9CVUF3LUZXMUdreUdJcHUtWkhIcVNtU1E5NmNfcC05LXQ3aHBJaGNqOUxMZEhtQ1hYNWVKQmR3U3lzNm5fQ1ZiLXNvS2szVU1iTWVLN0hkazZhcS15NGdUX0YzZnFLcnlyeGVxSDRnbFNURndKR29IaWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxNNmJmTzczLUFGbU8tQ3dxY2RFTU1aeDY4ZVVQSXo2dlNUbzBHY3lmd2IyU2VzVk1nQTFYdTBxdDRLWkxQNTk1elR5ZkcyWUk4M1F1cDZUekYtcGhpZXl1SHZPel9vT19YT0xGLUIwdkVNZUVrZTczaTdXdU9kNUd5eFY4aU9oQ0JtVEc4dXFBNmNCdWpUa3V3YUg3M09PZ2xEYUlDd3VSS0dfSEhRXzlhUlducmpoSkx1WG5rZVFOLUhlVlNGRHpmNUFhdFVuRWNXR1V0X3hzRUoyc0k?oc=5</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Ureia cai 32%, mas compras seguem lentas - Agrolink</t>
+          <t>Visconde e Monerá estão na decisão da Copa do Calcário - FERJ</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -4548,19 +4548,19 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQN0l5anBLTS11NTdjc3huWTJtZWhGSkgzLUNRcEdwODFMeFpSRTBfZEdka3ctczB3c29GSjNvY24xbzRVOGVnS2xXRGRoRm1YR0k0bkQxb3RxV0I3ZDF6WlpLRjBzbEM4M2Z4ODZJQ2swSkV3X2xYLW1LRDQxc1pyX1B4MGhGNHBhbjlURDhxdlBhUnM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNdTE4ODV2amJMQVVTaUd3bXdPa1psaE91azdMNDIwTHJSd3NDdDRMZEstX3pzWHBmdXlhd2d0dXphTlNYelc2T19zVTRJVVJmWktXRDlac2Q0RVoxeWQ1TTl3R2NnVkRHNS1pWTljYm8xSjRzY1JrUV82SldFNEFsRkp5MjBDdjdSQnhNRF9ibmxDUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Lhoist</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Empresas ampliam vagas e buscam talentos - Portal UAI</t>
+          <t>Monerá e Visconde são os grandes finalistas da Copa do Calcário - jornaldaregiao.com</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxNNmJmTzczLUFGbU8tQ3dxY2RFTU1aeDY4ZVVQSXo2dlNUbzBHY3lmd2IyU2VzVk1nQTFYdTBxdDRLWkxQNTk1elR5ZkcyWUk4M1F1cDZUekYtcGhpZXl1SHZPel9vT19YT0xGLUIwdkVNZUVrZTczaTdXdU9kNUd5eFY4aU9oQ0JtVEc4dXFBNmNCdWpUa3V3YUg3M09PZ2xEYUlDd3VSS0dfSEhRXzlhUlducmpoSkx1WG5rZVFOLUhlVlNGRHpmNUFhdFVuRWNXR1V0X3hzRUoyc0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOb2tvdUhDbG0yZzRQc0dxa0l1eS14YzVtQjdEdV9CVUF3LUZXMUdreUdJcHUtWkhIcVNtU1E5NmNfcC05LXQ3aHBJaGNqOUxMZEhtQ1hYNWVKQmR3U3lzNm5fQ1ZiLXNvS2szVU1iTWVLN0hkazZhcS15NGdUX0YzZnFLcnlyeGVxSDRnbFNURndKR29IaWc?oc=5</t>
         </is>
       </c>
     </row>
@@ -4665,12 +4665,12 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Ureia mais barata, mas não o suficiente - AgFeed</t>
+          <t>Tudo igual nos jogos de ida das semifinais da Copa do Calcário - FERJ</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -4680,19 +4680,19 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQNERlNFpxYnhTaVVMdkhzcG9RWG1rN1M4T0VWR1lLbmRGSE1OR1E0UkhxMUw5ZGtJWjd2dmJabHZ6eWF3UFRBZ2JfWDhjS1gzaTJUSWVDd21BY2tuN3ZTcmNqMGNsZjhuUFA4RnNld0pPZmtwTGg5ajZsdllNeG5WaFlCbTlUREtUcmhudEx3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNZGFjM1JnOHMteTdBanNpN1RhaDJ6SWsxdGZCWFgyamtLYlNKazU3YmhBWnJqajFzZk9WNWRSNTRERklLUVVxTWRqWENTRFlmX0EzSU1vU3V6dk9CN2M2YURvUkV5UDRsNmdCSDV1T2xUVzF5Zktubk9wRWtGSHhFQWdkYlBBcE5KUUx3NWUzQW5mMkVTY3lCTlFmRUI?oc=5</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Tudo igual nos jogos de ida das semifinais da Copa do Calcário - FERJ</t>
+          <t>Ureia mais barata, mas não o suficiente - AgFeed</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNZGFjM1JnOHMteTdBanNpN1RhaDJ6SWsxdGZCWFgyamtLYlNKazU3YmhBWnJqajFzZk9WNWRSNTRERklLUVVxTWRqWENTRFlmX0EzSU1vU3V6dk9CN2M2YURvUkV5UDRsNmdCSDV1T2xUVzF5Zktubk9wRWtGSHhFQWdkYlBBcE5KUUx3NWUzQW5mMkVTY3lCTlFmRUI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQNERlNFpxYnhTaVVMdkhzcG9RWG1rN1M4T0VWR1lLbmRGSE1OR1E0UkhxMUw5ZGtJWjd2dmJabHZ6eWF3UFRBZ2JfWDhjS1gzaTJUSWVDd21BY2tuN3ZTcmNqMGNsZjhuUFA4RnNld0pPZmtwTGg5ajZsdllNeG5WaFlCbTlUREtUcmhudEx3?oc=5</t>
         </is>
       </c>
     </row>
@@ -4731,12 +4731,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Preços da ureia recuam 25% - mas nem isso anima o mercado - AgFeed</t>
+          <t>Copa do Calcário: vagas para a grande final serão decididas no próximo domingo - Serra News</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPajBDOHUtVWZFN2QwalllTlN0eEhJOG03dE5Ia1JQNlpwRW52MVVjbG5Ya1ZYaGt0QU04dVB4b2ZSdU53blVHcHVVRThzVEs0bFpoY3ZOcjJUay1EVjZXZW00TTNJc19RV0gtdUxtNGVZRFNFM2FjaHk1NkRjR0dGWkVfS0NfZFJzWFNFUw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNem9RT0xBWGhHc0dKc0t1NjBWaUdkVGxVcGhRbE1GYmU2WDV3WDdMQ2ZfQnBhZGQ2YlMxZFo4NmsxR1NLeWVJbkxHdFRmT3VIVnpNRlZrVjktNDZYR05fQnVPYzJoQkpJdlhQVTRuSDAtWTdfT3JWamRTUGhOQW9xV2JkSFllT1UzTnNMbk9vaw?oc=5</t>
         </is>
       </c>
     </row>
@@ -4797,12 +4797,12 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Copa do Calcário: vagas para a grande final serão decididas no próximo domingo - Serra News</t>
+          <t>Mosaic suspende mineração em Tapira por 30 dias e acende alerta em Uberaba - JM Online</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -4812,19 +4812,19 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNem9RT0xBWGhHc0dKc0t1NjBWaUdkVGxVcGhRbE1GYmU2WDV3WDdMQ2ZfQnBhZGQ2YlMxZFo4NmsxR1NLeWVJbkxHdFRmT3VIVnpNRlZrVjktNDZYR05fQnVPYzJoQkpJdlhQVTRuSDAtWTdfT3JWamRTUGhOQW9xV2JkSFllT1UzTnNMbk9vaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMU1lSmhaSEJPbE5tbmdCU3ozeXVFcUdfX2dGZ2k3c3hGUzNaX2NCTUlfMlZiZjBLa2xXSHpFUURHbFBwLWRVZFdKOXJFVjBhb2t5SnZjVGJYcS1zRGlPNVN3dFRuVHF3WEtXeFkxelM2dUV4S0tLME41WVBFV1lZZWJSbFNZVzQwSEZNUk9teEtQM1M5eV90cnBpeWpCSW5kVDFNZl96aFd4TEd6aEV0OUMyMTLSAbwBQVVfeXFMTjl1UzR0Q2dTWHFEN0FqdktmQ0Nlc2p3YXBYLVpNTnlGVUFXOGNwUXNuMTZRdWZoQ2ttSHFzNEZsY2ltWjdqT05uUVpPSjdaUkR2YTFXYXV6RVZERU5rRk52ZGU1d2Vac2ptRDFTVXFVWGgzZTFCNzMyZ0VpZ1o4RWpLa044YUVEX2lMWEJYVDAta1RWRnhrV1BKYmZpSVpKSm56N2wzU3dCQldWV3R0VEJLNTJGbHdxY0VRdVo?oc=5</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Mosaic suspende mineração em Tapira por 30 dias e acende alerta em Uberaba - JM Online</t>
+          <t>Preços da ureia recuam 25% - mas nem isso anima o mercado - AgFeed</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -4834,7 +4834,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMU1lSmhaSEJPbE5tbmdCU3ozeXVFcUdfX2dGZ2k3c3hGUzNaX2NCTUlfMlZiZjBLa2xXSHpFUURHbFBwLWRVZFdKOXJFVjBhb2t5SnZjVGJYcS1zRGlPNVN3dFRuVHF3WEtXeFkxelM2dUV4S0tLME41WVBFV1lZZWJSbFNZVzQwSEZNUk9teEtQM1M5eV90cnBpeWpCSW5kVDFNZl96aFd4TEd6aEV0OUMyMTLSAbwBQVVfeXFMTjl1UzR0Q2dTWHFEN0FqdktmQ0Nlc2p3YXBYLVpNTnlGVUFXOGNwUXNuMTZRdWZoQ2ttSHFzNEZsY2ltWjdqT05uUVpPSjdaUkR2YTFXYXV6RVZERU5rRk52ZGU1d2Vac2ptRDFTVXFVWGgzZTFCNzMyZ0VpZ1o4RWpLa044YUVEX2lMWEJYVDAta1RWRnhrV1BKYmZpSVpKSm56N2wzU3dCQldWV3R0VEJLNTJGbHdxY0VRdVo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPajBDOHUtVWZFN2QwalllTlN0eEhJOG03dE5Ia1JQNlpwRW52MVVjbG5Ya1ZYaGt0QU04dVB4b2ZSdU53blVHcHVVRThzVEs0bFpoY3ZOcjJUay1EVjZXZW00TTNJc19RV0gtdUxtNGVZRFNFM2FjaHk1NkRjR0dGWkVfS0NfZFJzWFNFUw?oc=5</t>
         </is>
       </c>
     </row>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Embrapa cria calcário que reduz perdas e aumenta produtividade no campo - Exame</t>
+          <t>Embrapa cria calcário mais nutritivo e resistente à umidade - CompreRural</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPbUFVRVpOaU54dHozMHJBc3EzSlE1c0JBXzZkci1IR09EVEcxejBEekdPYXE4THV0SUtIemQ3QjItVTRwYXpZTHVUV3ctU3M5WHBVbjNJaVhHVnlNVGI3elZmUWlLWFlwZzNETEE0TjRNY1NkYklMYlQwQ1BNN0Z1Y1JsQ3FDZVItSmFuYzFKRnFXLVdNM1BjRnJlRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNY3VDcDE0TVJIcGRwOVozMnozYk12NFEtRnhYcVVJSTd2ZlpCR0Y4WlpXdmI1QTJaMVAxSDJQc285M3NGSGZNYTNVd001WVVxbW1XdGFpTzJfdlg3Y0lQVHBBWEVqMXVFLVFBcFZaSTVqWmR3eFZvejVZa00zako5Tk5GYk9IS0xNMURFSGZ2clUyZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Embrapa cria calcário mais nutritivo e resistente à umidade - CompreRural</t>
+          <t>Embrapa cria calcário que reduz perdas e aumenta produtividade no campo - Exame</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNY3VDcDE0TVJIcGRwOVozMnozYk12NFEtRnhYcVVJSTd2ZlpCR0Y4WlpXdmI1QTJaMVAxSDJQc285M3NGSGZNYTNVd001WVVxbW1XdGFpTzJfdlg3Y0lQVHBBWEVqMXVFLVFBcFZaSTVqWmR3eFZvejVZa00zako5Tk5GYk9IS0xNMURFSGZ2clUyZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPbUFVRVpOaU54dHozMHJBc3EzSlE1c0JBXzZkci1IR09EVEcxejBEekdPYXE4THV0SUtIemQ3QjItVTRwYXpZTHVUV3ctU3M5WHBVbjNJaVhHVnlNVGI3elZmUWlLWFlwZzNETEE0TjRNY1NkYklMYlQwQ1BNN0Z1Y1JsQ3FDZVItSmFuYzFKRnFXLVdNM1BjRnJlRQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Anvisa recolhe coco ralado por excesso de dióxido de enxofre; saiba quais são os riscos à saúde - Notícias ao Minuto Brasil</t>
+          <t>Anvisa manda recolher lote de coco ralado ‘Casa de Mãe’, da marca Qualicoco, por excesso de enxofre - Estadão</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPVlFOZlF1ZGhHU1NNYjlNdm1kVzNDT0IwX0pRZUVzaFkwUTVhRnFvdU1xcnhnNl9PYllWVmdnVDVkXzlFcVJhYVoydXo5TURlVHlnR3Y1bjNrRGtGMTg0SkFoODdPblU4Qy1fbW9IcGFVN1BZVWloSVlWemNpM19KVlE3OVRiV1MwZmt4UXdlUmR4ZzdqU09RNmgwdWpjVDBtcVRkNWZseF92SnZySUN4VXlCMzdxa0JIU1FDd2FkZlNBbmhUNHBLdDNEVFlfQ3gwblpPbk9qcHNheHkyb1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQYzh2cjdEME1NdHBVU0EwUEp4emJrSVMwWERxTW5FeFduT2prV3lyZ3lGbkFkOUtzcG01WV9sQUtObUl0N3FhbzhOVXI5eG1wWEwyN0ZrcDdSczdCa2plUFZTSWtGS21TODBYNGpWSDZpbTR0d0hwYWhJU29vbUlnaG5zcThDV2liYURCdHE3VDV4WWNVMlM5Um8yTUItMWI3ZFdEa0ZTZEFfa08yZHFOVksxdXo3SktXeGVrd2liNlU0b24yS0JWT2M5eHZnYU3SAdQBQVVfeXFMTmthZ3daS3ZoN1NrVzN0RXFfdXZJcHRkQTBwaVFmdmpfZGJlQVFaY0MwSmNYSDMydWZVeUN5NnVlWXZhQkNWX3BUSUpyQzQ3aUZKTk1yemJyNmhCTkNfSmM0V3NXc2t0eDEzcEQ2eHZxZkM3V3RZRlNjYkVaUmVmT2JvQ1lweDAySEZYem80MlE4TVItVGZaTi1yQ1paTktMQzhaTWNoWktGMGtiMXFjYnJLZFBocnBNbV9oYXJIWWNyaUwxSWlVNlpYR2VjS0pXZ0F3ZDk?oc=5</t>
         </is>
       </c>
     </row>
@@ -4978,7 +4978,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Coco ralado com excesso de enxofre: quais os riscos? Em quais sintomas prestar atenção? - Estadão</t>
+          <t>Anvisa recolhe coco ralado por excesso de dióxido de enxofre; saiba quais são os riscos à saúde - Notícias ao Minuto Brasil</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -4988,7 +4988,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPWmY3TXBIbWxobnFjUi1mTUozS2xCbTlaSGxKX2o0QTExdWszWk5USkR4ZVk0Zk5vcTIxSm9HZDRzazlGVjBDLVE4a2NTTnQ4eHpQM3cyNTFDVDd1aGs0cFhxUVBmbXlaUTNLMjljT0FSRWlMRm1iVkxMYk1uc2Nvd0JZencteGFkLXNFSWxySlhTNkdpemo2Y2N4ZlFOclJPMkNLUDdGU2FrYTJsRjIzdTE3RWVQUnhGbXJpVkJhcWhjclZJaWdXM2dueTFYRjNfMWE5WjBEWEFxUdIB3wFBVV95cUxOdGxrd3ZlRXQ3X0k0Rkx5VDk0OW5yQ0FyZ1A1QW5wTGhXZDA3blVtaVdobkM5YVFBcEhsUUlYRGYwVlVodlF1UmxsbVZaY0c2Z2lScV9hWnlOdlpZYzZDNXVLWWdiU0FvRExxZlQzQ2d3N3lTbk9tY3pXZEpJOWtZaDhOYVhVOXFFWExTVkYyMU5jUnk3VURmS0dMazRJUERGYS1BS2p5MFo5bXg3eFlPcVJtZ1NMQjBYRDFrWmRRbnpRdWlMU0VmaHI3T2tHUGp2b3I3bFZZYk9oWWhDX3pN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPVlFOZlF1ZGhHU1NNYjlNdm1kVzNDT0IwX0pRZUVzaFkwUTVhRnFvdU1xcnhnNl9PYllWVmdnVDVkXzlFcVJhYVoydXo5TURlVHlnR3Y1bjNrRGtGMTg0SkFoODdPblU4Qy1fbW9IcGFVN1BZVWloSVlWemNpM19KVlE3OVRiV1MwZmt4UXdlUmR4ZzdqU09RNmgwdWpjVDBtcVRkNWZseF92SnZySUN4VXlCMzdxa0JIU1FDd2FkZlNBbmhUNHBLdDNEVFlfQ3gwblpPbk9qcHNheHkyb1E?oc=5</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher lote de coco ralado ‘Casa de Mãe’, da marca Qualicoco, por excesso de enxofre - Estadão</t>
+          <t>Com excesso de enxofre, Anvisa ordena recolhimento de coco ralado da marca ‘Casa de Mãe’ - Grafitti News</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQYzh2cjdEME1NdHBVU0EwUEp4emJrSVMwWERxTW5FeFduT2prV3lyZ3lGbkFkOUtzcG01WV9sQUtObUl0N3FhbzhOVXI5eG1wWEwyN0ZrcDdSczdCa2plUFZTSWtGS21TODBYNGpWSDZpbTR0d0hwYWhJU29vbUlnaG5zcThDV2liYURCdHE3VDV4WWNVMlM5Um8yTUItMWI3ZFdEa0ZTZEFfa08yZHFOVksxdXo3SktXeGVrd2liNlU0b24yS0JWT2M5eHZnYU3SAdQBQVVfeXFMTmthZ3daS3ZoN1NrVzN0RXFfdXZJcHRkQTBwaVFmdmpfZGJlQVFaY0MwSmNYSDMydWZVeUN5NnVlWXZhQkNWX3BUSUpyQzQ3aUZKTk1yemJyNmhCTkNfSmM0V3NXc2t0eDEzcEQ2eHZxZkM3V3RZRlNjYkVaUmVmT2JvQ1lweDAySEZYem80MlE4TVItVGZaTi1yQ1paTktMQzhaTWNoWktGMGtiMXFjYnJLZFBocnBNbV9oYXJIWWNyaUwxSWlVNlpYR2VjS0pXZ0F3ZDk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPMlJWRTAxYnh2aVNNS3N6QkQwZkMxU2lCN19hMW5FNVNPYTBZRWpPU1VVQVk3blQyMnUyNkV4X0FjcDhnNE5vMkR3dzhwSHR6ek44M2E4V3hWU0FmM3NDLUVYV0s1N1dJTlYyazF4U196cGp2Ym1EWTc4amtOSDZDODhkbC1tM201cWZFY0luUXc2UkpSM0M2RDRPYlFBZy1TSVVUVHY3YUxXX3lhN09ManZmRmc?oc=5</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Com excesso de enxofre, Anvisa ordena recolhimento de coco ralado da marca ‘Casa de Mãe’ - Grafitti News</t>
+          <t>Coco ralado com excesso de enxofre: quais os riscos? Em quais sintomas prestar atenção? - Estadão</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -5032,19 +5032,19 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPMlJWRTAxYnh2aVNNS3N6QkQwZkMxU2lCN19hMW5FNVNPYTBZRWpPU1VVQVk3blQyMnUyNkV4X0FjcDhnNE5vMkR3dzhwSHR6ek44M2E4V3hWU0FmM3NDLUVYV0s1N1dJTlYyazF4U196cGp2Ym1EWTc4amtOSDZDODhkbC1tM201cWZFY0luUXc2UkpSM0M2RDRPYlFBZy1TSVVUVHY3YUxXX3lhN09ManZmRmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPWmY3TXBIbWxobnFjUi1mTUozS2xCbTlaSGxKX2o0QTExdWszWk5USkR4ZVk0Zk5vcTIxSm9HZDRzazlGVjBDLVE4a2NTTnQ4eHpQM3cyNTFDVDd1aGs0cFhxUVBmbXlaUTNLMjljT0FSRWlMRm1iVkxMYk1uc2Nvd0JZencteGFkLXNFSWxySlhTNkdpemo2Y2N4ZlFOclJPMkNLUDdGU2FrYTJsRjIzdTE3RWVQUnhGbXJpVkJhcWhjclZJaWdXM2dueTFYRjNfMWE5WjBEWEFxUdIB3wFBVV95cUxOdGxrd3ZlRXQ3X0k0Rkx5VDk0OW5yQ0FyZ1A1QW5wTGhXZDA3blVtaVdobkM5YVFBcEhsUUlYRGYwVlVodlF1UmxsbVZaY0c2Z2lScV9hWnlOdlpZYzZDNXVLWWdiU0FvRExxZlQzQ2d3N3lTbk9tY3pXZEpJOWtZaDhOYVhVOXFFWExTVkYyMU5jUnk3VURmS0dMazRJUERGYS1BS2p5MFo5bXg3eFlPcVJtZ1NMQjBYRDFrWmRRbnpRdWlMU0VmaHI3T2tHUGp2b3I3bFZZYk9oWWhDX3pN?oc=5</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Mineradora ligada à Vale fecha acordo de R$ 27 milhões por extração ilegal de calcário em Goiás - Jornal Opção</t>
+          <t>Retomada da Fafen atenderá a 7% do consumo da ureia no Brasil, diz presidente da Petrobras - UOL Economia</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5054,19 +5054,19 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQUWpoTWRpSkZ2YlpjVWJkbmtHSTROcVdZYVJmcGpwd085QUdoc1dxelhudXJvVlR2X0xvZnRMbjBFRE1YdDRGOTFjVWNuNTJ4bmQ3UU9UYmRSYUMxSmxpWHlJSE9Hb190d3VGdkoxejI5Q1VrSVpfVHp1eFpkd0YzSUl1YjducElqUmhmM1hSNDJHaTZHWHRuVktXY2R2dHQyMU5hNklqcElfSFJjVGc2WFlaQ19ZZXIxVTJQODJwLTJqRjNhbnZjLUNEa1NhQXZOXzhhRlNxdGU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQR3RBSFpsbjM4bDFaWVBBa1g3eE5La0VVV0dxaDdSQjVUc3c0WjlnbGg5bFFXRWVJQXUxRE82QXJjTzU2TzZoazNNYTJsdFBCNGtOeTZPcjQxS2tQVl9EcVR0YnI0N1ZpY0VSTnhTQUZMSjhwQ2otbTZVYVRISG9NZFZQREpfREw3RUlsOEl3SGJvMHpVajhONUlwTlF4YTVXVGhneTBXV2xoV3ppcFJVb3h1T3BaWVZUUUpZNGdEVnNKeEluXzl3Y21nM2lJODk4OU0zTDhrSGlrU2F3NHZzV2tEYmpBc3pfMlI5X3ZR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher coco ralado por excesso de enxofre - Pleno.News</t>
+          <t>Mineradora ligada à Vale fecha acordo de R$ 27 milhões por extração ilegal de calcário em Goiás - Jornal Opção</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5076,19 +5076,19 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNdHBVZWl1TWRoenctMVBqRFhvUkhUNVVkV3hGZ3Vkc2lNX2V3eTRXTVFqdmhZU2Y1OFdZUjJDMW9KV29MSWNfTi12SGhkb3lwZ2ViRnlsalhmY0JCVmJHTElIWGlpVi11Y2VMUnRleU5STUszZ1ZMeHRQMjB1Zk5uTEEtbjVMNUJrQXdNYnNUZ0pQakEwY0JrZk1nONIBowFBVV95cUxORFQ1MVBTQ1VsdTlOQ28xemxBLUNHaEtIUFctakRUckU5aEFKM1VhNU9vdVE3WDZ6NWtFaVZnd09NWk1IUDd5XzBKZTVFbVN1R0U3a1N2Yk5sczBIZDhERmQyZjNIMG51d3NjTFd1VFJaOWN0bmRPa1RCZWQwUjVjRnV1c29kZHpoa3R2c2VOangxc2VaTlItNUNTajJmQVhBNUlV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQUWpoTWRpSkZ2YlpjVWJkbmtHSTROcVdZYVJmcGpwd085QUdoc1dxelhudXJvVlR2X0xvZnRMbjBFRE1YdDRGOTFjVWNuNTJ4bmQ3UU9UYmRSYUMxSmxpWHlJSE9Hb190d3VGdkoxejI5Q1VrSVpfVHp1eFpkd0YzSUl1YjducElqUmhmM1hSNDJHaTZHWHRuVktXY2R2dHQyMU5hNklqcElfSFJjVGc2WFlaQ19ZZXIxVTJQODJwLTJqRjNhbnZjLUNEa1NhQXZOXzhhRlNxdGU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Comercialização de fertilizantes no Brasil tem atraso relevante - CNN Brasil</t>
+          <t>Anvisa manda recolher lote de coco ralado por excesso de enxofre - MS Todo dia</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -5098,19 +5098,19 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaGlLX3NOTUxkam9rd0NRVDI5Rlp5VDlZVjVfMWh2andDSXJGaXhVWEJTaWZ0b3haQ2tBMmFVV3NOVlVuOC1MNzlUNGFtbFRncDZZcGZwZEJmQVNxZl9GTTZhUUZYUzdEREFzbURVaGZnWlAzN1J1UERhbEhvZ0NHNGlDYk1sZFR2OFA2MDUyYVBHeHRtU0ZjLU9TNjNDT2M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOaEFRLWlCUTNMR05sNEtuSzg5T05GVFIzdVlCUHBreS1Pa2NxU3RtSzZaQnNpYmZDRXVadVhVaFhUU0NTQV9HQ0pCUFpqQW1fczZBX3RyUGN2QXhzcldjRWVqanBseDNzTnJKMVJndmRZck9Wa1RqWWx0OXBQc3ZYZlVhUzRaRVhUQzI0SUszalJMQ1RMZTllblpHMV9oUnd4bmdVVFNWVWs2akZP?oc=5</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher lote de coco ralado por excesso de enxofre - MS Todo dia</t>
+          <t>Comercialização de fertilizantes no Brasil tem atraso relevante - CNN Brasil</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -5120,19 +5120,19 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOaEFRLWlCUTNMR05sNEtuSzg5T05GVFIzdVlCUHBreS1Pa2NxU3RtSzZaQnNpYmZDRXVadVhVaFhUU0NTQV9HQ0pCUFpqQW1fczZBX3RyUGN2QXhzcldjRWVqanBseDNzTnJKMVJndmRZck9Wa1RqWWx0OXBQc3ZYZlVhUzRaRVhUQzI0SUszalJMQ1RMZTllblpHMV9oUnd4bmdVVFNWVWs2akZP?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNaGlLX3NOTUxkam9rd0NRVDI5Rlp5VDlZVjVfMWh2andDSXJGaXhVWEJTaWZ0b3haQ2tBMmFVV3NOVlVuOC1MNzlUNGFtbFRncDZZcGZwZEJmQVNxZl9GTTZhUUZYUzdEREFzbURVaGZnWlAzN1J1UERhbEhvZ0NHNGlDYk1sZFR2OFA2MDUyYVBHeHRtU0ZjLU9TNjNDT2M?oc=5</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Retomada da Fafen atenderá a 7% do consumo da ureia no Brasil, diz presidente da Petrobras - UOL Economia</t>
+          <t>Anvisa manda recolher e proíbe venda de lote de coco ralado por excesso de enxofre - ND Mais</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -5142,7 +5142,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQR3RBSFpsbjM4bDFaWVBBa1g3eE5La0VVV0dxaDdSQjVUc3c0WjlnbGg5bFFXRWVJQXUxRE82QXJjTzU2TzZoazNNYTJsdFBCNGtOeTZPcjQxS2tQVl9EcVR0YnI0N1ZpY0VSTnhTQUZMSjhwQ2otbTZVYVRISG9NZFZQREpfREw3RUlsOEl3SGJvMHpVajhONUlwTlF4YTVXVGhneTBXV2xoV3ppcFJVb3h1T3BaWVZUUUpZNGdEVnNKeEluXzl3Y21nM2lJODk4OU0zTDhrSGlrU2F3NHZzV2tEYmpBc3pfMlI5X3ZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE9HMUF4TXN5WUx0RTZMTUktampKOHB4MjQtTWZyR1ROQ05MOXNYQW95NHpuZjlieXJCYlNGN3U1ZjhCTzlRaEMyWlZ1eUh1TldxaFREdmktMm9IQ0VHSUpDS2U3TFJNZFNiVy1FeWZDVld1X1c2NEpqX09OVQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher e proíbe venda de lote de coco ralado por excesso de enxofre - ND Mais</t>
+          <t>Anvisa manda recolher lote de coco ralado após identificar excesso de enxofre; confira marca - Rádio Metrópole</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE9HMUF4TXN5WUx0RTZMTUktampKOHB4MjQtTWZyR1ROQ05MOXNYQW95NHpuZjlieXJCYlNGN3U1ZjhCTzlRaEMyWlZ1eUh1TldxaFREdmktMm9IQ0VHSUpDS2U3TFJNZFNiVy1FeWZDVld1X1c2NEpqX09OVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSjRVamltMjVSeTh5ZWpfTVZRQnNIRGdhc3AzNkRiQy1oSnFkQnZMczVraFl0WGNjSkhRcmRfclVoQkxtU1BROVNnaWhWaDNnd25MNHNWY28yUTVuMTNvSVpzelNBMjBvMGhCeWdXdlUtZWhwTG9HUV9kSFBDMUIwSTZxWURqQm9pc2xWd19MZ3p2bkZJdjRwUkVKS3plakJuNVdlN0FTd3BIcTdGY09PRXpoMGJtbXNuNUlqNE9zYWNqTVMwNXpXR1dtcllxUW9hM3pQODRscw?oc=5</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher lote de coco ralado após identificar excesso de enxofre; confira marca - Rádio Metrópole</t>
+          <t>Anvisa manda recolher lote de coco ralado por excesso de dióxido de enxofre - O POVO</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSjRVamltMjVSeTh5ZWpfTVZRQnNIRGdhc3AzNkRiQy1oSnFkQnZMczVraFl0WGNjSkhRcmRfclVoQkxtU1BROVNnaWhWaDNnd25MNHNWY28yUTVuMTNvSVpzelNBMjBvMGhCeWdXdlUtZWhwTG9HUV9kSFBDMUIwSTZxWURqQm9pc2xWd19MZ3p2bkZJdjRwUkVKS3plakJuNVdlN0FTd3BIcTdGY09PRXpoMGJtbXNuNUlqNE9zYWNqTVMwNXpXR1dtcllxUW9hM3pQODRscw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNYXFuR084YlVCYWlxRWFFZElvOXhoZGFYbXh6WXBHZzZOSm40Y3VtSUVzZjh3MVdSRGxvVVhUOWRWOHh4T1lQdUQzYVFBNXhadDhJUGpPVnBmeU1MWUo3Wk81T3JBeGkxVkUyNHlDaU11eldSckM1ZlpmQjJ0VEVFWTI4M1FtYkpxUVc0UVREUXpZZFI0clA1a1ZkS3FiNl9JMzZiVmtwN24xYWNfN0xFUUhKMlYwM1VGRm5PZ3R5cmVTNTBVRkpyb3pQM2w?oc=5</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher lote de coco ralado por excesso de dióxido de enxofre - O POVO</t>
+          <t>Anvisa manda recolher lote de coco ralado por excesso de enxofre - CNN Brasil</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNYXFuR084YlVCYWlxRWFFZElvOXhoZGFYbXh6WXBHZzZOSm40Y3VtSUVzZjh3MVdSRGxvVVhUOWRWOHh4T1lQdUQzYVFBNXhadDhJUGpPVnBmeU1MWUo3Wk81T3JBeGkxVkUyNHlDaU11eldSckM1ZlpmQjJ0VEVFWTI4M1FtYkpxUVc0UVREUXpZZFI0clA1a1ZkS3FiNl9JMzZiVmtwN24xYWNfN0xFUUhKMlYwM1VGRm5PZ3R5cmVTNTBVRkpyb3pQM2w?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPbEhqa29HQTVER2pnczg0QVFJclpNcDZJMlFLdDVCb1pnLWdEbGE3clRBLVkzak1SVXBSWTcza19aSlVtZklGV01lM2JyMms1ZElzUlZVSTZDVFNraUxpZDBkd1NYZVFNeXBKTkpTbl9VTlBvTWh3V3ppUm1BSzVqc09xa2x3RHl0MEFtS19jYnp4RGJSMFZKRm01VThReXhLSmc?oc=5</t>
         </is>
       </c>
     </row>
@@ -5259,12 +5259,12 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher lote de coco ralado por excesso de enxofre - CNN Brasil</t>
+          <t>Dá para substituir ureia por farelo de soja no proteico da seca? Especialista responde - Giro do Boi - Canal Rural</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -5274,7 +5274,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPbEhqa29HQTVER2pnczg0QVFJclpNcDZJMlFLdDVCb1pnLWdEbGE3clRBLVkzak1SVXBSWTcza19aSlVtZklGV01lM2JyMms1ZElzUlZVSTZDVFNraUxpZDBkd1NYZVFNeXBKTkpTbl9VTlBvTWh3V3ppUm1BSzVqc09xa2x3RHl0MEFtS19jYnp4RGJSMFZKRm01VThReXhLSmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQR082Wi1qR1lQM0swUUVtTUN1NkhLeXlVbDZJSGFRRjVVaWFEb1hSN3IwS2ZCOVZsLWdvMnFtNFo3aFlGcHlMeUd0LVA4ZzFTWEtyZm81Y1dhZkhCMDR4SHVyeW1tQlpjelVoT1VrbU5LMXRESkprTVN5Z2l4TnJYU0tFTGpiVHlUaFZadWJFeUp2b29qUDV3VXVNQmswcXkxUDdrX2FwV05USVRSdFVMWVBnQXBXMDBfbEVBT1RiVU5SM0ZIdk5VMU1hcw?oc=5</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher lote de coco ralado após identificar excesso de enxofre - G1</t>
+          <t>Anvisa manda recolher coco ralado por excesso de enxofre - Pleno.News</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxQeDRscjA1UGJuUmh2b05TWVBXUlI3RjlSLVJ5Y3pidkJjaWtZeTVrYnBfNFczOFFpNFpGTG5SUUxRbXBRS2tCUHZEWTBjUzNHZFJyMGlSYzRzNGl1eEE5Xy1LOW14azE3QUNHdjd1cDF4TEJ0MUNoM3JoWmNsLWkyQ0tqNTNkMHFoSmZBbEFWWDBCNDh4UHBNSWFaN21nOW1QYzFCQWRvcDA4WnhvWGZvV0h5SEppcGdJMWxLREVmdXZzUU5uUkNUUNIB1wFBVV95cUxOUHRpNVVsWVRvLXE4MjR4NFRkN1JiSFVaZnE2X2RQRnlNOUMwWmJ1SkZ2R0ZQWkNVaVh5VGtWclVFUFZkUDQ1SDBTREd0aXAzUkY4VFZ1RnhaZDVZRVBTMXV5NXY2aXJIQWdIUkk4UllaTlNZSlZUcWhLQ19TZUVHNS1zMmdNckRhaU9LcUlzUFVub1R5YzZiU2wzWXlxQlRfdHhsRzZjV21Kem43WFh3VnpJY3hvcXZzRFprdll1U3YtU3YtVVE5OVdJLXBvbzlWenNraUNMUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNdHBVZWl1TWRoenctMVBqRFhvUkhUNVVkV3hGZ3Vkc2lNX2V3eTRXTVFqdmhZU2Y1OFdZUjJDMW9KV29MSWNfTi12SGhkb3lwZ2ViRnlsalhmY0JCVmJHTElIWGlpVi11Y2VMUnRleU5STUszZ1ZMeHRQMjB1Zk5uTEEtbjVMNUJrQXdNYnNUZ0pQakEwY0JrZk1nONIBowFBVV95cUxORFQ1MVBTQ1VsdTlOQ28xemxBLUNHaEtIUFctakRUckU5aEFKM1VhNU9vdVE3WDZ6NWtFaVZnd09NWk1IUDd5XzBKZTVFbVN1R0U3a1N2Yk5sczBIZDhERmQyZjNIMG51d3NjTFd1VFJaOWN0bmRPa1RCZWQwUjVjRnV1c29kZHpoa3R2c2VOangxc2VaTlItNUNTajJmQVhBNUlV?oc=5</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Anvisa recolhe lote de coco ralado por excesso de enxofre; veja a marca e o que fazer - Veja Saúde</t>
+          <t>Anvisa determina recolhimento de lote de coco ralado por excesso de enxofre; veja marca - GZH</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNZDQ3Zy1xb2VGTVJnVnRoeUVxY1NMMC1yRFV3RDhKWFhZUGluN3ZPVUxEZEtYSlcxUF8zX3d4ZElaV3VDSXQxOGEwMUllSFNEVmJFenJ6ZE40djdJSWVubWxLVDFldFR2WmdybFp5Y2FjemhkQ18yam5VcjJ0UkVUb3g3ZXJRaTV2R1lIZTVEY3hEb2tlOVFNb0VuVVhPOVlTZnJpWWpWRTRQeTMwMkxfUWxrRDFIQ1h4dTF0djczbTl1QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNZklVdWVqSnZBODhORUZwWlFOeXFpSHlEN01yMWd6YW1ZeE5lZXhRSFVHbFdlU3BmT05kTkdZYnY5dE5kelRsdXBDY29aWTAxWjV1ZENBdHhpQ1hqT1d4dHBKOTQxREMyTV94bXQ3MGk5RWRwTTBlQTJrNmF5cWMwcXI4VWZOYUllRElnVm11dW56N1NUZ1FjVkdmQzlsc0xaLW5lakRlVkM4X1JuMzFIYm1wbXBZOHpwZ0Mwb3NWaXhOMkU1UGt5a1NSb3hYZzRnN0FaVmhqZ242Vk9OYlhyd3BKTlgtN0JQWUhxZ2w0b01iSGNBRm5qa1BheFU2S1dV?oc=5</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5352,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Anvisa manda recolher coco ralado por excesso de enxofre; veja se você tem em casa - Exame</t>
+          <t>Anvisa recolhe lote de coco ralado por excesso de enxofre; veja a marca e o que fazer - Veja Saúde</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -5362,19 +5362,19 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNZzd6c1RaVDEtMFk3TnFhekVMSDNOQnAyUkVxaHkyQklSbWMwYTQ4b0tFSVJtTGZ4R0pONmthWmFOWDRNRTQ4YnFjWkh2ZDFfdlA1VGFidmpTQTVQdUxMaWpmd2Y5QldZZkxlQ1U5SHdHa1hOMzVUQmV3bzRJeV9GUDE1b0FMRE5sOVByV3pJOHNOWTBxNGhWRkRRbFM3SEppcHNCR3RrNHQ3MUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNZDQ3Zy1xb2VGTVJnVnRoeUVxY1NMMC1yRFV3RDhKWFhZUGluN3ZPVUxEZEtYSlcxUF8zX3d4ZElaV3VDSXQxOGEwMUllSFNEVmJFenJ6ZE40djdJSWVubWxLVDFldFR2WmdybFp5Y2FjemhkQ18yam5VcjJ0UkVUb3g3ZXJRaTV2R1lIZTVEY3hEb2tlOVFNb0VuVVhPOVlTZnJpWWpWRTRQeTMwMkxfUWxrRDFIQ1h4dTF0djczbTl1QQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Dá para substituir ureia por farelo de soja no proteico da seca? Especialista responde - Giro do Boi - Canal Rural</t>
+          <t>Anvisa manda recolher lote de coco ralado após identificar excesso de enxofre - G1</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQR082Wi1qR1lQM0swUUVtTUN1NkhLeXlVbDZJSGFRRjVVaWFEb1hSN3IwS2ZCOVZsLWdvMnFtNFo3aFlGcHlMeUd0LVA4ZzFTWEtyZm81Y1dhZkhCMDR4SHVyeW1tQlpjelVoT1VrbU5LMXRESkprTVN5Z2l4TnJYU0tFTGpiVHlUaFZadWJFeUp2b29qUDV3VXVNQmswcXkxUDdrX2FwV05USVRSdFVMWVBnQXBXMDBfbEVBT1RiVU5SM0ZIdk5VMU1hcw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxQeDRscjA1UGJuUmh2b05TWVBXUlI3RjlSLVJ5Y3pidkJjaWtZeTVrYnBfNFczOFFpNFpGTG5SUUxRbXBRS2tCUHZEWTBjUzNHZFJyMGlSYzRzNGl1eEE5Xy1LOW14azE3QUNHdjd1cDF4TEJ0MUNoM3JoWmNsLWkyQ0tqNTNkMHFoSmZBbEFWWDBCNDh4UHBNSWFaN21nOW1QYzFCQWRvcDA4WnhvWGZvV0h5SEppcGdJMWxLREVmdXZzUU5uUkNUUNIB1wFBVV95cUxOUHRpNVVsWVRvLXE4MjR4NFRkN1JiSFVaZnE2X2RQRnlNOUMwWmJ1SkZ2R0ZQWkNVaVh5VGtWclVFUFZkUDQ1SDBTREd0aXAzUkY4VFZ1RnhaZDVZRVBTMXV5NXY2aXJIQWdIUkk4UllaTlNZSlZUcWhLQ19TZUVHNS1zMmdNckRhaU9LcUlzUFVub1R5YzZiU2wzWXlxQlRfdHhsRzZjV21Kem43WFh3VnpJY3hvcXZzRFprdll1U3YtU3YtVVE5OVdJLXBvbzlWenNraUNMUQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Anvisa determina recolhimento de lote de coco ralado por excesso de enxofre; veja marca - GZH</t>
+          <t>Anvisa manda recolher coco ralado por excesso de enxofre; veja se você tem em casa - Exame</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNZklVdWVqSnZBODhORUZwWlFOeXFpSHlEN01yMWd6YW1ZeE5lZXhRSFVHbFdlU3BmT05kTkdZYnY5dE5kelRsdXBDY29aWTAxWjV1ZENBdHhpQ1hqT1d4dHBKOTQxREMyTV94bXQ3MGk5RWRwTTBlQTJrNmF5cWMwcXI4VWZOYUllRElnVm11dW56N1NUZ1FjVkdmQzlsc0xaLW5lakRlVkM4X1JuMzFIYm1wbXBZOHpwZ0Mwb3NWaXhOMkU1UGt5a1NSb3hYZzRnN0FaVmhqZ242Vk9OYlhyd3BKTlgtN0JQWUhxZ2w0b01iSGNBRm5qa1BheFU2S1dV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNZzd6c1RaVDEtMFk3TnFhekVMSDNOQnAyUkVxaHkyQklSbWMwYTQ4b0tFSVJtTGZ4R0pONmthWmFOWDRNRTQ4YnFjWkh2ZDFfdlA1VGFidmpTQTVQdUxMaWpmd2Y5QldZZkxlQ1U5SHdHa1hOMzVUQmV3bzRJeV9GUDE1b0FMRE5sOVByV3pJOHNOWTBxNGhWRkRRbFM3SEppcHNCR3RrNHQ3MUU?oc=5</t>
         </is>
       </c>
     </row>
@@ -5523,12 +5523,12 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Mosaic anuncia iniciativas selecionadas no Edital da Água 2026 - IBRAM - Mineração do Brasil</t>
+          <t>Falta de demanda pressiona e preços da ureia recuam no mercado internacional - Notícias Agrícolas</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOdld0UllhbUlrZ0dxa3Z5TjRkSXI3VTNYcmxENU1CakwyWGs1a2R0ajFKNUtpZV9EZ1V0OWtDbXBVOWZrbUoxcWJOT2ZFWkwxNzhhNnRaYVBGdl85ay0xZUJHb19HNGxkVkczNUdPc2p0eHFBLTdRNlJmdTJJN1hHbFZEOTBGYzMtX3N4Q3BhcEc4N3pEWWVF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOLWFOeS1Jbm1MT0FjNVYwWTkxNVI5MVZvYWpFTHdSYkJtcklhQzkwbTgyUU5PX0VlcjZ2eWo2ZVpveDE3ZTIzRW9kVWlELTctbW54eTNodWVQelBYUXJ6bUJWMnZJRTNYTEhWOTFxMGpLa3BLbENKMW1DQ0pQUUdiT1dFb2FPYkJlUVQ0U3JZR05lZTNCYm9jalFrNDgxVXhVM2p6V0xtcXZxVVkw0gGyAUFVX3lxTE9YcUlfc05SQjlHeDViTVhvcmIzT3JNdU5ORnVqek9HdGg3NzhDdjNFY2ZjZHFzNXFDc0w5TzBVUTEzdkI0dmhMMXVIcGt0WDF5QzhBZFBEbm5EbHhLOVgzSEFpZEZUWGhSdVh5MEhNZmJhcFJxVzVQclZsS1pDWE9IVUZ5dFVUdjhlOW0wOUlyQllUR240TGRINXFpZG9SQkNCN3JpSko2MFVwTnRxRVVGdnc?oc=5</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Ureia cai pela quinta semana nos portos - Agrolink</t>
+          <t>Cotações da ureia recuam pela 5ª semana seguida com demanda enfraquecida - Canal Rural</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -5560,19 +5560,19 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOem1iVWpuSWx2Qk9PN0xvMVNEaGZEM1kzQWdmeWRFdTh4VjVJLTVNTDhRY1Z6ZnYyYVhkWUNYVm51U3ZNb0JiaExrb2RYcXBlX0NaZGNQUk5KZ1FremQ0NzZTWk5GQXZ6UXBxYm4yRUxTNTRwTDdiRnh1M042a1JCM3VZUXpoVlJRZU92ejA5QV9BZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNalY1bGttNXJOYUVBSVFzeVNDd2pBQXkwUUhvLVhFZFJYd0kyYl81UHNuMW1pR01sSElyVXJVbTNYVTU0QVV6M1ZTb2M3MV8wbFN6U2p3WkhWd1hlcXFJR2NFSW9DcXYtWC1JNF82UlJSUXRtYmt1VUgwVHhZcDNHWG1qZk5majdOWldPblpLYnloR0NTcWt5dFhXMkNiTzl2emszMG5CczJabUZaMFdCeWNCUlRKQQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Produção de fertilizantes desaba por conflito no Oriente Médio - VEJA</t>
+          <t>Definidos os semifinalistas da Copa do Calcário 2026 - jornaldaregiao.com</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -5582,19 +5582,19 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQd3NMRG1QdXN1NzBmNUp3bUhRUWpBQ1FZOWxLVzNyUnNLZ1FZYkZDRkhXTEhIWDZFX3FuU1kwckNiTG1VSUI1M3h2RU0zR1pQYmlHVDdrZHJNZ1hBSFVrWm5ySk4ybG5RQlh5MzVqMk9OQnR0TFNWaXFuYjREMHFLU2syNFRfelEzVXBER3dQT2JQbW5nU1BhdjJ1OUhEcW8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPd3lVWExUMExpNnYzRHRkVWcxbS1lV1hMbE9mMHlZTkFTSkd1NFJ1Z3lxYXhtZzNpOVNJTjJOV2Z4UmhkMzkwNmlaRmtKOWlPQmE3ZVhoX2pCQ1N1d00wT09UY0YyTHJ4TFIwRTM3Y3M1bU9QeklBaDNvRWVGdmpoLU44OGpSNms?oc=5</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Definidos os semifinalistas da Copa do Calcário 2026 - jornaldaregiao.com</t>
+          <t>Produção de fertilizantes desaba por conflito no Oriente Médio - VEJA</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPd3lVWExUMExpNnYzRHRkVWcxbS1lV1hMbE9mMHlZTkFTSkd1NFJ1Z3lxYXhtZzNpOVNJTjJOV2Z4UmhkMzkwNmlaRmtKOWlPQmE3ZVhoX2pCQ1N1d00wT09UY0YyTHJ4TFIwRTM3Y3M1bU9QeklBaDNvRWVGdmpoLU44OGpSNms?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQd3NMRG1QdXN1NzBmNUp3bUhRUWpBQ1FZOWxLVzNyUnNLZ1FZYkZDRkhXTEhIWDZFX3FuU1kwckNiTG1VSUI1M3h2RU0zR1pQYmlHVDdrZHJNZ1hBSFVrWm5ySk4ybG5RQlh5MzVqMk9OQnR0TFNWaXFuYjREMHFLU2syNFRfelEzVXBER3dQT2JQbW5nU1BhdjJ1OUhEcW8?oc=5</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Cotações da ureia recuam pela 5ª semana seguida com demanda enfraquecida - Canal Rural</t>
+          <t>Ureia cai pela quinta semana nos portos - Agrolink</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNalY1bGttNXJOYUVBSVFzeVNDd2pBQXkwUUhvLVhFZFJYd0kyYl81UHNuMW1pR01sSElyVXJVbTNYVTU0QVV6M1ZTb2M3MV8wbFN6U2p3WkhWd1hlcXFJR2NFSW9DcXYtWC1JNF82UlJSUXRtYmt1VUgwVHhZcDNHWG1qZk5majdOWldPblpLYnloR0NTcWt5dFhXMkNiTzl2emszMG5CczJabUZaMFdCeWNCUlRKQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOem1iVWpuSWx2Qk9PN0xvMVNEaGZEM1kzQWdmeWRFdTh4VjVJLTVNTDhRY1Z6ZnYyYVhkWUNYVm51U3ZNb0JiaExrb2RYcXBlX0NaZGNQUk5KZ1FremQ0NzZTWk5GQXZ6UXBxYm4yRUxTNTRwTDdiRnh1M042a1JCM3VZUXpoVlJRZU92ejA5QV9BZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -5655,12 +5655,12 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Falta de demanda pressiona e preços da ureia recuam no mercado internacional - Notícias Agrícolas</t>
+          <t>Mosaic anuncia iniciativas selecionadas no Edital da Água 2026 - IBRAM - Mineração do Brasil</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -5670,7 +5670,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOLWFOeS1Jbm1MT0FjNVYwWTkxNVI5MVZvYWpFTHdSYkJtcklhQzkwbTgyUU5PX0VlcjZ2eWo2ZVpveDE3ZTIzRW9kVWlELTctbW54eTNodWVQelBYUXJ6bUJWMnZJRTNYTEhWOTFxMGpLa3BLbENKMW1DQ0pQUUdiT1dFb2FPYkJlUVQ0U3JZR05lZTNCYm9jalFrNDgxVXhVM2p6V0xtcXZxVVkw0gGyAUFVX3lxTE9YcUlfc05SQjlHeDViTVhvcmIzT3JNdU5ORnVqek9HdGg3NzhDdjNFY2ZjZHFzNXFDc0w5TzBVUTEzdkI0dmhMMXVIcGt0WDF5QzhBZFBEbm5EbHhLOVgzSEFpZEZUWGhSdVh5MEhNZmJhcFJxVzVQclZsS1pDWE9IVUZ5dFVUdjhlOW0wOUlyQllUR240TGRINXFpZG9SQkNCN3JpSko2MFVwTnRxRVVGdnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOdld0UllhbUlrZ0dxa3Z5TjRkSXI3VTNYcmxENU1CakwyWGs1a2R0ajFKNUtpZV9EZ1V0OWtDbXBVOWZrbUoxcWJOT2ZFWkwxNzhhNnRaYVBGdl85ay0xZUJHb19HNGxkVkczNUdPc2p0eHFBLTdRNlJmdTJJN1hHbFZEOTBGYzMtX3N4Q3BhcEc4N3pEWWVF?oc=5</t>
         </is>
       </c>
     </row>
@@ -5743,12 +5743,12 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Crise internacional pode afetar produção de fertilizantes em Catalão, alerta Metabase - Badiinho</t>
+          <t>Severiano de Almeida adquire distribuidor de calcário para atender contrapartida do Programa Terra Forte - Jornal Bom Dia</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE9UOVFBd2FaZHdNSjBOeGVrdTZ3dnBwaWNxVEdCSEEydTROLWhfVXYzdHB5UTdPUzZsN2JqbFVfQVItV1htb1N3Z2s5Q0l6cVdBYjZlSlZ2bVZ3WFBUX0ZtaU5EOWJ6dTBWaHcxaGNwRXF6YWRvdmhV0gF8QVVfeXFMTnU4U1hjc0VldVhHQVBQMkNDNm5fdFNNN1FDN1hzNDdJWU1DazJiNGVzM05BYm1XamR5eWJQMEg0QXJRQUJOU01MeWdMNEVUTUhZdVduQnZDZGJGVUNHbFJsTWcwMDFTd0lYLUkwZnczTE1PZkZvcUhTUmsyLQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxQcG9FWW8yeVV3REc1bWxBY1I1NFh5TmJxbE5BakhjcklocVNvMDVISHNhQjE0NU43Q2tOeGdUaDktQlpFLW5ySHQ3ck5iQ3p2Y1J2aFc3UmJHeTF6cUwxemQ5ejVYQzFxY3Y2djVrQkxTdDh0TnV1NW9vRlNjS29XR1dwSTNOUVhXNVdjTzVMQ3Y3YnpZajZDRHRRUmQ0Z04tRkFUaGFURWFHM3Q3S1gza0xOZXFBMkVNei1LMGZsY3FCV3J2bHdUWUdQOElRTG4yaFltX3VCckFkaFNEZ1R3?oc=5</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Casa Criativa CMOC seleciona projetos com impacto social - Valor Econômico</t>
+          <t>Crise internacional pode afetar produção de fertilizantes em Catalão, alerta Metabase - Badiinho</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -5780,19 +5780,19 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxOWHlwcHo5UU9SbmRMZFF6aWxMN1BnMjRXLWNFUDZGYnVVMFZTeHpnWG1ldV9hM2NqVFVkRHAxdHAtMmp3OEVzOEdxV1RGRldNOVozVDhVVUhpTXVCWmZvdFN4enZrZko0RmVydk9Yb3U0QUtaUURVS0NGWU9ELU40ZnFsRjgwNlc1YzBLQi1PcXo3WDNfWmhrdTlJSEpfZkVyajVGTHFCOUpjMGJpZFYwVkZERW1FeFFfMm1UZlRMa1B2UdIB0AFBVV95cUxPcGNGakszQVlpNWp3X2FGdHdHRUpzY0hxbjJQajVKUThjSnZsbHV5QUY5ZFJIZFkwV0RvejZWNnNnQlZjWHI1Nmk1OFRWb29vb21qTXQ5aUtmNUgzY1JTNktuTjg0Q090S1R4VFBsVWFtYWpCMmIwel9xVGtnREZxYTNfeDJrQTVBb1RxOExCeEZDWkhxVnpCaWR3VzlSRTlvXzFuWVJLZEJsSUJDN1NtbDhGRnNrOG5NOGZNOFYyME5vUDJvdlRBRFhGNXctNFdp?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE9UOVFBd2FaZHdNSjBOeGVrdTZ3dnBwaWNxVEdCSEEydTROLWhfVXYzdHB5UTdPUzZsN2JqbFVfQVItV1htb1N3Z2s5Q0l6cVdBYjZlSlZ2bVZ3WFBUX0ZtaU5EOWJ6dTBWaHcxaGNwRXF6YWRvdmhV0gF8QVVfeXFMTnU4U1hjc0VldVhHQVBQMkNDNm5fdFNNN1FDN1hzNDdJWU1DazJiNGVzM05BYm1XamR5eWJQMEg0QXJRQUJOU01MeWdMNEVUTUhZdVduQnZDZGJGVUNHbFJsTWcwMDFTd0lYLUkwZnczTE1PZkZvcUhTUmsyLQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Severiano de Almeida adquire distribuidor de calcário para atender contrapartida do Programa Terra Forte - Jornal Bom Dia</t>
+          <t>Casa Criativa CMOC seleciona projetos com impacto social - Valor Econômico</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxQcG9FWW8yeVV3REc1bWxBY1I1NFh5TmJxbE5BakhjcklocVNvMDVISHNhQjE0NU43Q2tOeGdUaDktQlpFLW5ySHQ3ck5iQ3p2Y1J2aFc3UmJHeTF6cUwxemQ5ejVYQzFxY3Y2djVrQkxTdDh0TnV1NW9vRlNjS29XR1dwSTNOUVhXNVdjTzVMQ3Y3YnpZajZDRHRRUmQ0Z04tRkFUaGFURWFHM3Q3S1gza0xOZXFBMkVNei1LMGZsY3FCV3J2bHdUWUdQOElRTG4yaFltX3VCckFkaFNEZ1R3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxOWHlwcHo5UU9SbmRMZFF6aWxMN1BnMjRXLWNFUDZGYnVVMFZTeHpnWG1ldV9hM2NqVFVkRHAxdHAtMmp3OEVzOEdxV1RGRldNOVozVDhVVUhpTXVCWmZvdFN4enZrZko0RmVydk9Yb3U0QUtaUURVS0NGWU9ELU40ZnFsRjgwNlc1YzBLQi1PcXo3WDNfWmhrdTlJSEpfZkVyajVGTHFCOUpjMGJpZFYwVkZERW1FeFFfMm1UZlRMa1B2UdIB0AFBVV95cUxPcGNGakszQVlpNWp3X2FGdHdHRUpzY0hxbjJQajVKUThjSnZsbHV5QUY5ZFJIZFkwV0RvejZWNnNnQlZjWHI1Nmk1OFRWb29vb21qTXQ5aUtmNUgzY1JTNktuTjg0Q090S1R4VFBsVWFtYWpCMmIwel9xVGtnREZxYTNfeDJrQTVBb1RxOExCeEZDWkhxVnpCaWR3VzlSRTlvXzFuWVJLZEJsSUJDN1NtbDhGRnNrOG5NOGZNOFYyME5vUDJvdlRBRFhGNXctNFdp?oc=5</t>
         </is>
       </c>
     </row>
@@ -5853,12 +5853,12 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Ureia cai 14% em quatro semanas, mas preço ainda está 43% acima do nível pré-conflito - Agrolink</t>
+          <t>AgriConnection e Mosaic lançam Fiagro de até R$ 100 milhões para o mercado de fertilizantes - AgFeed</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -5868,19 +5868,19 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNcDRET2JCb0V6aVhxVWROTHZEY1Vkcy1wSGFONnVQZGFqY1VmaU1hVFBFRmRIYzVod2tvNm42WlJXVXhxMXB1am5aMnlXYnlnY0V5QU5pWU52TUZaekpsUmJtaXB0NnJEaUpXSUtsMjBrT01KWmZqLVdrWTc4MDVxM3BfWU9KVHhRZHA1TFdGeWtMeXF5dmVDTXJfU05qYVdLSERnZll6WXVaa3ZDOFhWemRQck1YM3lkMkVoXzV3dWluc3c5MTBNdFJvOEFmZlU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOUmlJREVBVDhtRldoNDVjX3RoRkNEYVB1QU13RjFmNmV4MHFNRnp1Qk0wdENJNU41Yk9aVTVNNURDU1V4VUpfczlXOFhUYmlfYUN3NnNnSncxY2RNYWFJQlBXdEZJRmNmSnVTeTRDcmhtU3FzNVdybzliOUJwTkFONTV4MGFydDlxakwtblZiTzNlOEx1cHJxd3BUTlhrYjRyR3RkSmFKc0EyTXRqRDhqV3ZoUGd0YXMxdWxkVjJjTQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>TECNOLOGIA | CMOC lança projeto para levar inclusão digital a comunidades - Brasil Mineral</t>
+          <t>Mosaic e Inpasa assinam novo acordo de barter focado em insumos - CNN Brasil</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -5890,19 +5890,19 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQanZUMi1FN3JGZDNCVXJ3dTJvYUdrYXlhMnJBQV9ka3QzVXZnZ0t2RFpQaEFndUNPOTZzMHlEXzI1UFlsaFlHTGJDTnFhU2RXZ2JfRFdWMVVieTZmSW96Q1VTVWdWZVgzSW1xTHBxeFhydUZUY2tqZTRMQTh0V2RMOTFycDJoMGl0dVVDaUZXV2hkUVFoalFOZGNMeEVsUlVQWjZrcQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOVm00RUZmWGVBMzJ5Vnc4aDB3ZktTenoyMmJXanVXWF9xYTlNT3VmalhFbk9lYlNiT3h5cFZMdk5qZ0xkUkpTMkM0bkxhNHZvRk51SDZENWliR3FmRUNxMEFJQ3d5U3FNb2hhRUdCWUs2X1UxeFgzQjhMbmItbmhaSzhyQkVFSHF2ZV81UWRVb2VDTF91cnVvVGNZSW0xU28?oc=5</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Calluz aposta em calcário com alto teor de magnésio - RCN 67</t>
+          <t>TECNOLOGIA | CMOC lança projeto para levar inclusão digital a comunidades - Brasil Mineral</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -5912,19 +5912,19 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE90MUpQNDhERWltS2FYaVNXZ3NvZTNaRmVXMFo4OUZrbUFmODR5REtNSmJDOVd3bnFqTnRZZHctUXV3U2N2OVg2ZDkwRGMyUjVJUkwxX2dSYWdoZ05ZeTNXQnBfdHE2SEY3OF9BQkVFLWVUQW1fejZWRVRR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQanZUMi1FN3JGZDNCVXJ3dTJvYUdrYXlhMnJBQV9ka3QzVXZnZ0t2RFpQaEFndUNPOTZzMHlEXzI1UFlsaFlHTGJDTnFhU2RXZ2JfRFdWMVVieTZmSW96Q1VTVWdWZVgzSW1xTHBxeFhydUZUY2tqZTRMQTh0V2RMOTFycDJoMGl0dVVDaUZXV2hkUVFoalFOZGNMeEVsUlVQWjZrcQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Mosaic e Inpasa assinam novo acordo de barter focado em insumos - CNN Brasil</t>
+          <t>Calluz aposta em calcário com alto teor de magnésio - RCN 67</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -5934,19 +5934,19 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOVm00RUZmWGVBMzJ5Vnc4aDB3ZktTenoyMmJXanVXWF9xYTlNT3VmalhFbk9lYlNiT3h5cFZMdk5qZ0xkUkpTMkM0bkxhNHZvRk51SDZENWliR3FmRUNxMEFJQ3d5U3FNb2hhRUdCWUs2X1UxeFgzQjhMbmItbmhaSzhyQkVFSHF2ZV81UWRVb2VDTF91cnVvVGNZSW0xU28?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE90MUpQNDhERWltS2FYaVNXZ3NvZTNaRmVXMFo4OUZrbUFmODR5REtNSmJDOVd3bnFqTnRZZHctUXV3U2N2OVg2ZDkwRGMyUjVJUkwxX2dSYWdoZ05ZeTNXQnBfdHE2SEY3OF9BQkVFLWVUQW1fejZWRVRR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>AgriConnection e Mosaic lançam Fiagro de até R$ 100 milhões para o mercado de fertilizantes - AgFeed</t>
+          <t>Ureia cai 14% em quatro semanas, mas preço ainda está 43% acima do nível pré-conflito - Agrolink</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOUmlJREVBVDhtRldoNDVjX3RoRkNEYVB1QU13RjFmNmV4MHFNRnp1Qk0wdENJNU41Yk9aVTVNNURDU1V4VUpfczlXOFhUYmlfYUN3NnNnSncxY2RNYWFJQlBXdEZJRmNmSnVTeTRDcmhtU3FzNVdybzliOUJwTkFONTV4MGFydDlxakwtblZiTzNlOEx1cHJxd3BUTlhrYjRyR3RkSmFKc0EyTXRqRDhqV3ZoUGd0YXMxdWxkVjJjTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNcDRET2JCb0V6aVhxVWROTHZEY1Vkcy1wSGFONnVQZGFqY1VmaU1hVFBFRmRIYzVod2tvNm42WlJXVXhxMXB1am5aMnlXYnlnY0V5QU5pWU52TUZaekpsUmJtaXB0NnJEaUpXSUtsMjBrT01KWmZqLVdrWTc4MDVxM3BfWU9KVHhRZHA1TFdGeWtMeXF5dmVDTXJfU05qYVdLSERnZll6WXVaa3ZDOFhWemRQck1YM3lkMkVoXzV3dWluc3c5MTBNdFJvOEFmZlU?oc=5</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Copa do Calcário: Macuco, Monerá e Altense garantem vaga nas semifinais - FERJ</t>
+          <t>Macuco, Monerá e Altense estão na semifinal da Copa Calcário - jornaldaregiao.com</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6044,19 +6044,19 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPNHZMQkhrMlBjTmpobDAwc0lrUFNZd2NqZnlFRzhDU2VfdThPNF96dW5UckVacHdhVWZJTlhJQzFrZ215NTNZaXFTaU1oanN2bTVJR0RVZFpMWG0zUm51My1wckdVTWhJZmJVSV85WUhHNHJxakd1bW5iWTU4aXFWQmkzZnBfa0tad0Exdzl5eExNN2RLd0JpUnU3WUdRNi1vaDB3SEVOZHE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQelB6RDJLanhUTVA5cXJpcC1aMlhDRmJuWnJ3SVl4NGFCWTZPbVI5VW9HcU0xMXd6bEZIQ0tWYTNQejVJQkl6Nmcxc0Z5aS04VEhoNy1qLWNoODdwTmg1LWpMWHRCWVppUkdTLWNQNGlZSU5XQ19BVzFualhvYnFBUXNLejdJWllLQTZleEFLMVI?oc=5</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Como encontrar enxofre em Subnautica 2 - Insider Gaming</t>
+          <t>Copa do Calcário: Macuco, Monerá e Altense garantem vaga nas semifinais - FERJ</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -6066,19 +6066,19 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1DeUNMSGxnbU9GRnk4Y3hGbWNzYldCMzlBd3hfM0N0R1FUcVJoeHRUMWhwYjlMUXhZRktDUU9JMHRIa2E0cTUwWl9Ld201bnF6UmZ1X1hOSl9fQ0xfbV9LVU5jNWdISk0xcE8wcERtaW4xeEZS?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPNHZMQkhrMlBjTmpobDAwc0lrUFNZd2NqZnlFRzhDU2VfdThPNF96dW5UckVacHdhVWZJTlhJQzFrZ215NTNZaXFTaU1oanN2bTVJR0RVZFpMWG0zUm51My1wckdVTWhJZmJVSV85WUhHNHJxakd1bW5iWTU4aXFWQmkzZnBfa0tad0Exdzl5eExNN2RLd0JpUnU3WUdRNi1vaDB3SEVOZHE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Macuco, Monerá e Altense estão na semifinal da Copa Calcário - jornaldaregiao.com</t>
+          <t>Como encontrar enxofre em Subnautica 2 - Insider Gaming</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -6088,7 +6088,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQelB6RDJLanhUTVA5cXJpcC1aMlhDRmJuWnJ3SVl4NGFCWTZPbVI5VW9HcU0xMXd6bEZIQ0tWYTNQejVJQkl6Nmcxc0Z5aS04VEhoNy1qLWNoODdwTmg1LWpMWHRCWVppUkdTLWNQNGlZSU5XQ19BVzFualhvYnFBUXNLejdJWllLQTZleEFLMVI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1DeUNMSGxnbU9GRnk4Y3hGbWNzYldCMzlBd3hfM0N0R1FUcVJoeHRUMWhwYjlMUXhZRktDUU9JMHRIa2E0cTUwWl9Ld201bnF6UmZ1X1hOSl9fQ0xfbV9LVU5jNWdISk0xcE8wcERtaW4xeEZS?oc=5</t>
         </is>
       </c>
     </row>
@@ -6117,12 +6117,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Reunião discute bônus e estabilidade de trabalhadores afetados pela Mosaic - Prefeitura de Araxá</t>
+          <t>BARRAGENS | CMOC Brasil Unidade Ouro promove workshop de segurança - Brasil Mineral</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -6132,19 +6132,19 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOa0hzTkNxSFM2TDh6d24yeVVEb1RzU2dvOTJRRmR3OHRXMl9yNjk2TjNhcEQwLVF4TlBRME9OUVR6ZmFVOTdNZVF4MGZWNDU3dDl5bV9BWk9IcXlUMTZqYmYzUnhibHRQei1WeklNLU1yNkhwRmJqNjBOTi05QkJoUXJsZnJqUEtFZXlIREtZNVBic1N2RkJVMWVVb1BwZGRGZGNodXBDbUNUS2MydU9EUg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOdDFyUHVYU1pJeTZZNzNxUlR2N0RyTlBIaldQT1BORENXVjZ5QmYzMDM5Z2NTUGg4Z0Q4aEtJWktlUS1Ed3c3WjJqOHNwZVhWLTN3c3d4OFVXUWJBNndDa1V5YUliYkNpSWpYN08xWld5MjJUVFVLRmRTVmNfQktGUVppWE9sRExYMTdjZUwxQkdoQmVpUFNsaWdCSjA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>BARRAGENS | CMOC Brasil Unidade Ouro promove workshop de segurança - Brasil Mineral</t>
+          <t>Reunião discute bônus e estabilidade de trabalhadores afetados pela Mosaic - Prefeitura de Araxá</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOdDFyUHVYU1pJeTZZNzNxUlR2N0RyTlBIaldQT1BORENXVjZ5QmYzMDM5Z2NTUGg4Z0Q4aEtJWktlUS1Ed3c3WjJqOHNwZVhWLTN3c3d4OFVXUWJBNndDa1V5YUliYkNpSWpYN08xWld5MjJUVFVLRmRTVmNfQktGUVppWE9sRExYMTdjZUwxQkdoQmVpUFNsaWdCSjA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOa0hzTkNxSFM2TDh6d24yeVVEb1RzU2dvOTJRRmR3OHRXMl9yNjk2TjNhcEQwLVF4TlBRME9OUVR6ZmFVOTdNZVF4MGZWNDU3dDl5bV9BWk9IcXlUMTZqYmYzUnhibHRQei1WeklNLU1yNkhwRmJqNjBOTi05QkJoUXJsZnJqUEtFZXlIREtZNVBic1N2RkJVMWVVb1BwZGRGZGNodXBDbUNUS2MydU9EUg?oc=5</t>
         </is>
       </c>
     </row>
@@ -6227,12 +6227,12 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Ureia cai após meses de valorização - Agrolink</t>
+          <t>Mosaic Fertilizantes tem prejuízo de US$ 422 mi com paralisações em Minas - Diário do Comércio</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -6242,19 +6242,19 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOamEzNkdxNEZfcGNucldUQll1RjZYQzBwZE1sYlh4Ty1MaFdpSUZuckVHTk9uVXU1WTRPLTRLZ2Z1eEVVVU1Wa0haSXZURmhycm0tTEJubGJnZEE3ODRaQmt6bUVkUVlJTkVJWDlTUUVxSWZid3RzOHBhelAwZ082WGs3dkxnMXVwaU9PbQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1OTzdvNnBuejJSeVRQaXZRQXBnTHVzNFoxNUp6dl9JcEVDUlVoUmpEcTNpUXRlSG1nNHVKSTd4d1E0eWFTemR2UzJyWnhYZXB2SFc5RWlILXJnaGpoQjh3N0hxV0R2MVQzbU9BU2EySHpIY0VjVUJ6YWZJM1gyUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Cal Cruzeiro</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Kaio Jorge marca, Cruzeiro suporta pressão e avança às oitavas da Copa do Brasil - tmc.com.br</t>
+          <t>Mosaic registra prejuízo no 1º trimestre e reduz produção diante da alta dos custos de matérias-primas - GlobalFert</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -6264,19 +6264,19 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNajlTUWF0U2hUVWdZek85WmpHOWtqcks2OE5lNHpVczlfZEUwMmdoSm1ub25JQUk1dUIzMFQ0VG9RaExVZXdsbHk4S2ZBdmpuWmd3NEFwZ0tFalVMU1c5UktST0YwUFY4UEtpajBqVUFDV2ZmQ2ZMVW5nb1ZJX1ZmZmZyQnNtbFVUOTBVVGVFRFJoRklnZFFJdm9IUnB3NTdORkRYMTVkS3UzTWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxPUFFYa0l4STNuY0phdjkxVi10MTN0WnVnTGp5bVVrWDRKajFzZm9nRU84MEtLNXdYc3dQZHE2LTNfV2poUGZHZ0xuWGlaS0pRUmRfTlBkeERWMmxYZ3FNd3VYZWQ3ZUdHc3A4eExHeU5ONTRJREpud3ZnZ0puMW81TXJlbFBmdGpWQnljWU5nMURSNDZ2T3psV2tYdjFrNjl4Y3Mya19id3NKUlU2ZEdJcFBQNE02OXRseU9HMmdmaVlBdFdwa3MyaklWX1JVRHBkbERaTWllZXhEZ2NHaFNr?oc=5</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Cal Cruzeiro</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Mosaic Fertilizantes tem prejuízo de US$ 422 mi com paralisações em Minas - Diário do Comércio</t>
+          <t>Kaio Jorge marca, Cruzeiro suporta pressão e avança às oitavas da Copa do Brasil - tmc.com.br</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1OTzdvNnBuejJSeVRQaXZRQXBnTHVzNFoxNUp6dl9JcEVDUlVoUmpEcTNpUXRlSG1nNHVKSTd4d1E0eWFTemR2UzJyWnhYZXB2SFc5RWlILXJnaGpoQjh3N0hxV0R2MVQzbU9BU2EySHpIY0VjVUJ6YWZJM1gyUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNajlTUWF0U2hUVWdZek85WmpHOWtqcks2OE5lNHpVczlfZEUwMmdoSm1ub25JQUk1dUIzMFQ0VG9RaExVZXdsbHk4S2ZBdmpuWmd3NEFwZ0tFalVMU1c5UktST0YwUFY4UEtpajBqVUFDV2ZmQ2ZMVW5nb1ZJX1ZmZmZyQnNtbFVUOTBVVGVFRFJoRklnZFFJdm9IUnB3NTdORkRYMTVkS3UzTWM?oc=5</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Novo revestimento de ureia controla liberação e reduz perdas - Agrolink</t>
+          <t>Ureia cai após meses de valorização - Agrolink</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -6308,19 +6308,19 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQZ01QdFBLLUUtYkI4VmRsYkpIMF9KZ0x4QV9fWGR1ak1YWTQ4enZhMkFCbkQ2dmJFbHgtVlRObml5X1Z3VWZVcnlrd2xSVFlJdzl3ZGdzTjNKUnM1b1pacXlZRjhxZ2RrNEZXWmVaZHBxdzZuMGFyNFJaVEhnVmtOYjJiMVV6enZUODk3bEgzdzRBME5rMkQ2a1NIbklNeGVmWlJ6YWZUamYwQTB4SThBLWxXMzhFcG1jLXFYR3Y5WFd2d3pFT2psV2ItaXRDelhYeURN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOamEzNkdxNEZfcGNucldUQll1RjZYQzBwZE1sYlh4Ty1MaFdpSUZuckVHTk9uVXU1WTRPLTRLZ2Z1eEVVVU1Wa0haSXZURmhycm0tTEJubGJnZEE3ODRaQmt6bUVkUVlJTkVJWDlTUUVxSWZid3RzOHBhelAwZ082WGs3dkxnMXVwaU9PbQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Mosaic registra prejuízo no 1º trimestre e reduz produção diante da alta dos custos de matérias-primas - GlobalFert</t>
+          <t>Novo revestimento de ureia controla liberação e reduz perdas - Agrolink</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxPUFFYa0l4STNuY0phdjkxVi10MTN0WnVnTGp5bVVrWDRKajFzZm9nRU84MEtLNXdYc3dQZHE2LTNfV2poUGZHZ0xuWGlaS0pRUmRfTlBkeERWMmxYZ3FNd3VYZWQ3ZUdHc3A4eExHeU5ONTRJREpud3ZnZ0puMW81TXJlbFBmdGpWQnljWU5nMURSNDZ2T3psV2tYdjFrNjl4Y3Mya19id3NKUlU2ZEdJcFBQNE02OXRseU9HMmdmaVlBdFdwa3MyaklWX1JVRHBkbERaTWllZXhEZ2NHaFNr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQZ01QdFBLLUUtYkI4VmRsYkpIMF9KZ0x4QV9fWGR1ak1YWTQ4enZhMkFCbkQ2dmJFbHgtVlRObml5X1Z3VWZVcnlrd2xSVFlJdzl3ZGdzTjNKUnM1b1pacXlZRjhxZ2RrNEZXWmVaZHBxdzZuMGFyNFJaVEhnVmtOYjJiMVV6enZUODk3bEgzdzRBME5rMkQ2a1NIbklNeGVmWlJ6YWZUamYwQTB4SThBLWxXMzhFcG1jLXFYR3Y5WFd2d3pFT2psV2ItaXRDelhYeURN?oc=5</t>
         </is>
       </c>
     </row>
@@ -6359,12 +6359,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Margens derretem no Brasil e Mosaic começa 2026 no vermelho (mesmo com alta na receita) - AgFeed</t>
+          <t>Demanda fraca derruba preços da ureia mas não destrava mercado - CNN Brasil</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -6374,19 +6374,19 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxORklOTkFqdEJTSkRkVUgwalFVWjdVOVNRTjZzOFBhS1h4Xzl1YnM4dU56QWY3UnFHeVdpaGNFdnVwTzctWURPQUVwZExqN1MzZWYwemxndGxVVE93eUxybzEzQVFxbkVWWVJhMU5hOHU5TGpUTGNRZ1dWVXRuV2xBNHZBMUprWEpYYnYyX3Y3ekhRbVNvWWpfSVpYZ1NTeURnOXJfc1Z2eUFERkh5TlZGUjBmMzlKS1ox?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxONnJwX0hzX1RaX3dlVGxVVjVBczRMV3Jtd1dBaXBNeU4tVUFJLU9iNGNPY0JKSGFxUjBUVDlONWNvNDRrd1NLOTFWYTJPNjFhVGVIUW4xVDNyWlE3OVlmWjhQWUgyZk0wOU56bTJfcTJ3dkJCYU9Ub0JSUVlMWDFCT0txUzU0ZlJJNXpTMGlnRUw1cjhwd25rYjAyNjBvdw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Cal Cruzeiro</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Polícia Militar apreende arma de fogo, munições e drogas no bairro Jardim Cruzeiro - Acorda Cidade</t>
+          <t>COMMODITIES | Enxofre impacta aumento do preço do níquel na Indonésia - Brasil Mineral</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNMkN6R0NicFFIMjViTjNQYWFwZ2xLUEhFNWw3UTJnMENJcEJKS0pmWWhsRTRRMFpObEhjU0dOdTU0Y2tyT0h5Q21MaVhhM2NkWHFtQ0RzTGZJWUVTbGNCQzFCN0RfZ19KS1ZXa2FhS2E4bHY4VG5ybVJIc3VhbnZHWlRRZEFZeXJSTG1HenJDNFZqSWRocmdDdW9JTjc0d05IRGNsWTRja09ZMkxKYW1uRWNCMFZXV3NTMmZyTlpVZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQVkZIWHBTbDkyUzZ6RktMXzZBenVZRWFfN1NTeUxRaDJGSkxTVmlmamFpM2ZxdjlTQWV6WHJtMG9EU1Jzd094RnpXQVZDQ0lQWVhTWXM2bDYtNWRNYkdpcFlhWUtGN0tvWXR4SXJXUTNlcWhKQzBxWXJGalV2Zk1rX1B4LXpyNEN0b3lEWkZwQ3lLUnB4VGM0ZnA3clFnQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -6425,12 +6425,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Lhoist</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Mosaic tem prejuízo líquido de US$ 258 milhões no trimestre - CNN Brasil</t>
+          <t>Lhoist avança na jornada sustentável com operação de caminhão elétrico - Jornal Correio Centro Oeste Arcos</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOZC1GeGtLMy0wY2l4ay1zQ3RUblZncTFoTzdEM2s3b3dQeEdWQjZ5X2ZDLTI3VDNJZkdwQTl0S3N2UGN1OUw5Q2Vla19aS0p1RV91R3JMN0RzOVd3UGJnNGh0N1BCckRvSndoMmxYMERNU2RIQ0wwRlR6U19nb2h6bHJoWEEyeWxIN0xrYnFfdTlFT3VMMDlrMg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPUzRlUV9RRTlBUlptdlZCSXNGbG1laThEN09iMTh3TkF0NUxHcTV4Ujd3bktsME9mY29RT2lUaXQ0dDhyeTBHSTZzM3R3ZldLbXhQRUxOd0ZsdndzUm1pSXUwZTRkY0Jfbkp1V3YyTjIydFppYk83ODhoRUlVMlNOVWdNem5LcS1qRWZ0bGlGVGdGcnk0clNVbGpKV2VVOXNs?oc=5</t>
         </is>
       </c>
     </row>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Mosaic registra prejuízo de US$ 258 milhões no primeiro trimestre - Valor Econômico</t>
+          <t>Margens derretem no Brasil e Mosaic começa 2026 no vermelho (mesmo com alta na receita) - AgFeed</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -6462,19 +6462,19 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNNDNrdFRsS2JuRFptTkVYV0YyVUtodDQ0c042RjJoQy16R09COHFtYmUyekVpc042X25qN2Nkc2x4bmFlTnBSa0htTGVCSHk1bTBMcGs1UlRWaHJLV1VzaTZJNy1YQy1VQ2w3T2tCOTJxbEt2OVB3X081VDFoVnlod2lCQVdQa2RSZ2dHd2JBTjVJTUJOUVJEQUZFVW9POTRhT1IwRm1YbzFKUHN2VGRlWmJJOXB3anM3Y3MtWmI5N2JKcFJy0gHTAUFVX3lxTFBVMWFxcFVLcTAwdDJ4YU1mVlh4MC1Fa3RKSmZWQ0poM01heVJ1MnRJczJJcm9NT244T2ViX0p4ZFg4QURiM3FMLUh1WEJmdTE4Y0Y5cEs2Q3R1aDhPX0tvRlM2QzB5MXFyS3drZll4al9FanByZ0FZV3hNMlZja1VhV0stY0hpejczVzZrbGxyeEVBYkRVaWFCbmdwWW9Fa3FCb0YydmZiNGxsVmUyLXNNeVpmRV9XZG5LaGRGdmRqN1h0ZXFXa1VPZUVhdmNOMFQzV3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxORklOTkFqdEJTSkRkVUgwalFVWjdVOVNRTjZzOFBhS1h4Xzl1YnM4dU56QWY3UnFHeVdpaGNFdnVwTzctWURPQUVwZExqN1MzZWYwemxndGxVVE93eUxybzEzQVFxbkVWWVJhMU5hOHU5TGpUTGNRZ1dWVXRuV2xBNHZBMUprWEpYYnYyX3Y3ekhRbVNvWWpfSVpYZ1NTeURnOXJfc1Z2eUFERkh5TlZGUjBmMzlKS1ox?oc=5</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Lhoist</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Lhoist avança na jornada sustentável com operação de caminhão elétrico - Jornal Correio Centro Oeste Arcos</t>
+          <t>Mosaic tem prejuízo líquido de US$ 258 milhões no trimestre - CNN Brasil</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -6484,19 +6484,19 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPUzRlUV9RRTlBUlptdlZCSXNGbG1laThEN09iMTh3TkF0NUxHcTV4Ujd3bktsME9mY29RT2lUaXQ0dDhyeTBHSTZzM3R3ZldLbXhQRUxOd0ZsdndzUm1pSXUwZTRkY0Jfbkp1V3YyTjIydFppYk83ODhoRUlVMlNOVWdNem5LcS1qRWZ0bGlGVGdGcnk0clNVbGpKV2VVOXNs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOZC1GeGtLMy0wY2l4ay1zQ3RUblZncTFoTzdEM2s3b3dQeEdWQjZ5X2ZDLTI3VDNJZkdwQTl0S3N2UGN1OUw5Q2Vla19aS0p1RV91R3JMN0RzOVd3UGJnNGh0N1BCckRvSndoMmxYMERNU2RIQ0wwRlR6U19nb2h6bHJoWEEyeWxIN0xrYnFfdTlFT3VMMDlrMg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Cal Cruzeiro</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Demanda fraca derruba preços da ureia mas não destrava mercado - CNN Brasil</t>
+          <t>Polícia Militar apreende arma de fogo, munições e drogas no bairro Jardim Cruzeiro - Acorda Cidade</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -6506,19 +6506,19 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxONnJwX0hzX1RaX3dlVGxVVjVBczRMV3Jtd1dBaXBNeU4tVUFJLU9iNGNPY0JKSGFxUjBUVDlONWNvNDRrd1NLOTFWYTJPNjFhVGVIUW4xVDNyWlE3OVlmWjhQWUgyZk0wOU56bTJfcTJ3dkJCYU9Ub0JSUVlMWDFCT0txUzU0ZlJJNXpTMGlnRUw1cjhwd25rYjAyNjBvdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNMkN6R0NicFFIMjViTjNQYWFwZ2xLUEhFNWw3UTJnMENJcEJKS0pmWWhsRTRRMFpObEhjU0dOdTU0Y2tyT0h5Q21MaVhhM2NkWHFtQ0RzTGZJWUVTbGNCQzFCN0RfZ19KS1ZXa2FhS2E4bHY4VG5ybVJIc3VhbnZHWlRRZEFZeXJSTG1HenJDNFZqSWRocmdDdW9JTjc0d05IRGNsWTRja09ZMkxKYW1uRWNCMFZXV3NTMmZyTlpVZw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>COMMODITIES | Enxofre impacta aumento do preço do níquel na Indonésia - Brasil Mineral</t>
+          <t>Mosaic registra prejuízo de US$ 258 milhões no primeiro trimestre - Valor Econômico</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQVkZIWHBTbDkyUzZ6RktMXzZBenVZRWFfN1NTeUxRaDJGSkxTVmlmamFpM2ZxdjlTQWV6WHJtMG9EU1Jzd094RnpXQVZDQ0lQWVhTWXM2bDYtNWRNYkdpcFlhWUtGN0tvWXR4SXJXUTNlcWhKQzBxWXJGalV2Zk1rX1B4LXpyNEN0b3lEWkZwQ3lLUnB4VGM0ZnA3clFnQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNNDNrdFRsS2JuRFptTkVYV0YyVUtodDQ0c042RjJoQy16R09COHFtYmUyekVpc042X25qN2Nkc2x4bmFlTnBSa0htTGVCSHk1bTBMcGs1UlRWaHJLV1VzaTZJNy1YQy1VQ2w3T2tCOTJxbEt2OVB3X081VDFoVnlod2lCQVdQa2RSZ2dHd2JBTjVJTUJOUVJEQUZFVW9POTRhT1IwRm1YbzFKUHN2VGRlWmJJOXB3anM3Y3MtWmI5N2JKcFJy0gHTAUFVX3lxTFBVMWFxcFVLcTAwdDJ4YU1mVlh4MC1Fa3RKSmZWQ0poM01heVJ1MnRJczJJcm9NT244T2ViX0p4ZFg4QURiM3FMLUh1WEJmdTE4Y0Y5cEs2Q3R1aDhPX0tvRlM2QzB5MXFyS3drZll4al9FanByZ0FZV3hNMlZja1VhV0stY0hpejczVzZrbGxyeEVBYkRVaWFCbmdwWW9Fa3FCb0YydmZiNGxsVmUyLXNNeVpmRV9XZG5LaGRGdmRqN1h0ZXFXa1VPZUVhdmNOMFQzV3M?oc=5</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Carga de enxofre é derramada na Rodovia Ayrton Senna após acidente entre dois caminhões em Itaquaquecetuba - G1</t>
+          <t>Vazamento de enxofre interdita rodovia Ayrton Senna, em São Paulo - band.com.br</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPMjJXYVBLSHRScWpkR1pXa1F4R1Q2R1N5UzczQ3JGSkxaaGJrOUc5aGVzbU4xZTJ6WVVBMTVJeWJLS0l3VmlUMExTT09oUmFEbUR0ZldLTXUwSmJ2UkR1MFVCUkN2dzMzLWxtTkNfOGh5aFdyNjJzVUM2Wkgyc1dfcEJDUnZCQk4xUUR5cjZpT2VfNHlxVUFZYVphTTNWd2Y1U1NUTy1fcnFIM2p6S3dpR1BfMHRKeG1yS2ppVm5sTmMwZk3SAdIBQVVfeXFMTmVyUjFibUtlTnhSRkRwbFl2LVQ2RE9BdTdQRUM0Z2dSUmF6RnFRUlNrS3pIZzNBTy10NDdEWXBNYTVJZlB6X05CeTQycjdjelI4c1VHZ2QxRDdia0s5NFR0b3p1aGZPUi1RQlBiTDlRY3RLekdXXzBBdzQ2RUVLRDRhNGxlSUZBbjJXVlRKRkV1ZjhxXzlkanRqZmdERzZYemJnOFRzRWNLTHd1SnIxSmk0T3dtT2NhWHJiTjRUM0ZUbkVIdmZUS3R4OVJueS1LbzRR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPYzM4TXRIamotWmZsZG83T0prMmNwb0ZRSnVFY3UxTEFqWnJIWVlmLW9Db3VzX1FSaURNN0RodkhTaGw2R0JkcHFIQWEwV2tPN2tUVnRVYzItUkNRUGQ0UFR4ZmZtWmJRbldEVzB1RWxzLVpfamZUUWVEdU9oZ2xMcHE5cFAtZVhvQXcxTjhERXcwWnJhenhjSmFfSk0wRUdJN184RlMwbEU5aWtHN0JOdmxUVXI1ZW1mZjBHUw?oc=5</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Carga de enxofre cai na pista da Rodovia Ayrton Senna após acidente - G1</t>
+          <t>Carga de enxofre é derramada na Rodovia Ayrton Senna após acidente entre dois caminhões em Itaquaquecetuba - G1</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -6572,7 +6572,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPVURlU1pkY2xFUkxKczI2WGNkZnJBMk1MOHhSRTI2ZEJWMUhfdjBFU1F1TGpMbUl6eVkxc1FWOWlheHNpN1hIQ3NRejI1Y2dsbHZwTS1fSmlJZnFtWWZuM2gtUUZhblBKdGFMelF1cTdLN0xJUWd2dkh2UUQwWGlBUGgyTDdtLWtVRXJrc3FXX3pmZENBb0RKc21MVndkUHR6VGxYM0RjN3FMelhpOF9zQmgtTkNnNy01QVl1ZFg2eXV1b3MzdUxFYTFPeUZWQdIB3AFBVV95cUxNNVFUeU9TN3Z2S3N5M240dmZOTmg3VnNjX1p4NzZkdXl5NU4zc0dFbGEySjJ3enNQb3VPSkdGdGJBVHVBZ2dLa3hxUnNsX1JPQmNiX2RKVEE2SE1KemhlbnhPLTJRc3U5VnRFeVpXdThGNFlXZDk0YjlyazlxTWNfT3o3R2RfVVBrSi1TNWlJQjQ1VnY2b0tienVBSlpvbHhJbWtCLU0xamNJWTRMLTA0bmFLZ2dhRm1SSm9VVjI2ZmtobWxpd3J5aDNFajFOODJ2U3NyVnNJNjFLRzQy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPMjJXYVBLSHRScWpkR1pXa1F4R1Q2R1N5UzczQ3JGSkxaaGJrOUc5aGVzbU4xZTJ6WVVBMTVJeWJLS0l3VmlUMExTT09oUmFEbUR0ZldLTXUwSmJ2UkR1MFVCUkN2dzMzLWxtTkNfOGh5aFdyNjJzVUM2Wkgyc1dfcEJDUnZCQk4xUUR5cjZpT2VfNHlxVUFZYVphTTNWd2Y1U1NUTy1fcnFIM2p6S3dpR1BfMHRKeG1yS2ppVm5sTmMwZk3SAdIBQVVfeXFMTmVyUjFibUtlTnhSRkRwbFl2LVQ2RE9BdTdQRUM0Z2dSUmF6RnFRUlNrS3pIZzNBTy10NDdEWXBNYTVJZlB6X05CeTQycjdjelI4c1VHZ2QxRDdia0s5NFR0b3p1aGZPUi1RQlBiTDlRY3RLekdXXzBBdzQ2RUVLRDRhNGxlSUZBbjJXVlRKRkV1ZjhxXzlkanRqZmdERzZYemJnOFRzRWNLTHd1SnIxSmk0T3dtT2NhWHJiTjRUM0ZUbkVIdmZUS3R4OVJueS1LbzRR?oc=5</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Vazamento de enxofre interdita rodovia Ayrton Senna, em São Paulo - band.com.br</t>
+          <t>Carga de enxofre cai na pista da Rodovia Ayrton Senna após acidente - G1</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPYzM4TXRIamotWmZsZG83T0prMmNwb0ZRSnVFY3UxTEFqWnJIWVlmLW9Db3VzX1FSaURNN0RodkhTaGw2R0JkcHFIQWEwV2tPN2tUVnRVYzItUkNRUGQ0UFR4ZmZtWmJRbldEVzB1RWxzLVpfamZUUWVEdU9oZ2xMcHE5cFAtZVhvQXcxTjhERXcwWnJhenhjSmFfSk0wRUdJN184RlMwbEU5aWtHN0JOdmxUVXI1ZW1mZjBHUw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPVURlU1pkY2xFUkxKczI2WGNkZnJBMk1MOHhSRTI2ZEJWMUhfdjBFU1F1TGpMbUl6eVkxc1FWOWlheHNpN1hIQ3NRejI1Y2dsbHZwTS1fSmlJZnFtWWZuM2gtUUZhblBKdGFMelF1cTdLN0xJUWd2dkh2UUQwWGlBUGgyTDdtLWtVRXJrc3FXX3pmZENBb0RKc21MVndkUHR6VGxYM0RjN3FMelhpOF9zQmgtTkNnNy01QVl1ZFg2eXV1b3MzdUxFYTFPeUZWQdIB3AFBVV95cUxNNVFUeU9TN3Z2S3N5M240dmZOTmg3VnNjX1p4NzZkdXl5NU4zc0dFbGEySjJ3enNQb3VPSkdGdGJBVHVBZ2dLa3hxUnNsX1JPQmNiX2RKVEE2SE1KemhlbnhPLTJRc3U5VnRFeVpXdThGNFlXZDk0YjlyazlxTWNfT3o3R2RfVVBrSi1TNWlJQjQ1VnY2b0tienVBSlpvbHhJbWtCLU0xamNJWTRMLTA0bmFLZ2dhRm1SSm9VVjI2ZmtobWxpd3J5aDNFajFOODJ2U3NyVnNJNjFLRzQy?oc=5</t>
         </is>
       </c>
     </row>
@@ -6623,12 +6623,12 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Preço futuro da ureia para 2026 cai forte no início de maio - Farmnews</t>
+          <t>Alta do enxofre pressiona uso de fosfatado no país - Agrolink</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -6638,19 +6638,19 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQZENuS3MwY1NDNlVENVlLT3FhbGpTMUZacGNmc3lKR2NINjRRdkNGUndsRW1QaEhPVG1yMkx5eG5mYTRpMENzbXRVVVlZSXFPQnJKMF9UbjBNeW1xTTl0cXdjOEpMQk5CaktWT0c0anZvVEFwQkQ3LXdhRWkzNXN5eE9yTldTUzg5Ul9QLWo2WWZDbk5BbUMw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPUUZENVBnUk80LW5TNnBRdFNyeU12V2xuTnpKT1k1dk1ySmhXWmJZU0V4SDF4dnduV3Exck9vUTI4SU9OX3BROHc1NG1Jbm82S2FQVTEzdE9lR2xwV2h2ZGhGWGJvYW1tXzdNSHR4ZGExRWU4WFRXZnZkb2x3UWV1OFFPVFBVTWFibkZDLVZCMUpKRExEa2RyVUdsR3pCT0gx?oc=5</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Alta do enxofre pressiona uso de fosfatado no país - Agrolink</t>
+          <t>Preço futuro da ureia para 2026 cai forte no início de maio - Farmnews</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -6660,7 +6660,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPUUZENVBnUk80LW5TNnBRdFNyeU12V2xuTnpKT1k1dk1ySmhXWmJZU0V4SDF4dnduV3Exck9vUTI4SU9OX3BROHc1NG1Jbm82S2FQVTEzdE9lR2xwV2h2ZGhGWGJvYW1tXzdNSHR4ZGExRWU4WFRXZnZkb2x3UWV1OFFPVFBVTWFibkZDLVZCMUpKRExEa2RyVUdsR3pCT0gx?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQZENuS3MwY1NDNlVENVlLT3FhbGpTMUZacGNmc3lKR2NINjRRdkNGUndsRW1QaEhPVG1yMkx5eG5mYTRpMENzbXRVVVlZSXFPQnJKMF9UbjBNeW1xTTl0cXdjOEpMQk5CaktWT0c0anZvVEFwQkQ3LXdhRWkzNXN5eE9yTldTUzg5Ul9QLWo2WWZDbk5BbUMw?oc=5</t>
         </is>
       </c>
     </row>
@@ -6689,12 +6689,12 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Preços da ureia começam a desacelerar após forte alta com conflito - CNN Brasil</t>
+          <t>Mineração vira aposta bilionária no Equador: China fecha acordo de US$ 1,7 bilhão para explorar uma das maiores jazidas de ouro do país, promete US$ 4,39 bilhões ao Estado e amplia sua força na América do Sul - CPG Click Petróleo e Gás</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPd0VHZGk0YmpqT3Jzd0hnMVRySDYzYU9wZC1ieXJPc1dPX081SkpEdDZNUUNBYUJMWlNNVk5mQVp0eEdPNVA3d1B2d1VTREo3QmJvYkQ1YjZfdG9zMHgzTnludnA4U1VFcUNCd1d0SjVzWDdYd0JNM2xSLWs1czZmcTVPZllkTkdDbFlPblQ4MEttaUdySWo1enhoakxocEk5SVpF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAJBVV95cUxNYWlRUWx5RGM2b3h1UEJTdzNRcmRXVzRRQjBWcFY5cDRiVjhwMUIyeE9tdGh5LXUxLU5QcUxxNDBfQkVYa3BWVUV0enZxYlh5cDVISlNNY1ZRVXd6LXY0bFgwQ2diUUp6YmtWb3gtSTZQR0hfUmE5Y2dpWXk4RW03MVVfODFZNmt0Y2hORTQ3TEZrWmR5TXdfWlNuLU9HSTItUGQwb1R5R25zWi04ZzdsU3VWcjJUVnJzaFdzT2pQQkp4RDBSR0NOX3hmXzBmSGdxQk5hcU1aM2ZLMkJkRmpZRjI1enBHN25HVWw1TFVpMUxfTTY3bF9hdUxQZHZzTFpPaDloMzh0cmJfZUUxeWJHSUNxdXFkcnFVQW1Bb2xQYnhYZ1J6U2xJNWtRbkZHbS1D?oc=5</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Após forte alta, preço da ureia começa a cair, mostra levantamento - Canal Rural</t>
+          <t>Preços da ureia começam a desacelerar após forte alta com conflito - CNN Brasil</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -6748,19 +6748,19 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQcUZLcjlzMlFBNFM4Nlo2U2ZYdk1hc2YyOGg3Rng2VThuZVY3cXk2V1BXNWFjaWQyb3lvbnM1d2E0b1BwVFYwZzhEX2drSWxyQllLQlM5S25Uamd6U0pYTVo0cjFjcjRHMGJVXzQ0SUM3V2tIR3hpTER6NjF0OUZ2T1VNNWxyeWloRjlTRDlqSkhtcTFBQk50akZscERXME9DRjF4dWtnaGRvbFU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPd0VHZGk0YmpqT3Jzd0hnMVRySDYzYU9wZC1ieXJPc1dPX081SkpEdDZNUUNBYUJMWlNNVk5mQVp0eEdPNVA3d1B2d1VTREo3QmJvYkQ1YjZfdG9zMHgzTnludnA4U1VFcUNCd1d0SjVzWDdYd0JNM2xSLWs1czZmcTVPZllkTkdDbFlPblQ4MEttaUdySWo1enhoakxocEk5SVpF?oc=5</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Mineração vira aposta bilionária no Equador: China fecha acordo de US$ 1,7 bilhão para explorar uma das maiores jazidas de ouro do país, promete US$ 4,39 bilhões ao Estado e amplia sua força na América do Sul - CPG Click Petróleo e Gás</t>
+          <t>Rodada quente e com muitos gols na Copa do Calcário - FERJ</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAJBVV95cUxNYWlRUWx5RGM2b3h1UEJTdzNRcmRXVzRRQjBWcFY5cDRiVjhwMUIyeE9tdGh5LXUxLU5QcUxxNDBfQkVYa3BWVUV0enZxYlh5cDVISlNNY1ZRVXd6LXY0bFgwQ2diUUp6YmtWb3gtSTZQR0hfUmE5Y2dpWXk4RW03MVVfODFZNmt0Y2hORTQ3TEZrWmR5TXdfWlNuLU9HSTItUGQwb1R5R25zWi04ZzdsU3VWcjJUVnJzaFdzT2pQQkp4RDBSR0NOX3hmXzBmSGdxQk5hcU1aM2ZLMkJkRmpZRjI1enBHN25HVWw1TFVpMUxfTTY3bF9hdUxQZHZzTFpPaDloMzh0cmJfZUUxeWJHSUNxdXFkcnFVQW1Bb2xQYnhYZ1J6U2xJNWtRbkZHbS1D?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxObWdVQ1R0NC1YZThsV1NPR1p3bnY1S3JpZ29Rd1l5dWtYNkUycTlma1FrUUNmLU91aF94eFlSa01qMmszRUgzWkoyd0xQWnhHS0RDRF9oSnd2N29lQUROVDhiUzJjUmlWcWw5SDViQnh3MWY2SGJiVVREX1dyYkN3S3RsWnlfcTBX?oc=5</t>
         </is>
       </c>
     </row>
@@ -6782,7 +6782,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Após disparada, ureia perde sustentação e inicia movimento de queda global - Notícias Agrícolas</t>
+          <t>Após forte alta, preço da ureia começa a cair, mostra levantamento - Canal Rural</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxONTVhVThiOV9DeDdTeWhZaFR1dmZZWm5GMmpYSXR3SHFBT0U3MWItc2xEcGRPZVBLXzRvbmNqY2J3TlcxM243aFA0RElmS0djdmhzTC03bnZjQUotUnZkQ1REcExJYmxHTUlkZkxyOGtWUHpRZC14eVMtSGszNndqWTc2R3VhUlZhQnFYQXUxR2ZUdk01MUxFUVlKaWMyX1NBVWFtbU1rNnhMNTBfYWxoTm9wX1daT3MyU1ExNTlNU1pOb25FbGFBSy1QWFgzX3hheDRWSVdfNTlXRnPSAeABQVVfeXFMTnQ0NzRKRFItenRCVzlHMFJMUWNBem1GQ1lTWkdHZm54cy11cURxamdwMHp5MUJ2bVZmWVRoWThDejhvTVlWYU53OHBpMTNmYnZ1ZWNNQ2xDWW5ILUVmUDJBMktfRjRYc3ZSeUJXWU5PNEpKUDFoeU52RmZSRlBZcUVXV2p4Q3FCel9iTTU2aVV6V29nZXdTNmdlMnBxUWFqNWhtbnc3ZmpqZm5IUHFvYnJueFpzMldlcnBxSXZHbUxjNHdTRDFCRl9zSTBpdDJGWGlHMmpfRkVxRm1sOHJmTXI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQcUZLcjlzMlFBNFM4Nlo2U2ZYdk1hc2YyOGg3Rng2VThuZVY3cXk2V1BXNWFjaWQyb3lvbnM1d2E0b1BwVFYwZzhEX2drSWxyQllLQlM5S25Uamd6U0pYTVo0cjFjcjRHMGJVXzQ0SUM3V2tIR3hpTER6NjF0OUZ2T1VNNWxyeWloRjlTRDlqSkhtcTFBQk50akZscERXME9DRjF4dWtnaGRvbFU?oc=5</t>
         </is>
       </c>
     </row>
@@ -6804,7 +6804,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Preços da ureia cedem após dois meses em alta - Globo Rural</t>
+          <t>Após disparada, ureia perde sustentação e inicia movimento de queda global - Notícias Agrícolas</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -6814,19 +6814,19 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPQTFfM1dYaG9xa0s1eXk4bXRQb0d6V2Q0NzFvOEJ4dlB2b2NRMlkxRE5ZZUZQdlV1ZFdyWGljN3Z5RVRFUTVuTjZ4cDIyUDdrZWpWMUJtNHJrZmxsWV9zZkRobXoyd0VBRXFvYXB0WDFsSC1vMDZBN2haLXYyUFp6UWtzQTlYb0xSMERMWElPN3FZSDFQN0l4ckd1U3RIaDM4cnRNNUoyUdIBtgFBVV95cUxOVlRkd0NYWjUzZEhHblM0eGlJdjlNblRaWDAwWWlNclRFbXVYY3VBQmczNVpEdWdzOXJqNHY5dUVZVWVYMzNsNHNsRTYxenZkMXRqQkNYUlU3YWxWajc5NmZld2dwRmRzaER1T1lTdG1KZ0hUdVJqeW9kNDBjWTRfaHo5eG1oZThZTzVsQ0M2aXljcURYWk1YWGdxeno1M1JkTTlZZjVKR2x5U2xrTUNSeUJfMmRJdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxONTVhVThiOV9DeDdTeWhZaFR1dmZZWm5GMmpYSXR3SHFBT0U3MWItc2xEcGRPZVBLXzRvbmNqY2J3TlcxM243aFA0RElmS0djdmhzTC03bnZjQUotUnZkQ1REcExJYmxHTUlkZkxyOGtWUHpRZC14eVMtSGszNndqWTc2R3VhUlZhQnFYQXUxR2ZUdk01MUxFUVlKaWMyX1NBVWFtbU1rNnhMNTBfYWxoTm9wX1daT3MyU1ExNTlNU1pOb25FbGFBSy1QWFgzX3hheDRWSVdfNTlXRnPSAeABQVVfeXFMTnQ0NzRKRFItenRCVzlHMFJMUWNBem1GQ1lTWkdHZm54cy11cURxamdwMHp5MUJ2bVZmWVRoWThDejhvTVlWYU53OHBpMTNmYnZ1ZWNNQ2xDWW5ILUVmUDJBMktfRjRYc3ZSeUJXWU5PNEpKUDFoeU52RmZSRlBZcUVXV2p4Q3FCel9iTTU2aVV6V29nZXdTNmdlMnBxUWFqNWhtbnc3ZmpqZm5IUHFvYnJueFpzMldlcnBxSXZHbUxjNHdTRDFCRl9zSTBpdDJGWGlHMmpfRkVxRm1sOHJmTXI?oc=5</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Rodada quente e com muitos gols na Copa do Calcário - FERJ</t>
+          <t>Preços da ureia cedem após dois meses em alta - Globo Rural</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -6836,7 +6836,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxObWdVQ1R0NC1YZThsV1NPR1p3bnY1S3JpZ29Rd1l5dWtYNkUycTlma1FrUUNmLU91aF94eFlSa01qMmszRUgzWkoyd0xQWnhHS0RDRF9oSnd2N29lQUROVDhiUzJjUmlWcWw5SDViQnh3MWY2SGJiVVREX1dyYkN3S3RsWnlfcTBX?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPQTFfM1dYaG9xa0s1eXk4bXRQb0d6V2Q0NzFvOEJ4dlB2b2NRMlkxRE5ZZUZQdlV1ZFdyWGljN3Z5RVRFUTVuTjZ4cDIyUDdrZWpWMUJtNHJrZmxsWV9zZkRobXoyd0VBRXFvYXB0WDFsSC1vMDZBN2haLXYyUFp6UWtzQTlYb0xSMERMWElPN3FZSDFQN0l4ckd1U3RIaDM4cnRNNUoyUdIBtgFBVV95cUxOVlRkd0NYWjUzZEhHblM0eGlJdjlNblRaWDAwWWlNclRFbXVYY3VBQmczNVpEdWdzOXJqNHY5dUVZVWVYMzNsNHNsRTYxenZkMXRqQkNYUlU3YWxWajc5NmZld2dwRmRzaER1T1lTdG1KZ0hUdVJqeW9kNDBjWTRfaHo5eG1oZThZTzVsQ0M2aXljcURYWk1YWGdxeno1M1JkTTlZZjVKR2x5U2xrTUNSeUJfMmRJdw?oc=5</t>
         </is>
       </c>
     </row>
@@ -6909,12 +6909,12 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Mercado de fertilizantes vive momento mais difícil em décadas, diz Mosaic - The AgriBiz</t>
+          <t>Em meio à crise dos fertilizantes, Petrobras volta a produzir ureia no Paraná após seis anos - VEJA</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -6924,7 +6924,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNZXpsRmRrRjkycUpIaUJaY1V2cWxzelVBZnAtTm5ETEdJY1lQTUUtTHFVMkNBTkZyem9xVHUtS1cyaVpmSHdnc3doMTdFWkdGTThsbEJNU3dFSDVIRjZIaUlxODlHd2F1cUdJU3NuTGpQT01OMUN3MnhkR3o4S2gwd1dMMWR2QV81X2tOZ21PS2JIbU5STlAzT1hNV0wyczdVbHlLMGtFVFVpYXlHMnFyNk1UVmo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNU2E5eUdWYzFxMHoxdzFrdktxNndmLXhpOC1mY0kwcUVPdWpoVnVkZVgxRXZQY1N2UFJNRmozQ0p5UVlWREZKaGFLMWR6WUU0UmxSTG5xaE1lSWJ1QjdaOWhMQVNUY29Lams4WnE3bS1Tb3JhaUR6MDJSbWtkUU9ZOGlvSS1IOHFWSGJjY01PYTBkN1d0UE5xWHZTTDFmUEpiUTEwN1BQWWNpZnRXRjBxLXR4MktvUWJOMzRfVVl5TWNwRENEUnc?oc=5</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Petrobras inicia produção de ureia na Ansa, unidade que estava hibernada desde 2020 - Valor Econômico</t>
+          <t>Fafen PR volta a produzir ureia: fertilizante na fábrica é comida na mesa! - FUP - Federação Única dos Petroleiros</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNcVNQNzR3X3ZiZC1IbXR0Q1U5M3d4TXVWcTNMRU1GOGhOd0pKYkpXeUpnS2VkcHJieWpNVDhUdnpDeFlud29jWEFSZ2Z1MjJIVE90QmpIc2NSbkxlbG5iQW1xeVZsU1hiS0RrR2hDTDVmU3duTFpBTGRjbGRtLWdjWkF1cnFtVU1YRkN4VTNOU1JLZm5hakh0RWFsblV2SlNhT1d2djhINGN4MTlSX0xfZXBncFRmbUVVdlppWFlhSXF5T2xuMnFiNWlla1VkcFVPWi02WVNkONIB5gFBVV95cUxORWpyQ285M1U3ekpPWWVwMER6dTNMTWlZZ3h3VFBwSmRiZ1Y0dnZvb0NtaVlXR0FSank5ZklXMkl6NUhFcG1wcWFuX3lld0VSeFktQU1PUUxESFg5VE0zRlBPaVNfb1VFZTE3ZUFsRDB4N1ZYVUo1dXMxN210RW84LU5scWp4MXppTEZLWFlEeC1mdE9hYkhOTmNoaVUzOFA2d3lvVkZ1cWxCM1A5YWxMUW0tamkxS3BqSUNxRUlWcFo1cUZ2bFVtdlIyd2xKM2FjQTBkcmJjVWdtSlI4WFNlRkxHZlBQdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPcmtibVp2QVZDY19yQXhVZC1ybWpjb0dqUXhGMlo5OFhodXpBczFOWThhLTc3RHBvdHNxVU9iSXZyQnVMdm8xUmtWbkNNcHRTWUYweXNpcTc3bUI5Ym56Z1pzckdTazllVFRzTzVrLUVJYm5ydDlkXy1mclNEdTlncWVFN0g5U1JfbnBoTmVzTTE1eHJCVDdF?oc=5</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Petrobras inicia produção de ureia em unidade no Paraná - InfoMoney</t>
+          <t>Petrobras inicia produção de ureia em usina desativada há 6 anos - Poder360</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -6990,19 +6990,19 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOR2lLUEZxMlhlTzhWUGp5WmZaaFA2RV80WkpYazZtVXd2ZldSM2ZzaFBHNnFNTFpIZ1JVLTdZWUxnMzJMOERZTHV6SXN4ZDJieFdqS05ZWFpvbVdMVXRqNmo4VWZ1OXpMZDl5bS14UjgtQ1RtVmRFZmZmZmg4cXhlLXptYjRjMzNPTEEzNFNLRUxCRjREOTRoLXJR0gGfAUFVX3lxTFBnQUE0ZEJtcV9KYXBNYXZzVXlQSjRaZzFfWlRKcUM5R2hHc0dYUkVnM25TSFQteExCc3FZODF1WFhNcGk0VExmcUx3M3BFejYtNENYUmpwYWtpQ2Q4Z0JJd3RUbUpqMFY5Tml5LU5vZUVMb0praTRCSFY5UmJDakFlcy1qMGxFU1FtbnRId3dxTnJJUllvWmdCM19kNGw1cw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPRGJmX0JoNWk0dFFBRGRrcXBleVZaUjVud1dPakQwcUt0X25QUTFEUVh4N0MzWDVTRUlJZ3NOaXF4cWNfZkktckFlRGRTRlRYRkNKOXJFSFI2VlRKUDRMOVpUWWM4b2NSa1NYM2VtX3FSdUVwZ1U1LVJDcVJTc0FoMjN3Ui1RWkg5MF92Q0FXLTRocDZMUWpfR1VIbVVmS01qWGYxblhFTm0?oc=5</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Fafen PR volta a produzir ureia: fertilizante na fábrica é comida na mesa! - FUP - Federação Única dos Petroleiros</t>
+          <t>Mercado de fertilizantes vive momento mais difícil em décadas, diz Mosaic - The AgriBiz</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPcmtibVp2QVZDY19yQXhVZC1ybWpjb0dqUXhGMlo5OFhodXpBczFOWThhLTc3RHBvdHNxVU9iSXZyQnVMdm8xUmtWbkNNcHRTWUYweXNpcTc3bUI5Ym56Z1pzckdTazllVFRzTzVrLUVJYm5ydDlkXy1mclNEdTlncWVFN0g5U1JfbnBoTmVzTTE1eHJCVDdF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNZXpsRmRrRjkycUpIaUJaY1V2cWxzelVBZnAtTm5ETEdJY1lQTUUtTHFVMkNBTkZyem9xVHUtS1cyaVpmSHdnc3doMTdFWkdGTThsbEJNU3dFSDVIRjZIaUlxODlHd2F1cUdJU3NuTGpQT01OMUN3MnhkR3o4S2gwd1dMMWR2QV81X2tOZ21PS2JIbU5STlAzT1hNV0wyczdVbHlLMGtFVFVpYXlHMnFyNk1UVmo?oc=5</t>
         </is>
       </c>
     </row>
@@ -7024,7 +7024,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Ansa retoma produção de ureia no Paraná após R$ 870 milhões de investimento - CNN Brasil</t>
+          <t>Petrobras inicia produção de ureia em unidade no Paraná - InfoMoney</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPRVZqOUg0Y2U1WWVlQm55NTlPcXdFMVFzM1BMdjJ5V3NRNDNsZ0dGb0JDVGU4LXlOSEJ5SUk2UXpOR0hhZ2pVTER2ZzBCREwwRWFaeWZ4ZkVweHQtbjhRNndfMUhCZnpDcnptcmNsYjBqelFOem5IZHB4UW5hcGQyRWdjUFpjNk1OT1BILTV0bk04VHBrSTJrTU1uLXFfYml6elA3OUVuUC1ya0QyRlBn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOR2lLUEZxMlhlTzhWUGp5WmZaaFA2RV80WkpYazZtVXd2ZldSM2ZzaFBHNnFNTFpIZ1JVLTdZWUxnMzJMOERZTHV6SXN4ZDJieFdqS05ZWFpvbVdMVXRqNmo4VWZ1OXpMZDl5bS14UjgtQ1RtVmRFZmZmZmg4cXhlLXptYjRjMzNPTEEzNFNLRUxCRjREOTRoLXJR0gGfAUFVX3lxTFBnQUE0ZEJtcV9KYXBNYXZzVXlQSjRaZzFfWlRKcUM5R2hHc0dYUkVnM25TSFQteExCc3FZODF1WFhNcGk0VExmcUx3M3BFejYtNENYUmpwYWtpQ2Q4Z0JJd3RUbUpqMFY5Tml5LU5vZUVMb0praTRCSFY5UmJDakFlcy1qMGxFU1FtbnRId3dxTnJJUllvWmdCM19kNGw1cw?oc=5</t>
         </is>
       </c>
     </row>
@@ -7046,7 +7046,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Em meio à crise dos fertilizantes, Petrobras volta a produzir ureia no Paraná após seis anos - VEJA</t>
+          <t>Petrobras inicia produção de ureia na Ansa, unidade que estava hibernada desde 2020 - Valor Econômico</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNU2E5eUdWYzFxMHoxdzFrdktxNndmLXhpOC1mY0kwcUVPdWpoVnVkZVgxRXZQY1N2UFJNRmozQ0p5UVlWREZKaGFLMWR6WUU0UmxSTG5xaE1lSWJ1QjdaOWhMQVNUY29Lams4WnE3bS1Tb3JhaUR6MDJSbWtkUU9ZOGlvSS1IOHFWSGJjY01PYTBkN1d0UE5xWHZTTDFmUEpiUTEwN1BQWWNpZnRXRjBxLXR4MktvUWJOMzRfVVl5TWNwRENEUnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNcVNQNzR3X3ZiZC1IbXR0Q1U5M3d4TXVWcTNMRU1GOGhOd0pKYkpXeUpnS2VkcHJieWpNVDhUdnpDeFlud29jWEFSZ2Z1MjJIVE90QmpIc2NSbkxlbG5iQW1xeVZsU1hiS0RrR2hDTDVmU3duTFpBTGRjbGRtLWdjWkF1cnFtVU1YRkN4VTNOU1JLZm5hakh0RWFsblV2SlNhT1d2djhINGN4MTlSX0xfZXBncFRmbUVVdlppWFlhSXF5T2xuMnFiNWlla1VkcFVPWi02WVNkONIB5gFBVV95cUxORWpyQ285M1U3ekpPWWVwMER6dTNMTWlZZ3h3VFBwSmRiZ1Y0dnZvb0NtaVlXR0FSank5ZklXMkl6NUhFcG1wcWFuX3lld0VSeFktQU1PUUxESFg5VE0zRlBPaVNfb1VFZTE3ZUFsRDB4N1ZYVUo1dXMxN210RW84LU5scWp4MXppTEZLWFlEeC1mdE9hYkhOTmNoaVUzOFA2d3lvVkZ1cWxCM1A5YWxMUW0tamkxS3BqSUNxRUlWcFo1cUZ2bFVtdlIyd2xKM2FjQTBkcmJjVWdtSlI4WFNlRkxHZlBQdw?oc=5</t>
         </is>
       </c>
     </row>
@@ -7068,7 +7068,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Petrobras inicia produção de ureia em usina desativada há 6 anos - Poder360</t>
+          <t>Ansa retoma produção de ureia no Paraná após R$ 870 milhões de investimento - CNN Brasil</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7078,19 +7078,19 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPRGJmX0JoNWk0dFFBRGRrcXBleVZaUjVud1dPakQwcUt0X25QUTFEUVh4N0MzWDVTRUlJZ3NOaXF4cWNfZkktckFlRGRTRlRYRkNKOXJFSFI2VlRKUDRMOVpUWWM4b2NSa1NYM2VtX3FSdUVwZ1U1LVJDcVJTc0FoMjN3Ui1RWkg5MF92Q0FXLTRocDZMUWpfR1VIbVVmS01qWGYxblhFTm0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPRVZqOUg0Y2U1WWVlQm55NTlPcXdFMVFzM1BMdjJ5V3NRNDNsZ0dGb0JDVGU4LXlOSEJ5SUk2UXpOR0hhZ2pVTER2ZzBCREwwRWFaeWZ4ZkVweHQtbjhRNndfMUhCZnpDcnptcmNsYjBqelFOem5IZHB4UW5hcGQyRWdjUFpjNk1OT1BILTV0bk04VHBrSTJrTU1uLXFfYml6elA3OUVuUC1ya0QyRlBn?oc=5</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Mercado de enxofre corto de compressão varre através da cadeia de suprimentos - Sunsirs</t>
+          <t>CMOC assegura projeto Cangrejos por US$1,7bi no Equador - BNamericas</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFBQbnRCaEVzdkRzQ0tXZHFVZWd1cmFPVlJxcDc5VDY4bnRxaUx2YmRBdXdLOW9TaEhfWTk1Vmp2SldCZktYcmRfNzRaLVozOE9pZ3p4NEZEdTZXNmk1a2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPUDFMYWdTWDQ3ZGljdUF2VDY3UkRwLS1xNXBxLWZQVEpEMG5nU1dvTjdqZ0lyZ2JFRC0xelhXR2FINldleXlJWUJDOTBwU0NEQm14LWlqNVFOcWVPc1Q4a0tXWTNQYTFkZThzUkE4MElVeXBXOVdqaXZUNTJyQlpIMFhzX0xXclg4QWtqR1kxOVZES1NyVWc?oc=5</t>
         </is>
       </c>
     </row>
@@ -7112,7 +7112,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>CMOC assegura projeto Cangrejos por US$1,7bi no Equador - BNamericas</t>
+          <t>Unidade da CMOC assina acordo de US$ 1,7 bilhão para desenvolver mina de ouro e cobre no Equador - Valor Econômico</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -7122,19 +7122,19 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPUDFMYWdTWDQ3ZGljdUF2VDY3UkRwLS1xNXBxLWZQVEpEMG5nU1dvTjdqZ0lyZ2JFRC0xelhXR2FINldleXlJWUJDOTBwU0NEQm14LWlqNVFOcWVPc1Q4a0tXWTNQYTFkZThzUkE4MElVeXBXOVdqaXZUNTJyQlpIMFhzX0xXclg4QWtqR1kxOVZES1NyVWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQWXI3c2c1Nkg5UTVTWkJ2QTVPNEd1Tmt0aUowbms1aFFrbEt3VTdtYTlQYWpNS0RiNVR1NU45ZWR6enpSdDhSbHZVNDNsSUdjSHJxbmxSUWt3U1NieGMtYTU0RDRtWXV2eUowSzdyem9UNUFfcHQwbXRqc2FldjZacDl0MVhFYmdJek9IWVZKWlRLbEoxUS1aTmVFdERsNHhhY180MzhhcERmWlhZZzc5VkhoSENab3JFUXM5V1pJUnZ6MVVWeVprbkpCUzQtTXIzRGtfd01rRWtQXzZFQUVKZXdSONIB8gFBVV95cUxOcEN2M0tCSFEtSVA4Y0ZtQV9EOWlFUERlR3JFb2RzZHFZVjVQWTZyUk9DZC1tTFpFcU8zeGNMR2pBRzl3ZDVKRElVa0RTTmxxZnNSWFJTNHVxX3c1b3FBX3JSLVhKcVdQY05BT1hRQ0ZibWJBWWttX2hDUjFFRk1TRTNBRV9DbGRSZHZkNlFIMkwtSlJNMkpoNTNGcVQ1ZVBSSDJpeW81eGRIT3B1aHM4alhLVkJPREk5cnFBdjdSSzZkMk9tVU1Oa3Fyd3ZrZWJKTXY5bDhFaWxfT3djU2FSdVpjclBXWHdLUml1MG5Ic2xHQQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Unidade da CMOC assina acordo de US$ 1,7 bilhão para desenvolver mina de ouro e cobre no Equador - Valor Econômico</t>
+          <t>Mercado de enxofre corto de compressão varre através da cadeia de suprimentos - Sunsirs</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7144,19 +7144,19 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQWXI3c2c1Nkg5UTVTWkJ2QTVPNEd1Tmt0aUowbms1aFFrbEt3VTdtYTlQYWpNS0RiNVR1NU45ZWR6enpSdDhSbHZVNDNsSUdjSHJxbmxSUWt3U1NieGMtYTU0RDRtWXV2eUowSzdyem9UNUFfcHQwbXRqc2FldjZacDl0MVhFYmdJek9IWVZKWlRLbEoxUS1aTmVFdERsNHhhY180MzhhcERmWlhZZzc5VkhoSENab3JFUXM5V1pJUnZ6MVVWeVprbkpCUzQtTXIzRGtfd01rRWtQXzZFQUVKZXdSONIB8gFBVV95cUxOcEN2M0tCSFEtSVA4Y0ZtQV9EOWlFUERlR3JFb2RzZHFZVjVQWTZyUk9DZC1tTFpFcU8zeGNMR2pBRzl3ZDVKRElVa0RTTmxxZnNSWFJTNHVxX3c1b3FBX3JSLVhKcVdQY05BT1hRQ0ZibWJBWWttX2hDUjFFRk1TRTNBRV9DbGRSZHZkNlFIMkwtSlJNMkpoNTNGcVQ1ZVBSSDJpeW81eGRIT3B1aHM4alhLVkJPREk5cnFBdjdSSzZkMk9tVU1Oa3Fyd3ZrZWJKTXY5bDhFaWxfT3djU2FSdVpjclBXWHdLUml1MG5Ic2xHQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFBQbnRCaEVzdkRzQ0tXZHFVZWd1cmFPVlJxcDc5VDY4bnRxaUx2YmRBdXdLOW9TaEhfWTk1Vmp2SldCZktYcmRfNzRaLVozOE9pZ3p4NEZEdTZXNmk1a2c?oc=5</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Uma nova Mosaic, com menos ativos, mais bioinsumos e “sem plano de deixar o Brasil” - AgFeed</t>
+          <t>Copa do Calcário: Macuco lidera e disputa segue acirrada após nova rodada - Serra News</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -7166,7 +7166,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQOGk5c2lwZUhVRXBjb2VSNW5xU283VzdIRl9JTDU0RFk5bEZGM0ZxVEJaaWJERkp3TUtNY0FxX1NpTUlGSWxYTzl5RVRxcEdid0NNaEhDS3RXTjQzQkp0ZjFlNGhsUHd4V1ZjaVBXZWFTMS1qMjctLXZGcU9xeVdMTGJMMzZDQkVOUlA3TU0yNl9hSDFyejloZHRXT0lfRUtlN0g2S1JGQjdSRlFaOXkycA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVzdyNUh6M1JxbnZwVjlaS0Z0Ui05cjJWMkg0bDlOWmNSeUFJYlNMMDFJT1VXSDMxbVlfWk1UYWJqSGNpOXVXQkRfMnBXN2FycUxjbF9HbGczY0x3MmdQekEyWEZNV3RkWFFkTlMxb3h4TmRvb2VDQU1STVd3aEtxbE9uZ0ZNT25lNzVVa1FDSWdWQXpGZjA3aTNaS2YyTjBI?oc=5</t>
         </is>
       </c>
     </row>
@@ -7178,7 +7178,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Copa do Calcário: Macuco lidera e disputa segue acirrada após nova rodada - Serra News</t>
+          <t>Macuco vence novamente e segue na liderança da Copa do Calcário - FERJ</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVzdyNUh6M1JxbnZwVjlaS0Z0Ui05cjJWMkg0bDlOWmNSeUFJYlNMMDFJT1VXSDMxbVlfWk1UYWJqSGNpOXVXQkRfMnBXN2FycUxjbF9HbGczY0x3MmdQekEyWEZNV3RkWFFkTlMxb3h4TmRvb2VDQU1STVd3aEtxbE9uZ0ZNT25lNzVVa1FDSWdWQXpGZjA3aTNaS2YyTjBI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNVTgySERJNzFBLVRJY0tDRV81b19aVkctQ0lXdzZrRmVHdUtISTRwbUloajBPNFdXNHZsdDVpU2RDNFE5V2hjU2VfZWIxT1V4Njc5TjJFLTNHejc3ZGNfbzJWVzI4SnZDR1ZISy1XQklsWGIxUHlCSWFPX09jUUVEeERud0tSNGZlQm9rLXNGQlJUb0NEdnR2aA?oc=5</t>
         </is>
       </c>
     </row>
@@ -7217,12 +7217,12 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Macuco vence novamente e segue na liderança da Copa do Calcário - FERJ</t>
+          <t>Uma nova Mosaic, com menos ativos, mais bioinsumos e “sem plano de deixar o Brasil” - AgFeed</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -7232,7 +7232,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNVTgySERJNzFBLVRJY0tDRV81b19aVkctQ0lXdzZrRmVHdUtISTRwbUloajBPNFdXNHZsdDVpU2RDNFE5V2hjU2VfZWIxT1V4Njc5TjJFLTNHejc3ZGNfbzJWVzI4SnZDR1ZISy1XQklsWGIxUHlCSWFPX09jUUVEeERud0tSNGZlQm9rLXNGQlJUb0NEdnR2aA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQOGk5c2lwZUhVRXBjb2VSNW5xU283VzdIRl9JTDU0RFk5bEZGM0ZxVEJaaWJERkp3TUtNY0FxX1NpTUlGSWxYTzl5RVRxcEdid0NNaEhDS3RXTjQzQkp0ZjFlNGhsUHd4V1ZjaVBXZWFTMS1qMjctLXZGcU9xeVdMTGJMMzZDQkVOUlA3TU0yNl9hSDFyejloZHRXT0lfRUtlN0g2S1JGQjdSRlFaOXkycA?oc=5</t>
         </is>
       </c>
     </row>
@@ -7283,12 +7283,12 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Guerra no Oriente Médio faz ureia disparar e segue pressionando preços dos fertilizantes - Canal Rural</t>
+          <t>Vem aí mais uma aquisição no setor de terras raras no Brasil - O GLOBO</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -7298,19 +7298,19 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOV0xwZE9OSUFnQ0FXRzZvZlBXamZsaHRVT3Z2T1l3YlhUb2dmTnIxanhJdU9YOW1NMWFFQmlQWTlPc280cnRTRjZJVXpDWWZGUmlMaW5jbWd6OXE2VHFTZEs3UXp3cVFEOEphZWZXRVR0NlVHT3BGbHBQN3V0UVIyYmt4bURHdVJCcDJ1d2tJUzFKVzVQdDY1eHQ5ajFPQ2MtZzhwdlNGanozQjAyVVRpMk0wd0xJSmxCRGxHZmFqbTBjUEt2V1J5UG9fTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOR1otWkdBQnhyYm10RnhmcW9jVEZlNGtDMWdkMTZVbFRTbTVCRWxYNkVWeWdnc0FwTEFOLTZPMGI5ZFo3bjkxdUgwdk04NF91blVDMk95S1BMWkg1ME1aTF9wOThmSFA1Z0hqYUl5X0ZVNS1nMHVEejhHS1FNdl8yT1FmNWhyR2JrTlFncThDNTJlOXpHUERqNklYT2RVYW5ReC1nZFh2dnAwNDd2SFdxMTZTOS15U2N3ZkpVM09CWHbSAc8BQVVfeXFMT0xXcVV6WXVXbmo3NUhJMjFyVnBLTUdubUtWMVIxNFhpUEhhMDZ6dUNkelZ5WjZWb3U3b2g0WHdXX2dJTjhYdWN0WjhkS29ZTXdHaEZQLThyLXFuakhPUXVMdUhZc01NOFhNZHFNcDRyclZENndiNnl2OXVoOG83RTFaMG1KaEVKenBhTzdLQ0FXelNvbG5aZ3NmVlRyd1V3cUg0Zm5lZHFHY2gxX0EtdG9vVER3ekN2SEJraXRLekEtRWhrbEFZZndLOGRFVU84?oc=5</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Vem aí mais uma aquisição no setor de terras raras no Brasil - O GLOBO</t>
+          <t>Guerra no Oriente Médio faz ureia disparar e segue pressionando preços dos fertilizantes - Canal Rural</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOR1otWkdBQnhyYm10RnhmcW9jVEZlNGtDMWdkMTZVbFRTbTVCRWxYNkVWeWdnc0FwTEFOLTZPMGI5ZFo3bjkxdUgwdk04NF91blVDMk95S1BMWkg1ME1aTF9wOThmSFA1Z0hqYUl5X0ZVNS1nMHVEejhHS1FNdl8yT1FmNWhyR2JrTlFncThDNTJlOXpHUERqNklYT2RVYW5ReC1nZFh2dnAwNDd2SFdxMTZTOS15U2N3ZkpVM09CWHbSAc8BQVVfeXFMT0xXcVV6WXVXbmo3NUhJMjFyVnBLTUdubUtWMVIxNFhpUEhhMDZ6dUNkelZ5WjZWb3U3b2g0WHdXX2dJTjhYdWN0WjhkS29ZTXdHaEZQLThyLXFuakhPUXVMdUhZc01NOFhNZHFNcDRyclZENndiNnl2OXVoOG83RTFaMG1KaEVKenBhTzdLQ0FXelNvbG5aZ3NmVlRyd1V3cUg0Zm5lZHFHY2gxX0EtdG9vVER3ekN2SEJraXRLekEtRWhrbEFZZndLOGRFVU84?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOV0xwZE9OSUFnQ0FXRzZvZlBXamZsaHRVT3Z2T1l3YlhUb2dmTnIxanhJdU9YOW1NMWFFQmlQWTlPc280cnRTRjZJVXpDWWZGUmlMaW5jbWd6OXE2VHFTZEs3UXp3cVFEOEphZWZXRVR0NlVHT3BGbHBQN3V0UVIyYmt4bURHdVJCcDJ1d2tJUzFKVzVQdDY1eHQ5ajFPQ2MtZzhwdlNGanozQjAyVVRpMk0wd0xJSmxCRGxHZmFqbTBjUEt2V1J5UG9fTQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -7503,12 +7503,12 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Alta histórica do enxofre eleva custos e pressiona cadeia de fertilizantes em 2026 - RADAR DIGITAL BRASÍLIA</t>
+          <t>Copa do Calcário começa com grandes jogos e celebração dos 24 anos da Liga de Macuco - FERJ</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -7518,19 +7518,19 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQaFZWeGVvRU9TMG5XZlBvZ3JiRGU0UlpKS1lucmlueW9ncG0wZnVFOFVjRWFJRVRiVm1Ua3A4UVhQdU9hcXdGQWljSmhmcjRyeTlZY2FVR2xWOENBZzd6THRnZVJVMGlmd1R0Y3o1aFM5WWlWMXpieHpBQ1FucDkwLS1MZ0VRRnJ4aG5YWk85dDNjNkplb0xkbTU2cFVzMDc3bFRydktaMFI3X3FWRHpMS3g3Y1VrMmJSR2Nwdk1MU3plaUxGU3dUd0p2QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQS3Nfenl1TmpwNXFzTDhyTXJOM1JLeHlmRENybjZrWUpqak9GbTR0TDZ4dDJuQmw0eUhVWC1TVE43SHg5RWNUbTlFUDhWX0xJYldYZTZPUkNaMHoyS3lwVW1fSGZtbmFhSlNGU2xVZTdrNDg5MXVXeHpNQ1RnalI1ZWhlbkRySVZTcVdjMGtEMVFOdTJsU0t0TERPcnROOFkyWFVERDVTWVFFMUU0Ty02SndibEE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Copa do Calcário começa com grandes jogos e celebração dos 24 anos da Liga de Macuco - FERJ</t>
+          <t>Alta histórica do enxofre eleva custos e pressiona cadeia de fertilizantes em 2026 - RADAR DIGITAL BRASÍLIA</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -7540,7 +7540,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQS3Nfenl1TmpwNXFzTDhyTXJOM1JLeHlmRENybjZrWUpqak9GbTR0TDZ4dDJuQmw0eUhVWC1TVE43SHg5RWNUbTlFUDhWX0xJYldYZTZPUkNaMHoyS3lwVW1fSGZtbmFhSlNGU2xVZTdrNDg5MXVXeHpNQ1RnalI1ZWhlbkRySVZTcVdjMGtEMVFOdTJsU0t0TERPcnROOFkyWFVERDVTWVFFMUU0Ty02SndibEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQaFZWeGVvRU9TMG5XZlBvZ3JiRGU0UlpKS1lucmlueW9ncG0wZnVFOFVjRWFJRVRiVm1Ua3A4UVhQdU9hcXdGQWljSmhmcjRyeTlZY2FVR2xWOENBZzd6THRnZVJVMGlmd1R0Y3o1aFM5WWlWMXpieHpBQ1FucDkwLS1MZ0VRRnJ4aG5YWk85dDNjNkplb0xkbTU2cFVzMDc3bFRydktaMFI3X3FWRHpMS3g3Y1VrMmJSR2Nwdk1MU3plaUxGU3dUd0p2QQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -7569,12 +7569,12 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Queda da ureia acompanha alívio geopolítico - Agrolink</t>
+          <t>St George tem interesse em comprar ativos da Mosaic em Araxá, dizem fontes - CNN Brasil</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -7584,7 +7584,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQNEppb0R2TFlCUmIzRW0xckJYSWVvQUJ5cTc3MldveFBqTVZtbU95MFVfNVJLYVR1SUhVM1BFTXd1OHZhVzVoVkQtczA4NXVwLTc0VUdpY0RjN002TXk1aDlnM0w5U1ZvWUUySHREcG9LZUZfdFl2QmxubUpnbEJWdUE3UGZZNXRrNmFOWUFwVDUtRkJsVTBn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxONlhxcHQzelN2ZlNmOEhFbzI1SFN0TXdwbFNLbHk3Zl9WSEg3c3RTZFhvVWpBUWt1TnBoYjR5TG1SUDlRakNZRy1CcktIaFpyTWJicEdpdlN1dDVCUHJrR2JpLTJhbjFzTWE1RzYzUDc1VGo2ZDI0MHMtMDlaUXhVNUdLZmZxTWFsYW1ERm94bEVkNlZiRm15UjhLZUJlcjFaV1lqcW1JeGRmZmVjelE?oc=5</t>
         </is>
       </c>
     </row>
@@ -7613,12 +7613,12 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>St George tem interesse em comprar ativos da Mosaic em Araxá, dizem fontes - CNN Brasil</t>
+          <t>Queda da ureia acompanha alívio geopolítico - Agrolink</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -7628,19 +7628,19 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxONlhxcHQzelN2ZlNmOEhFbzI1SFN0TXdwbFNLbHk3Zl9WSEg3c3RTZFhvVWpBUWt1TnBoYjR5TG1SUDlRakNZRy1CcktIaFpyTWJicEdpdlN1dDVCUHJrR2JpLTJhbjFzTWE1RzYzUDc1VGo2ZDI0MHMtMDlaUXhVNUdLZmZxTWFsYW1ERm94bEVkNlZiRm15UjhLZUJlcjFaV1lqcW1JeGRmZmVjelE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQNEppb0R2TFlCUmIzRW0xckJYSWVvQUJ5cTc3MldveFBqTVZtbU95MFVfNVJLYVR1SUhVM1BFTXd1OHZhVzVoVkQtczA4NXVwLTc0VUdpY0RjN002TXk1aDlnM0w5U1ZvWUUySHREcG9LZUZfdFl2QmxubUpnbEJWdUE3UGZZNXRrNmFOWUFwVDUtRkJsVTBn?oc=5</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>INSCRIÇÃO NO PROGRAMA DE CALCÁRIO ATÉ O FINAL DO MÊS - Prefeitura de Mato Leitão</t>
+          <t>Mosaic anuncia paralisação em Araxá e Patrocínio com corte de funcionários e queda de 1 milhão de toneladas na produção de fosfato - G1</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -7650,19 +7650,19 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPQ2xHNUVCT202aDlGai1PVTBaS0tmbFAyaDVCYThDdVpQdTFhcWlzTGtDWThuWkhVRU5zTDdwOF9ENUlSd2k2TUNuUktNU3Y1WXpMck1qMkVCeHprRVpUZE9KSUNMQ3lfaWRSMkVwS2hEbXVFTDNmZndjZkh1ek9VQU43VV9SR09aUHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowJBVV95cUxPYVNQbkdxNThhSW1ydHJLMUlzcjQ1eE1vbFMyZVZiSVkzVE1KbC1lcEVYZnZnV3lLNW1wWG03VzJ4OWdQTTBBRDlDUzI4NXlmYlhmM0l6MjhJY2Z6Z2tLbjFHVHc1dW9aTlA5OEd3aEFaN2Y0MXlIdDNEM1BCQ3NqS1ZidzMtc2VSUWhBWVk0cUJIY2V4VWRsQnQyM1lPTmMyTEhFZmZ6ekNpQnFhM3FMRi1adFJpMmhjQWNVVWNZUFMyNnplbEgwOTZUZXg4d2hFYW9TUUJacldTbzR3QlVjRHpIYkFZZmJJRUJVdmRzdmtwbjE1VXdtRVd5OWlCOTZVZ1JidjgtQmdoOVYzdlZ0QWZqUVVYZDU5dU1rU3FaSjNvcWPSAbICQVVfeXFMT0NZVFdGbHgwUkYwU2xxM3RTWVd1YS1UdkVlc1VfS3pURUU5OTQ0NzVmekVFb01UUjVkbkVrVWJXaWZ5SUtNQTlfQWx2NWJ3emd3bXR4WkFEUmg0Z3hqa0RnLWk1YUVmZmNTLWpyQmhKSXVGM2pEbURiaDNHa1BDa3RvNGtoX3ItM2p3UEVoVXdHSjg2T0MxZExiVTk1RFlJaENuQU5hMnpabFZ3YTZ1SHZ2OVRjV2h4amRpVVBhYXBPZWVld1BkWVVLVThVVDBRSy11YWNWT01RV01MSXJYNS1aV29YUHZVZl9oazhEajBad1FkSmdKS01FcVlvYmxRcUtSVVR6am1qYU9UZHl4Y3o5ZlE3THNDb0lOMFIxVXJBOUF2TGVrSUJzeUlyMUFpczR3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Mosaic paralisa operações em Minas Gerais e reduz produção de fertilizantes - Canal Rural</t>
+          <t>INSCRIÇÃO NO PROGRAMA DE CALCÁRIO ATÉ O FINAL DO MÊS - Prefeitura de Mato Leitão</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -7672,7 +7672,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPNnVZeUNJdHBJOThrQTk2UW9EeXBQcFowX2p1TnlzS0I1Zmc4RGhkMkZIVXJTbUdsYUJKUGx0Y0ctTlAxUU1zcGNGU2ZxNWppSFRsaHU3aU9nNS0xZ093bkV3UlB3NzlVaXVDYTBCeXRJSmVoNUlSaktHRHhDbWF3dFdqSlpKOW9BU1pncGVBM3htRUVDbTZJVWo2S2VuQW1jWk1RZGlOdlpZM0RKZVFFMGVrSnBzQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPQ2xHNUVCT202aDlGai1PVTBaS0tmbFAyaDVCYThDdVpQdTFhcWlzTGtDWThuWkhVRU5zTDdwOF9ENUlSd2k2TUNuUktNU3Y1WXpMck1qMkVCeHprRVpUZE9KSUNMQ3lfaWRSMkVwS2hEbXVFTDNmZndjZkh1ek9VQU43VV9SR09aUHc?oc=5</t>
         </is>
       </c>
     </row>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Mosaic anuncia paralisação em Araxá e Patrocínio com corte de funcionários e queda de 1 milhão de toneladas na produção de fosfato - G1</t>
+          <t>Mosaic paralisa operações em Minas Gerais e reduz produção de fertilizantes - Canal Rural</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowJBVV95cUxPYVNQbkdxNThhSW1ydHJLMUlzcjQ1eE1vbFMyZVZiSVkzVE1KbC1lcEVYZnZnV3lLNW1wWG03VzJ4OWdQTTBBRDlDUzI4NXlmYlhmM0l6MjhJY2Z6Z2tLbjFHVHc1dW9aTlA5OEd3aEFaN2Y0MXlIdDNEM1BCQ3NqS1ZidzMtc2VSUWhBWVk0cUJIY2V4VWRsQnQyM1lPTmMyTEhFZmZ6ekNpQnFhM3FMRi1adFJpMmhjQWNVVWNZUFMyNnplbEgwOTZUZXg4d2hFYW9TUUJacldTbzR3QlVjRHpIYkFZZmJJRUJVdmRzdmtwbjE1VXdtRVd5OWlCOTZVZ1JidjgtQmdoOVYzdlZ0QWZqUVVYZDU5dU1rU3FaSjNvcWPSAbICQVVfeXFMT0NZVFdGbHgwUkYwU2xxM3RTWVd1YS1UdkVlc1VfS3pURUU5OTQ0NzVmekVFb01UUjVkbkVrVWJXaWZ5SUtNQTlfQWx2NWJ3emd3bXR4WkFEUmg0Z3hqa0RnLWk1YUVmZmNTLWpyQmhKSXVGM2pEbURiaDNHa1BDa3RvNGtoX3ItM2p3UEVoVXdHSjg2T0MxZExiVTk1RFlJaENuQU5hMnpabFZ3YTZ1SHZ2OVRjV2h4amRpVVBhYXBPZWVld1BkWVVLVThVVDBRSy11YWNWT01RV01MSXJYNS1aV29YUHZVZl9oazhEajBad1FkSmdKS01FcVlvYmxRcUtSVVR6am1qYU9UZHl4Y3o5ZlE3THNDb0lOMFIxVXJBOUF2TGVrSUJzeUlyMUFpczR3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPNnVZeUNJdHBJOThrQTk2UW9EeXBQcFowX2p1TnlzS0I1Zmc4RGhkMkZIVXJTbUdsYUJKUGx0Y0ctTlAxUU1zcGNGU2ZxNWppSFRsaHU3aU9nNS0xZ093bkV3UlB3NzlVaXVDYTBCeXRJSmVoNUlSaktHRHhDbWF3dFdqSlpKOW9BU1pncGVBM3htRUVDbTZJVWo2S2VuQW1jWk1RZGlOdlpZM0RKZVFFMGVrSnBzQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Mosaic vai paralisar operações de fosfato no Brasil - Notícias Agrícolas</t>
+          <t>Mosaic, fabricante de fertilizantes, vai paralisar produção de 1 milhão de toneladas de fosfato em meio à alta dos preços - InvestNews - InvestNews</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPbVRRUEJ0RXAyUWZwY1VnWXhDNTB2emJUa2VFVU5YYTZJaHJYSGlIODNkbExvel9VRldvU2JWbmdkTmZkZ196Z0hnUHpENFV5RExqSVNwTHByMlZwZUEyT3NLMW8wUl9KTFNiTFctNHozd2MzM2wtY2tTSElvRFhlQmtBdTgtV0trS1pjTWFnaFdwby1uanJ2MVMwcXltb2wwbXhOWUtYdWJuNXhLZ0dhYU81eWZ2UEYxQ19CeGV30gHDAUFVX3lxTE9GaWdoUGlIQVFfTWJGMlZTZ1JvLWZOc0JuTXJtekhTazJwc0lnam0yMVNFdGgzRGpoNks5VWNSLUtwN252d1FEcGwxMEJ5M1JjZTJGeDFwVUZNMThLVTd2cFVCRG4wUFBUNUtYWkZGV0lFdzVnQzIyZEZ2RWdSelRHUGxBYTJLZlJuWWI3eHc2NmhIUmVKYnNKZm05bHFkQ2RST0dTOENEblYtZDdaX204azg5V1BPdE9sMXBNZlhpUU0tQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxOMlE2aTNkQ1drWHNGNjhJckFIY3hkM1A2S3lfdkhJbXBtaDN5VmV4NHVPNFdra1FTXzV2ZUprdGNsaDZxa21sWmk2dlpabDJ3aUpROUE3YVdFd0VEZDdscnd0RjAzS3huS1N1Ujh0b01DVld0OUpWUDV4c091SW1kcjBDNFRHZDl0ZTdIMFBlTHRuRnZYenNneG4yUHFLa1BnZEhmY1ZhenhwSTJpb0NFdXE3dDBGVlI3aERwQ0NHWWk0d0JBdS04dFZzbHNySXZNcFp2YlJGNjVCNnZ3YUZtdW55MHhQa29QVnhn0gHwAUFVX3lxTE9IakdwRXpVeExMWDhnSkZFci1UWFRqLTZscWVWcS11Q3lSMmdnX2V4Mm1IUmw5WEF6MURadm1KdEdlLWxMWjlIa3lBNXVJYjVrSzdBTHA4QUFTblNrSV9uRDdLR2g0R3lrUTBSV2hEMi1IVHdHeUxFdVZCNU9xbTktc0xHWUVnLWliZThlUnplY3pGbDBnaXdPTFpicFZ1NEo4RGdjbVlEUW5HSDlIb2U3RUZQLTRlOVBWZVZQZDU3WDR3YkJZbmJ5WHBXa0RZZXIzc3hpbU5OSFo2cWF6M05iZHJUVzl1VWhaRnZUblhWVw?oc=5</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Mosaic põe ativos de Araxá à venda e paralisa minas de fosfato em Minas Gerais - The AgriBiz</t>
+          <t>Mosaic suspende operações em MG e mira corte de até US$ 80 milhões por ano - Exame</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOVFJXZkVVUUlxUFdTUTY3LURqTi1Xb2ZpY0FMZHJNZjRuSzdyWEFmMEFJYWJHeWxibjhIZGF6MWZEbHMzYzRmU1Z6eVB4WmY5YjlDVDd0bU1RNTRBdXFOQjJYRGQ1SVlFd0xLZ2hyYlExMHBOU3dYLUlJY1U1b2JRYzR6bmFFQ21LNl9peDNCT2JWUl9PTUlTcE9TX09PQm5ZWjhxY2VTX0JmbXRodjg4cXgxSDhYUGVGU0dqZA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNdEZqNHdRb0pLX2tyVWRjNVk0SmdMUEdIdjVMbGFOb25QLXdaNXFBU0w5a1REbXFUcjFKV2lYSUNYTk9UQXV1Q1hHeVozUDdCdWhvXzlhQ0lLM1dYZUZyaDBhNXNmV0xmWHJBMFVqV3BwUkxEY2s5N0FTMkE5ZW9tRG9qbW44WUVyNWF4ZXhqaURvWEFvOXhtV2EzZnJEZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Mosaic planeja venda de ativos e paralisa operações após impacto do enxofre - CNN Brasil</t>
+          <t>Mosaic vai paralisar operações de fosfato no Brasil - Notícias Agrícolas</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -7804,7 +7804,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNWjZGTlNiamVJY2FzNVQzeG1ScDYyZ2JadVBQOW00WFpNYVNVWG9aVXNXS3p1b1lXMFZVVHNHNktHLVZmUS1teWlzWVhwVVJXV091eE91V3BiZ3E0emdVTzA1NW5LZlVxRnhKb0tmcE9kLU5ZaGhxdlZ2QjdMcXEzZXRWN1paZGhxYzNxa3d4ajZwSDkwR0Fvc3ZHYmgtandQbTF5eU95MFZEMEVjb0U0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPbVRRUEJ0RXAyUWZwY1VnWXhDNTB2emJUa2VFVU5YYTZJaHJYSGlIODNkbExvel9VRldvU2JWbmdkTmZkZ196Z0hnUHpENFV5RExqSVNwTHByMlZwZUEyT3NLMW8wUl9KTFNiTFctNHozd2MzM2wtY2tTSElvRFhlQmtBdTgtV0trS1pjTWFnaFdwby1uanJ2MVMwcXltb2wwbXhOWUtYdWJuNXhLZ0dhYU81eWZ2UEYxQ19CeGV30gHDAUFVX3lxTE9GaWdoUGlIQVFfTWJGMlZTZ1JvLWZOc0JuTXJtekhTazJwc0lnam0yMVNFdGgzRGpoNks5VWNSLUtwN252d1FEcGwxMEJ5M1JjZTJGeDFwVUZNMThLVTd2cFVCRG4wUFBUNUtYWkZGV0lFdzVnQzIyZEZ2RWdSelRHUGxBYTJLZlJuWWI3eHc2NmhIUmVKYnNKZm05bHFkQ2RST0dTOENEblYtZDdaX204azg5V1BPdE9sMXBNZlhpUU0tQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>FERTILIZANTES | Mosaic anuncia paralisação das instalações de Araxá e Patrocínio e busca vender ativos de Araxá - Brasil Mineral</t>
+          <t>Mosaic suspende operações no Brasil e reduz produção em 1 milhão de toneladas - Investing.com Brasil - Finanças, Câmbio e Investimentos</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -7826,7 +7826,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPNVM2Q3ktX2tVc29Wb3RHZGdacTN1TXFhS0xET1k1YmVVWXY2MUI4NVNIUUJENUl6M1ZDM1lIQzNBUi1zYmVYcWJvM3JxSHJLSU13R3NCNG0yS0NfRUpWaGVSRV8wUUt4M2taUGdzX01qUHA3dFpPQ1QzSFpnLTU1TC1oZXBzQVAtcXl3cHhKZ25aNG9FbGt5TVdsNlRqOG1EVmxqNS1vSHZUNVFPWjJZcVZJT01KeGIza3FYYzUtWllscFVtSnlmMkVBMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOb1pWNXlKY05IeUlLM2M5NUFqWmYtWEgzYWR3UFh4Y2tISnlBZ0JWVnVfMF9POEFOM1k2dXZ2X0k0Z3FpVzYyNUsyRlJCTEs1Mmw0cGhibGdaTXNrMXMxWTA4VmwwSC00TkREbEJQTk5kekdxc3FFQkN1YmxrT1UxOHhyc2YxZFgtUWNLRXdmdi14SlZZY29CUzBxOE4xY3J5Nm41aDBrYVRQS2JyQUZfaDl2T2d3eXZRd1RUSE8xdUtzT3pQOXdDTmFtc2ZyQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Mosaic paralisa operação de fosfatados em MG e põe à venda ativos - Globo Rural</t>
+          <t>Mosaic põe ativos de Araxá à venda e paralisa minas de fosfato em Minas Gerais - The AgriBiz</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -7848,7 +7848,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNZmtnalFlYUVpZzc1V1FCQWVZR3d1dUR2SkJCeG43bi0teDJkVUZiclItMWp4YWxUd2tyaElmLUlEMzVnNnZsUmFhYzRLcVExdndfMml0SWJqV0plN19ZeGVwbC1JRWJuNjBmZUtXUm1ZTHhxRm5TNUJDN08tOHVGYWtBZjRZRHFJblBVeDhiT2J1UFJtS1ItcVZ2SWQzWmxHWmFYNjlqX0hfa3F4eC1SS2lfR1hNRFBMdWZV0gHKAUFVX3lxTE9xRW5TWVBCc3J3OE9JbGx1NTNnUHJlMVZXek42RDlWeTFHa2R2SXFiY3dwTkNldGZFUlhXS0xzMWdfVjRIVTdhMWdwMGQweHdCdi1Jckx5b2pQVEtZTkc4XzNpellPMEx6N2hOWXdMTjVhVjdzZGJPZEI5MjJQeS1jeFFxNWdMRVpTX3JmNldpRVpXY1ZaQXVaZVh4ZUtxeEQxWklhS1Z6YnhYellTMVBJYjkzcVVtZ2NvMkF3Slh0WmRFZW1ibWRnQWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOVFJXZkVVUUlxUFdTUTY3LURqTi1Xb2ZpY0FMZHJNZjRuSzdyWEFmMEFJYWJHeWxibjhIZGF6MWZEbHMzYzRmU1Z6eVB4WmY5YjlDVDd0bU1RNTRBdXFOQjJYRGQ1SVlFd0xLZ2hyYlExMHBOU3dYLUlJY1U1b2JRYzR6bmFFQ21LNl9peDNCT2JWUl9PTUlTcE9TX09PQm5ZWjhxY2VTX0JmbXRodjg4cXgxSDhYUGVGU0dqZA?oc=5</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Agora é definitivo: Mosaic fecha e coloca à venda fábrica de fertilizantes em Araxá - AgFeed</t>
+          <t>Mosaic paralisa operação de fosfatados em MG e põe à venda ativos - Globo Rural</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQVVZOR05sajZPcjc0SGtxemVRUVFyVnA4UjlZVlktLXppRjY1ZzVVZXBMbnlwX2VLNXpNajhWeHJMb3dqYWhlY3d6ZkhMdnVncWpoS18wa0p3UUxzZnJXN09NNDFRYloxaVc3QXI1bWVwZVpfWC1ES2Q3SVFzUVVockJyZkhOZ2dXN19TN1NvNVpXaWVQRmZTYlJVRkJqVDAtR3dnb29LX0pNVU00OUxCaHdFNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNZmtnalFlYUVpZzc1V1FCQWVZR3d1dUR2SkJCeG43bi0teDJkVUZiclItMWp4YWxUd2tyaElmLUlEMzVnNnZsUmFhYzRLcVExdndfMml0SWJqV0plN19ZeGVwbC1JRWJuNjBmZUtXUm1ZTHhxRm5TNUJDN08tOHVGYWtBZjRZRHFJblBVeDhiT2J1UFJtS1ItcVZ2SWQzWmxHWmFYNjlqX0hfa3F4eC1SS2lfR1hNRFBMdWZV0gHKAUFVX3lxTE9xRW5TWVBCc3J3OE9JbGx1NTNnUHJlMVZXek42RDlWeTFHa2R2SXFiY3dwTkNldGZFUlhXS0xzMWdfVjRIVTdhMWdwMGQweHdCdi1Jckx5b2pQVEtZTkc4XzNpellPMEx6N2hOWXdMTjVhVjdzZGJPZEI5MjJQeS1jeFFxNWdMRVpTX3JmNldpRVpXY1ZaQXVaZVh4ZUtxeEQxWklhS1Z6YnhYellTMVBJYjkzcVVtZ2NvMkF3Slh0WmRFZW1ibWRnQWc?oc=5</t>
         </is>
       </c>
     </row>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Mosaic, fabricante de fertilizantes, vai paralisar produção de 1 milhão de toneladas de fosfato em meio à alta dos preços - InvestNews - InvestNews</t>
+          <t>Agora é definitivo: Mosaic fecha e coloca à venda fábrica de fertilizantes em Araxá - AgFeed</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxOMlE2aTNkQ1drWHNGNjhJckFIY3hkM1A2S3lfdkhJbXBtaDN5VmV4NHVPNFdra1FTXzV2ZUprdGNsaDZxa21sWmk2dlpabDJ3aUpROUE3YVdFd0VEZDdscnd0RjAzS3huS1N1Ujh0b01DVld0OUpWUDV4c091SW1kcjBDNFRHZDl0ZTdIMFBlTHRuRnZYenNneG4yUHFLa1BnZEhmY1ZhenhwSTJpb0NFdXE3dDBGVlI3aERwQ0NHWWk0d0JBdS04dFZzbHNySXZNcFp2YlJGNjVCNnZ3YUZtdW55MHhQa29QVnhn0gHwAUFVX3lxTE9IakdwRXpVeExMWDhnSkZFci1UWFRqLTZscWVWcS11Q3lSMmdnX2V4Mm1IUmw5WEF6MURadm1KdEdlLWxMWjlIa3lBNXVJYjVrSzdBTHA4QUFTblNrSV9uRDdLR2g0R3lrUTBSV2hEMi1IVHdHeUxFdVZCNU9xbTktc0xHWUVnLWliZThlUnplY3pGbDBnaXdPTFpicFZ1NEo4RGdjbVlEUW5HSDlIb2U3RUZQLTRlOVBWZVZQZDU3WDR3YkJZbmJ5WHBXa0RZZXIzc3hpbU5OSFo2cWF6M05iZHJUVzl1VWhaRnZUblhWVw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQVVZOR05sajZPcjc0SGtxemVRUVFyVnA4UjlZVlktLXppRjY1ZzVVZXBMbnlwX2VLNXpNajhWeHJMb3dqYWhlY3d6ZkhMdnVncWpoS18wa0p3UUxzZnJXN09NNDFRYloxaVc3QXI1bWVwZVpfWC1ES2Q3SVFzUVVockJyZkhOZ2dXN19TN1NvNVpXaWVQRmZTYlJVRkJqVDAtR3dnb29LX0pNVU00OUxCaHdFNA?oc=5</t>
         </is>
       </c>
     </row>
@@ -7904,7 +7904,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Mosaic suspende operações no Brasil e reduz produção em 1 milhão de toneladas - Investing.com Brasil - Finanças, Câmbio e Investimentos</t>
+          <t>Mosaic planeja venda de ativos e paralisa operações após impacto do enxofre - CNN Brasil</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOb1pWNXlKY05IeUlLM2M5NUFqWmYtWEgzYWR3UFh4Y2tISnlBZ0JWVnVfMF9POEFOM1k2dXZ2X0k0Z3FpVzYyNUsyRlJCTEs1Mmw0cGhibGdaTXNrMXMxWTA4VmwwSC00TkREbEJQTk5kekdxc3FFQkN1YmxrT1UxOHhyc2YxZFgtUWNLRXdmdi14SlZZY29CUzBxOE4xY3J5Nm41aDBrYVRQS2JyQUZfaDl2T2d3eXZRd1RUSE8xdUtzT3pQOXdDTmFtc2ZyQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNWjZGTlNiamVJY2FzNVQzeG1ScDYyZ2JadVBQOW00WFpNYVNVWG9aVXNXS3p1b1lXMFZVVHNHNktHLVZmUS1teWlzWVhwVVJXV091eE91V3BiZ3E0emdVTzA1NW5LZlVxRnhKb0tmcE9kLU5ZaGhxdlZ2QjdMcXEzZXRWN1paZGhxYzNxa3d4ajZwSDkwR0Fvc3ZHYmgtandQbTF5eU95MFZEMEVjb0U0?oc=5</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Mosaic suspende operações em MG e mira corte de até US$ 80 milhões por ano - Exame</t>
+          <t>FERTILIZANTES | Mosaic anuncia paralisação das instalações de Araxá e Patrocínio e busca vender ativos de Araxá - Brasil Mineral</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -7936,7 +7936,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNdEZqNHdRb0pLX2tyVWRjNVk0SmdMUEdIdjVMbGFOb25QLXdaNXFBU0w5a1REbXFUcjFKV2lYSUNYTk9UQXV1Q1hHeVozUDdCdWhvXzlhQ0lLM1dYZUZyaDBhNXNmV0xmWHJBMFVqV3BwUkxEY2s5N0FTMkE5ZW9tRG9qbW44WUVyNWF4ZXhqaURvWEFvOXhtV2EzZnJEZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPNVM2Q3ktX2tVc29Wb3RHZGdacTN1TXFhS0xET1k1YmVVWXY2MUI4NVNIUUJENUl6M1ZDM1lIQzNBUi1zYmVYcWJvM3JxSHJLSU13R3NCNG0yS0NfRUpWaGVSRV8wUUt4M2taUGdzX01qUHA3dFpPQ1QzSFpnLTU1TC1oZXBzQVAtcXl3cHhKZ25aNG9FbGt5TVdsNlRqOG1EVmxqNS1vSHZUNVFPWjJZcVZJT01KeGIza3FYYzUtWllscFVtSnlmMkVBMA?oc=5</t>
         </is>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Indústria de fertilizantes alerta: pode haver desabastecimento - AgFeed</t>
+          <t>Alta do enxofre preocupa indústria de fertilizantes, que vê risco de desabastecimento - AgFeed</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPbXRMZ0dqOWVnR0xjWk9PTFBFUWNBdUd0SUhMOWFNZWFEay0tSlUwZXZTbG9MSnZ4eWVHTHFjRktzZ01ZRy1qdWh4cUdaQmFNWFpXR3BnMjRLcDNLcEFfM1dQSkpWX3k4emZfREtVZUt5OUZCbzhQXzAwLWhBdi1CWGcwd3E0WXkzOEthRlBISUpTUFAxYWRpVmE5ZWdKYXBkYWRydnVmNTRibUE4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOd3piekJKRGJmWE80SVlOQ2NWLVBibnRnc29HR253UlVrNndYQ0F2eUJ3V3BWaGQ0NE5RT0V5c25FeWMwekJxYV9SQUNxZ1NhNTdFQUZDbHF4VFF0LWVMc2lWR3lxd1ZqRGtqM3ZkWHozOElSQlVRYko0WWVaeHJxa2JQREdtSEJOS05iWkxhRkxOZ25RQ3VEMVZIR2xMeVVzc0luand4ZEpVTVNwelNzeTBDa0ItWTA?oc=5</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Alta do enxofre preocupa indústria de fertilizantes, que vê risco de desabastecimento - AgFeed</t>
+          <t>Indústria de fertilizantes alerta: pode haver desabastecimento - AgFeed</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOd3piekJKRGJmWE80SVlOQ2NWLVBibnRnc29HR253UlVrNndYQ0F2eUJ3V3BWaGQ0NE5RT0V5c25FeWMwekJxYV9SQUNxZ1NhNTdFQUZDbHF4VFF0LWVMc2lWR3lxd1ZqRGtqM3ZkWHozOElSQlVRYko0WWVaeHJxa2JQREdtSEJOS05iWkxhRkxOZ25RQ3VEMVZIR2xMeVVzc0luand4ZEpVTVNwelNzeTBDa0ItWTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPbXRMZ0dqOWVnR0xjWk9PTFBFUWNBdUd0SUhMOWFNZWFEay0tSlUwZXZTbG9MSnZ4eWVHTHFjRktzZ01ZRy1qdWh4cUdaQmFNWFpXR3BnMjRLcDNLcEFfM1dQSkpWX3k4emZfREtVZUt5OUZCbzhQXzAwLWhBdi1CWGcwd3E0WXkzOEthRlBISUpTUFAxYWRpVmE5ZWdKYXBkYWRydnVmNTRibUE4?oc=5</t>
         </is>
       </c>
     </row>
@@ -8031,12 +8031,12 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>Biofragane</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Ormuz: 20% da energia, 30% do GLP e 50% do enxofre - Agência de Notícias Brasil-Árabe - ANBA</t>
+          <t>Empresas compram terrenos no Distrito Industrial de Ponta Grossa e prefeitura arrecada R$ 11,8 milhões - Bem Paraná</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -8046,19 +8046,19 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE91akhDZG5kTFBRM2x2UVhuWGZfa1hOZENjNFotbEI4QnRDU2VYaGtjWm5jUHo3MnJWalZQLVdVbnU0SGl5WkNkd0ZBdXFXa2RYSF9DLTBEYnpLa2hoM1dYcmQ4SERVdlFVdjEtMXk1SnVRYkdY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxQdjVTa3FTVDU1VGZQay1sMlVFTkw3eHRVdXFlVWxrbGtMRnU3aFIyTnpWZ3NEeURSYjJJTDhlWTVOeUtoZWFrNm1zNnRtNEZNVXJMMlhWSFJJYXNzckdOTUxZUjcxYXczMzhqVGFhZHhPemVZbFhhYktFVXZDTzZjZlp6OGJ5czlxdjJnZnB5SzgtMVlpQTI1TmFKSFloZ0lyMHpsSHpQRm90cTdid0lKcmR3QTQ1RUpwS05LRzNJZmdWbm1UZXdGek1reDlKNU1LdzZzbUQ3NGJTQ0ZFQ2NBTWpnNTltU0VNMFdQSy1kM0dib3Np0gH6AUFVX3lxTE40RlkzbktwRTA5SmFTOGw2Ykt0TUd1ZlotUGtnRmpiSGFnWVR4Um95cUlILUwxYkVjcE01OVZreXdGdW9ERmVya0M0MHNCTUpjOS04cVhoSktGcnliRTBhUmdndlJ2NVVDb3dkQ2IwOVlRNHRCdEcyZ3laemtUdS0zQmVpdVBEX2FoVi1MbXlhenZ4R05sSlpNZUpTUkhhV0l1SUJYU1lhUDRnc1MzU2h3ZWQ2a1h2S05DZnlyRGRKbUlVcWFjT1NoNGhmR196T2F0OWR6YWZXaWxjTFdYU1lLMEpnR2ZPZ3ltRERhaGNYdUlJSjRraTdUYUE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Biofragane</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresas compram terrenos no Distrito Industrial de Ponta Grossa e prefeitura arrecada R$ 11,8 milhões - Bem Paraná</t>
+          <t>Ormuz: 20% da energia, 30% do GLP e 50% do enxofre - Agência de Notícias Brasil-Árabe - ANBA</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxQdjVTa3FTVDU1VGZQay1sMlVFTkw3eHRVdXFlVWxrbGtMRnU3aFIyTnpWZ3NEeURSYjJJTDhlWTVOeUtoZWFrNm1zNnRtNEZNVXJMMlhWSFJJYXNzckdOTUxZUjcxYXczMzhqVGFhZHhPemVZbFhhYktFVXZDTzZjZlp6OGJ5czlxdjJnZnB5SzgtMVlpQTI1TmFKSFloZ0lyMHpsSHpQRm90cTdid0lKcmR3QTQ1RUpwS05LRzNJZmdWbm1UZXdGek1reDlKNU1LdzZzbUQ3NGJTQ0ZFQ2NBTWpnNTltU0VNMFdQSy1kM0dib3Np0gH6AUFVX3lxTE40RlkzbktwRTA5SmFTOGw2Ykt0TUd1ZlotUGtnRmpiSGFnWVR4Um95cUlILUwxYkVjcE01OVZreXdGdW9ERmVya0M0MHNCTUpjOS04cVhoSktGcnliRTBhUmdndlJ2NVVDb3dkQ2IwOVlRNHRCdEcyZ3laemtUdS0zQmVpdVBEX2FoVi1MbXlhenZ4R05sSlpNZUpTUkhhV0l1SUJYU1lhUDRnc1MzU2h3ZWQ2a1h2S05DZnlyRGRKbUlVcWFjT1NoNGhmR196T2F0OWR6YWZXaWxjTFdYU1lLMEpnR2ZPZ3ltRERhaGNYdUlJSjRraTdUYUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE91akhDZG5kTFBRM2x2UVhuWGZfa1hOZENjNFotbEI4QnRDU2VYaGtjWm5jUHo3MnJWalZQLVdVbnU0SGl5WkNkd0ZBdXFXa2RYSF9DLTBEYnpLa2hoM1dYcmQ4SERVdlFVdjEtMXk1SnVRYkdY?oc=5</t>
         </is>
       </c>
     </row>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Ureia avança ao maior nível desde 2022, mas demanda brasileira perde força - CNN Brasil</t>
+          <t>Preço da ureia dispara e atinge maior patamar desde 2022 - Poder360</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -8090,19 +8090,19 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQai1ZMXRrWW8zbGNQRWwyOXVteEg3SnVUZWtIUGpJVTFKUmM5VmlkbDdnYWhIN3VDSmR1Sk5mOXVyU1ZSM1hBS1YzUnRkdXh4RkM2aGNTVzQtWDdsb29ab0J2RHFPR1lvWjV6eXZBaU5WbmhYSzBRb2N0ejFaSldHdTFveEtMb2pWZXZMbnlNSmxyU2lJaTB4T2w2QThOSHFqbEEtVXVXUFRaaVZCeHVrdElxbWp0RHA5Ny1kZGphcWJVR0RUWjhfZXJR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPZUIxSkk2bGJHRnlhMlNaYW5xVVdiZmctUGhDQ0NFQXlmakJzOFhwN0JrTVFOUzZmeGFaV0dwSUJsaDdZdy1DVEJRR0JDMjJGbVdEelpFNjQ1ZVQ2cFQ3Q1MzbmtrMklTT1p6UDd6MzBQcVVDT215MkluWWJnb0NQbjBTQnFHQXZwNXhGRXF1akk4bDJGMWY5SGF0SkM?oc=5</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Cal Cruzeiro</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Preço da ureia dispara e atinge maior patamar desde 2022 - Poder360</t>
+          <t>Caldense apresenta elenco para temporada de 2026 - onda poços</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPZUIxSkk2bGJHRnlhMlNaYW5xVVdiZmctUGhDQ0NFQXlmakJzOFhwN0JrTVFOUzZmeGFaV0dwSUJsaDdZdy1DVEJRR0JDMjJGbVdEelpFNjQ1ZVQ2cFQ3Q1MzbmtrMklTT1p6UDd6MzBQcVVDT215MkluWWJnb0NQbjBTQnFHQXZwNXhGRXF1akk4bDJGMWY5SGF0SkM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE95MkZIWmpVeXBPdDVYRy13QnhHYnZtd3dHOUpQcnV0VmliYmNLemhIZXRZTVhVMmFqTjRBMmNJQTl2dVF0TWJTWEV6M3k1MzBQbGpJVWN5MWhVNVlxTFl3ZVNCdlFld2RyX19qUlJRLWtUTlVLdXZBRFY3RDYyLTg?oc=5</t>
         </is>
       </c>
     </row>
@@ -8124,7 +8124,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Caldense apresenta elenco para temporada de 2026 - onda poços</t>
+          <t>Caldense apresenta jogadores que vão disputar o Módulo II do Mineiro de 2026 - PocosCom</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -8134,19 +8134,19 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE95MkZIWmpVeXBPdDVYRy13QnhHYnZtd3dHOUpQcnV0VmliYmNLemhIZXRZTVhVMmFqTjRBMmNJQTl2dVF0TWJTWEV6M3k1MzBQbGpJVWN5MWhVNVlxTFl3ZVNCdlFld2RyX19qUlJRLWtUTlVLdXZBRFY3RDYyLTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPaHBlSjh0OEN5c0hhaFNud3ZtU0pacFBRUlFfQkVTWVZBczJiWE5IZklZbjQ2ODBiZ3FOeFoteG91X2NVWE00anhaTDA5dGRidTA1MUxqYkRIaEtBblZ3SkY5VWdfRmc4RUxaeHV6VW5yUmNTeWNlREp6LUpSNmg2TFYwMzNWSll1NkJMTFhtT2FXWVJDTWtTaVAtMDJnaUU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Cal Cruzeiro</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Caldense apresenta jogadores que vão disputar o Módulo II do Mineiro de 2026 - PocosCom</t>
+          <t>Ureia avança ao maior nível desde 2022, mas demanda brasileira perde força - CNN Brasil</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -8156,7 +8156,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPaHBlSjh0OEN5c0hhaFNud3ZtU0pacFBRUlFfQkVTWVZBczJiWE5IZklZbjQ2ODBiZ3FOeFoteG91X2NVWE00anhaTDA5dGRidTA1MUxqYkRIaEtBblZ3SkY5VWdfRmc4RUxaeHV6VW5yUmNTeWNlREp6LUpSNmg2TFYwMzNWSll1NkJMTFhtT2FXWVJDTWtTaVAtMDJnaUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQai1ZMXRrWW8zbGNQRWwyOXVteEg3SnVUZWtIUGpJVTFKUmM5VmlkbDdnYWhIN3VDSmR1Sk5mOXVyU1ZSM1hBS1YzUnRkdXh4RkM2aGNTVzQtWDdsb29ab0J2RHFPR1lvWjV6eXZBaU5WbmhYSzBRb2N0ejFaSldHdTFveEtMb2pWZXZMbnlNSmxyU2lJaTB4T2w2QThOSHFqbEEtVXVXUFRaaVZCeHVrdElxbWp0RHA5Ny1kZGphcWJVR0RUWjhfZXJR?oc=5</t>
         </is>
       </c>
     </row>
@@ -8207,12 +8207,12 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>corretivo de solo</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Corretivo de solo sustentável entra para o programa RenovaBio e gera Créditos de Descarbonização | SEGS... - SEGS Portal Nacional</t>
+          <t>Ureia dispara 50% em 30 dias - Agrolink</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -8222,7 +8222,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxORmVta1REUjdPWkExNEhZTGZITGUzbEI2R1Rnak9WLUMxU0pRNUU3VGR6OWJiNl9GT01PZzFKRW04RmNWWnpIbnRFanBWb29IRVktdzVqaklGYWZxUXF5dllNeExCb1hsa1ZVRmJkeEsxdURUS3Jaa1VCRGl3dTg0T1h2Zmp3bWsteDhaSXBYR09jTTRNUWpuTGppVzBQdUs5eXRPQXpvRXhNbW1JMk5mVE5nT21zenVFbXA3Q1JaNVBYalVEdENiNzk3UzE0aEQwY2xV0gHYAUFVX3lxTE9jaFo0ckh1SXZ5OUY2TERFNEtfYW0zRXRfYkVvRUo3dXNwY1VLOW1QYmpINks4UzJ0X1pCcWQ2SG85a1p1VDNMaUIwczBCdGdlRGFvbVhrVmdkV2tMMGQtN0ktcTN1OUp5bWo1Wk1NaElZVDlXMVhRbFp6b29hVF9EbGRGLU9oY3B0dXN1RGtXdlpRcGxxd3NRWEdLbkJPTmVhMi04Z2txRVdWdTdvRE9HZ3ZmQ2RudklnZnB0ZEJyWS1tMnUzdTdCb3Q3allTb3dteXlyN0N6dQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPR09odVVVZHhCMVdaUTBiOXJndXB2a3E5V1BsSklCMWJvdmhZM010SGNXc1p5ajJoc1FSUzJWTmNDZGFnczBRYzlvc091a2hTYmgyWXZUWmNKam9ranNtNXBtR1Vmd3p4TlItNXUySFgxMnZPaVd4R29qY2RXVXdJM3ZvOA?oc=5</t>
         </is>
       </c>
     </row>
@@ -8251,12 +8251,12 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>corretivo de solo</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Ureia dispara 50% em 30 dias - Agrolink</t>
+          <t>Corretivo de solo sustentável entra para o programa RenovaBio e gera Créditos de Descarbonização | SEGS... - SEGS Portal Nacional</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPR09odVVVZHhCMVdaUTBiOXJndXB2a3E5V1BsSklCMWJvdmhZM010SGNXc1p5ajJoc1FSUzJWTmNDZGFnczBRYzlvc091a2hTYmgyWXZUWmNKam9ranNtNXBtR1Vmd3p4TlItNXUySFgxMnZPaVd4R29qY2RXVXdJM3ZvOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxORmVta1REUjdPWkExNEhZTGZITGUzbEI2R1Rnak9WLUMxU0pRNUU3VGR6OWJiNl9GT01PZzFKRW04RmNWWnpIbnRFanBWb29IRVktdzVqaklGYWZxUXF5dllNeExCb1hsa1ZVRmJkeEsxdURUS3Jaa1VCRGl3dTg0T1h2Zmp3bWsteDhaSXBYR09jTTRNUWpuTGppVzBQdUs5eXRPQXpvRXhNbW1JMk5mVE5nT21zenVFbXA3Q1JaNVBYalVEdENiNzk3UzE0aEQwY2xV0gHYAUFVX3lxTE9jaFo0ckh1SXZ5OUY2TERFNEtfYW0zRXRfYkVvRUo3dXNwY1VLOW1QYmpINks4UzJ0X1pCcWQ2SG85a1p1VDNMaUIwczBCdGdlRGFvbVhrVmdkV2tMMGQtN0ktcTN1OUp5bWo1Wk1NaElZVDlXMVhRbFp6b29hVF9EbGRGLU9oY3B0dXN1RGtXdlpRcGxxd3NRWEdLbkJPTmVhMi04Z2txRVdWdTdvRE9HZ3ZmQ2RudklnZnB0ZEJyWS1tMnUzdTdCb3Q3allTb3dteXlyN0N6dQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -8361,12 +8361,12 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>calcario agricola</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Sindical-BA alerta para impacto da nova tributação sobre calcário agrícola, que deve elevar custos do setor - Sistema FIEB</t>
+          <t>Alta da ureia pressiona mercado e pode impulsionar uso de alternativas em 2026 - Feed&amp;Food</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -8376,19 +8376,19 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOQUNveWVYZUNwX3BMRXdqRzdqUThDTkNOZk9vVWNMbHNsVlg2N1oxcDZjRV9nVHVrajNfaGVieG5RYVhiMDhjeGxobmdCRmhkQnFDSy1rR2hvbUhjb056WTNZeWpkSGpmVWhlMWxQTjJCN0dqRFRibmZRLVhOb1R5X3c5UmZBcmlYVTNYd2trZUNCak4xWHY1OTBtUHROZVZwUm5UVWJINWc2dzgwOVg2RnJMNFlaZ0p4aFIxdjBfWUZfUi1WaGd0MVJEeDhFa1ByeXhmVThUVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOZWl0bUdaQVRHdjR0MVZmM1kwREFfQjl4bl9pM3RETHFoc2QwUThjcWdFUmxzQnNSZ1Q1VjM3dXE0NXV6dEE0eURjNlZVTXVLZXpZVDdERkZWMVBjcjJjd0lrQWowSFptbVBpVGx2c1V2WDdweUJYQ0l6RVlHdHZUbXZKQkdKMDVxVkVYekV3dnhzUk5QeVd6WHZiM2pLU244eGk4SjNB?oc=5</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Alta da ureia pressiona mercado e pode impulsionar uso de alternativas em 2026 - Feed&amp;Food</t>
+          <t>Mosaic, gigante do agronegócio, aposta em IA para enfrentar volatilidade e reduzir custos logísticos - Globo Rural</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -8398,19 +8398,19 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOZWl0bUdaQVRHdjR0MVZmM1kwREFfQjl4bl9pM3RETHFoc2QwUThjcWdFUmxzQnNSZ1Q1VjM3dXE0NXV6dEE0eURjNlZVTXVLZXpZVDdERkZWMVBjcjJjd0lrQWowSFptbVBpVGx2c1V2WDdweUJYQ0l6RVlHdHZUbXZKQkdKMDVxVkVYekV3dnhzUk5QeVd6WHZiM2pLU244eGk4SjNB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxOME5qTE54MnlMcWFJeS02bUs2dGRlR0VSRWJHT001NEtPcS1XaURNbC1UaGd1Q2hkWld2ay1ITHptMTdBcHRPLUJPVzZWTkR5d21GNHJHZGEwZ3U3ckltNnNQN2x3WnQtT2FwdkJ1eTNDYVFSX2ZreUJ2dFQ3M1pOSENSRGhTeTg5djRfaWxWbC1FTEp5TWVBR24wVlNZNEhLc2N0VVB5XzAxWXZqbHNJU2hTUUQ2dlJRaTRkTGdId3NIREtxdWR1dXpqSVY4V1lQRlJzbTVodXFSOXBpT05RVkdpZmJSNXVpYzJGaUdLcjUwLWQyNGdoMWNlOVBVSU5PQmVjX1o5cmZPN1pY0gGbAkFVX3lxTE5YUjI3TVduTnRpaUdEeW0tYnZvSGpRdHd4MXE1VUtsc3ZsQ004emFwdGU4cFZqQ25XSnVTQjYxUG5DNE4xcHZKZk1JLXNjVk5hMkNuNmJZdllRVW5uQmtGQ0o3UVBJLWp5M0g4YXJPY3FqajNsVWttc2pJNjBFdHpkMVFEYWJvaGZUU1hQMXFzTDNleFhVakdxTmRPTElXTXA4U0xacTJfNFYwS0I4UE42S0wydUtudEU5d0RNOGYtQk83SVBtc3VFeTk3X3BhOHVFanBOd3VEaHYySllENWMxdnhDRUJXd2VfNXdhRDl0cHRkVU1BM3ViMWt2azdDbW03THJ0WGRBQllJaW1aRVM1WEJuSTdRNm9Bak0?oc=5</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>calcario agricola</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Mosaic, gigante do agronegócio, aposta em IA para enfrentar volatilidade e reduzir custos logísticos - Globo Rural</t>
+          <t>Sindical-BA alerta para impacto da nova tributação sobre calcário agrícola, que deve elevar custos do setor - Sistema FIEB</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxOME5qTE54MnlMcWFJeS02bUs2dGRlR0VSRWJHT001NEtPcS1XaURNbC1UaGd1Q2hkWld2ay1ITHptMTdBcHRPLUJPVzZWTkR5d21GNHJHZGEwZ3U3ckltNnNQN2x3WnQtT2FwdkJ1eTNDYVFSX2ZreUJ2dFQ3M1pOSENSRGhTeTg5djRfaWxWbC1FTEp5TWVBR24wVlNZNEhLc2N0VVB5XzAxWXZqbHNJU2hTUUQ2dlJRaTRkTGdId3NIREtxdWR1dXpqSVY4V1lQRlJzbTVodXFSOXBpT05RVkdpZmJSNXVpYzJGaUdLcjUwLWQyNGdoMWNlOVBVSU5PQmVjX1o5cmZPN1pY0gGbAkFVX3lxTE5YUjI3TVduTnRpaUdEeW0tYnZvSGpRdHd4MXE1VUtsc3ZsQ004emFwdGU4cFZqQ25XSnVTQjYxUG5DNE4xcHZKZk1JLXNjVk5hMkNuNmJZdllRVW5uQmtGQ0o3UVBJLWp5M0g4YXJPY3FqajNsVWttc2pJNjBFdHpkMVFEYWJvaGZUU1hQMXFzTDNleFhVakdxTmRPTElXTXA4U0xacTJfNFYwS0I4UE42S0wydUtudEU5d0RNOGYtQk83SVBtc3VFeTk3X3BhOHVFanBOd3VEaHYySllENWMxdnhDRUJXd2VfNXdhRDl0cHRkVU1BM3ViMWt2azdDbW03THJ0WGRBQllJaW1aRVM1WEJuSTdRNm9Bak0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOQUNveWVYZUNwX3BMRXdqRzdqUThDTkNOZk9vVWNMbHNsVlg2N1oxcDZjRV9nVHVrajNfaGVieG5RYVhiMDhjeGxobmdCRmhkQnFDSy1rR2hvbUhjb056WTNZeWpkSGpmVWhlMWxQTjJCN0dqRFRibmZRLVhOb1R5X3c5UmZBcmlYVTNYd2trZUNCak4xWHY1OTBtUHROZVZwUm5UVWJINWc2dzgwOVg2RnJMNFlaZ0p4aFIxdjBfWUZfUi1WaGd0MVJEeDhFa1ByeXhmVThUVQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -8432,7 +8432,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Comissão do Senado aprova redução de tributos que incidem sobre o calcário - Canal Rural</t>
+          <t>CRA aprova selo para café e alíquota menor sobre calcário - Senado Federal</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -8442,19 +8442,19 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPQ2h1ODE3WFlWWnVpN3Q0TVAwajZrUXVDbmRpeFFZSWt6WGJXLXNKSVREWFdXYUNQeVprdjlieGxDS0xxU3J0SkMwWlRPXzlvVFZWWTJNRVRvN0dSV044Y1pwMHprUmhqRURpcGRjWFVfaENjX0U5bE1UaW1KNFdvUExibEZad1A3SmpOQlNxZTFselNXMDdRLTdBOGRpZXpiWEgzMS1SN3FLNUdybkxQbndoa0NFT1By?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNY2pRTWs2S3NtQlQwenhTVkJoWWpXV1ZYWEJmS1ZBcVRJOUNnYUR1YUJEXzRneGxSdlZFenh3d1c4TXVLaktTSi1Xek5TUEU3d0ppS2s4ZTdBaG9QSzcxV1pmOVpZOU16Tjl1T05kT3lIaHNkRXBtck9UY2xOYnpVVFV1MWMxTjdFbXYzektEQ1I4Uy00MU41dTQ2ODhzV1p2MUpENTZ6bUV4dzlOaXc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>calcario agricola</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Desembargador da Bahia retoma negócio bilionário de ouro entre chineses e canadenses - Folha de S.Paulo</t>
+          <t>CRA aprova redução de tributos sobre calcário para uso agrícola - Senado Federal</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -8464,19 +8464,19 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQdXBkMXpzTml3eG90ck82aFdOU0U3Z0pDRWMtd0NzclBRVzI3WTY1by1pVEhkTkFLbjgwUVR4MUZpWXI5S3lOOC1CRVRPaTdNT3dSOEMwZDZKNTdzc09OcEQ1M1RNOTVEVmJBaWhCRGNWRDI3Qldval8yWTdLNG9oek41LVJHeUdKYXRzMVhaalN6TzFCdlFIbzhfMkJ1clduV25GYVVYVmdqSXJRYlg5d2FmdEMtZmlRazdUdm9JWU1GWTRwcjFLNFM0RW45OC1zbUHSAdcBQVVfeXFMTnJkMWwtODlkeXZTdWk1Q1hBZnZNREtzVHZqX3VVQlBOdDY4TTNIQnI4OEVFRUVtaWxHTkNxZlhKOFN6U2RFcE56bU5zMDdUWmt1YmQtZGtXczNfTzllalRhUW9yUjdPbFBFbFpSOUlCMlBaQXI0aEVwRHNMbEw0ckJzbWVlNExKZWUtYlpQRzhUUUR3aGFveFdJenF2SmM5WkdzNy1VRzUyTWNydjU3anVOT3M2X1VsLUV4VWRqRHc4bjJoVGhGQlJlR1dvaE01enEtMVlTWmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPZi01RmRheW9LUVdwbzZ0VWR5YTZHXzI1VVFsTEZ6OXFzaVM0V1JwYXRYdmpoQjExVnRfNEtKVUtFYjVMNy1PNkFXYW91anRyOUhibHRWcTNLcU5UaTBNY3BRdzNrXzdJZ0RQenlYSWEzQ1dsZ3B5dGVKRUp3Vm5RRHl2NDEwRGVFdWZuRVRILXdSYk1qN3l3UnUyMHZyVGg0bHdIM0swOFN4MGdaNjFjMER3Q2hORGlMLTN4Nw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>calcario agricola</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>CRA aprova selo para café e alíquota menor sobre calcário - Senado Federal</t>
+          <t>Disparada histórica do enxofre pressiona fertilizantes - Agrolink</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -8486,19 +8486,19 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNY2pRTWs2S3NtQlQwenhTVkJoWWpXV1ZYWEJmS1ZBcVRJOUNnYUR1YUJEXzRneGxSdlZFenh3d1c4TXVLaktTSi1Xek5TUEU3d0ppS2s4ZTdBaG9QSzcxV1pmOVpZOU16Tjl1T05kT3lIaHNkRXBtck9UY2xOYnpVVFV1MWMxTjdFbXYzektEQ1I4Uy00MU41dTQ2ODhzV1p2MUpENTZ6bUV4dzlOaXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOREtjdjl3OVV3M3BodzJUN2tTS09qQjdCaHVYcHJVak9fWlBKcl96ZWlkaWhYSmJSazVXQ3c4LUl4YTU4MXh6VjNwd09JaGRsblVrajRXNTlHUXp6X0V1Y0E1YmYwTXZxa2ZXX1AwNEVJcnpibWRMMTRXcG9ibGRSb21BOGNHMDFxZWJhVnRmeTJ4SjY1ejUzTlVqelJ6dE4xUkFpWkhn?oc=5</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>calcario agricola</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>CRA aprova redução de tributos sobre calcário para uso agrícola - Senado Federal</t>
+          <t>Desembargador da Bahia retoma negócio bilionário de ouro entre chineses e canadenses - Folha de S.Paulo</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -8508,7 +8508,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPZi01RmRheW9LUVdwbzZ0VWR5YTZHXzI1VVFsTEZ6OXFzaVM0V1JwYXRYdmpoQjExVnRfNEtKVUtFYjVMNy1PNkFXYW91anRyOUhibHRWcTNLcU5UaTBNY3BRdzNrXzdJZ0RQenlYSWEzQ1dsZ3B5dGVKRUp3Vm5RRHl2NDEwRGVFdWZuRVRILXdSYk1qN3l3UnUyMHZyVGg0bHdIM0swOFN4MGdaNjFjMER3Q2hORGlMLTN4Nw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQdXBkMXpzTml3eG90ck82aFdOU0U3Z0pDRWMtd0NzclBRVzI3WTY1by1pVEhkTkFLbjgwUVR4MUZpWXI5S3lOOC1CRVRPaTdNT3dSOEMwZDZKNTdzc09OcEQ1M1RNOTVEVmJBaWhCRGNWRDI3Qldval8yWTdLNG9oek41LVJHeUdKYXRzMVhaalN6TzFCdlFIbzhfMkJ1clduV25GYVVYVmdqSXJRYlg5d2FmdEMtZmlRazdUdm9JWU1GWTRwcjFLNFM0RW45OC1zbUHSAdcBQVVfeXFMTnJkMWwtODlkeXZTdWk1Q1hBZnZNREtzVHZqX3VVQlBOdDY4TTNIQnI4OEVFRUVtaWxHTkNxZlhKOFN6U2RFcE56bU5zMDdUWmt1YmQtZGtXczNfTzllalRhUW9yUjdPbFBFbFpSOUlCMlBaQXI0aEVwRHNMbEw0ckJzbWVlNExKZWUtYlpQRzhUUUR3aGFveFdJenF2SmM5WkdzNy1VRzUyTWNydjU3anVOT3M2X1VsLUV4VWRqRHc4bjJoVGhGQlJlR1dvaE01enEtMVlTWmc?oc=5</t>
         </is>
       </c>
     </row>
@@ -8537,12 +8537,12 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>calcario agricola</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Disparada histórica do enxofre pressiona fertilizantes - Agrolink</t>
+          <t>Comissão do Senado aprova redução de tributos que incidem sobre o calcário - Canal Rural</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -8552,7 +8552,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOREtjdjl3OVV3M3BodzJUN2tTS09qQjdCaHVYcHJVak9fWlBKcl96ZWlkaWhYSmJSazVXQ3c4LUl4YTU4MXh6VjNwd09JaGRsblVrajRXNTlHUXp6X0V1Y0E1YmYwTXZxa2ZXX1AwNEVJcnpibWRMMTRXcG9ibGRSb21BOGNHMDFxZWJhVnRmeTJ4SjY1ejUzTlVqelJ6dE4xUkFpWkhn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPQ2h1ODE3WFlWWnVpN3Q0TVAwajZrUXVDbmRpeFFZSWt6WGJXLXNKSVREWFdXYUNQeVprdjlieGxDS0xxU3J0SkMwWlRPXzlvVFZWWTJNRVRvN0dSV044Y1pwMHprUmhqRURpcGRjWFVfaENjX0U5bE1UaW1KNFdvUExibEZad1A3SmpOQlNxZTFselNXMDdRLTdBOGRpZXpiWEgzMS1SN3FLNUdybkxQbndoa0NFT1By?oc=5</t>
         </is>
       </c>
     </row>
@@ -8647,12 +8647,12 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>limestone</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Limestone: a pedra calcária em evidência na arquitetura - Archtrends - Portobello</t>
+          <t>Importação de ureia pelo Brasil cai forte em 2026 e preço segue em alta - Farmnews</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -8662,19 +8662,19 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE5Xa21Zc0YzY0pUazFLbDJVMmlTYzcwYTd3RG1OcjNNalZVblN0N2gwMV9NczFWZURPa2MwaXNMcmxfdE5seHo0QWozSFdBbmfSAVRBVV95cUxNUEhPRGZuQlpIS1NNTm1lMW8zblJQUVVYWkhNXzlfcVk4N3dfZHRRb0xCcE9IWTZIMHdhNnYtOE4wNjh4YlBrSTY4ZUtVenF6NDdKemg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQSTZnclR2WFM3LWRESEtlMndnQWFiTU05ZzVOcDdlQ1g3RTAzVklPYTZ0YkF5RGk4MTlGR05pMEVES0pFTXlvOVpmb0ppWHk2YS1ValFtMWUxcDB5WHhpdEpZTmhkT1kzMUpMVTlYNWcwb1RWQzJNSVNxbmhOdWlvT0YzdXRBblFaZlRqdXRzeGFZZDA0anprdXZOQ1k5Z1RyZUplVlJhTWtiQ00y?oc=5</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>limestone</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Importação de ureia pelo Brasil cai forte em 2026 e preço segue em alta - Farmnews</t>
+          <t>Limestone: a pedra calcária em evidência na arquitetura - Archtrends - Portobello</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -8684,19 +8684,19 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQSTZnclR2WFM3LWRESEtlMndnQWFiTU05ZzVOcDdlQ1g3RTAzVklPYTZ0YkF5RGk4MTlGR05pMEVES0pFTXlvOVpmb0ppWHk2YS1ValFtMWUxcDB5WHhpdEpZTmhkT1kzMUpMVTlYNWcwb1RWQzJNSVNxbmhOdWlvT0YzdXRBblFaZlRqdXRzeGFZZDA0anprdXZOQ1k5Z1RyZUplVlJhTWtiQ00y?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE5Xa21Zc0YzY0pUazFLbDJVMmlTYzcwYTd3RG1OcjNNalZVblN0N2gwMV9NczFWZURPa2MwaXNMcmxfdE5seHo0QWozSFdBbmfSAVRBVV95cUxNUEhPRGZuQlpIS1NNTm1lMW8zblJQUVVYWkhNXzlfcVk4N3dfZHRRb0xCcE9IWTZIMHdhNnYtOE4wNjh4YlBrSTY4ZUtVenF6NDdKemg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>Mosaic</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Conflito no Oriente Médio eleva preço da ureia e pressiona custo da safra em Mato Grosso, aponta Imea - Notícias Agrícolas</t>
+          <t>Mosaic avalia entrada no mercado de terras raras com projeto em Uberaba - CNN Brasil</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -8706,7 +8706,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxOTnZoc1RsVHBacHBYSTJrZFhacUlvY2h1emtmRktiU3ROajdCX1pHcy04VDJXUndNUWkzMXNfVlJia1p2YVFlbmg1dUd2S2pobG5yOVMyTHR0eWhoU1J1SGt3NlNUUmdUN0JIVjFPV042UDBpT1dDYjFTOTVkVmRLa1Q4anphUWpKQ2J2SUI5R1M3aFpiTmVOVk1wQVhCSFNUM1N5S3RqM0lmWGNXU0RJeUdQbGRQNldncEJid2V6UlVIMmhsUGNmbG1KTlctT3NSOVlnOHRLeW10XzA1OEJYQkhIOHdDV203U0lvWEZIcDQzU3A5Vno3SDFnQW4zWU3SAYQCQVVfeXFMT3NyRl9SQTFZeERRb0w4Sms4dkJNaXlIRVd4eXduNFdPVlgtbkh5ZE5NVUdHU3lEUExlNXdxQi1vMi1ESzQxaVoyRHpTRlBobWlUalRvdVJCNVp4Xy1sSWZzcE1penBXWDRocjFxSjUtVmNGbDkxcTFLOGRGMHROaDU5VVl6TFBLbXJwNl9lZFhDNkdsc21qQkF6WWxEV1dDTC1raEpEZmlHZzVvY1NkbWRBTC11eTdFME83VjBoM1pQRmFFRE5NWDRQQXBGSDFUODR2UFdtTG96V05FX25WTk92ZEU5a2p5ZmN2eW9hME1INzlyMWhWak5tdlZUQkdDaFVWUHo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOaDhHU1U4Z1ZUcDhvSzBheGZqQUxjOXFvZFpKQWI5Q0pTdG4yMkMxbGtoS0JtdDg2Tm5GQ0VRMC1NZ2tBRS12RFowanRSZ0V5b2F1R0Z5RGw2NlYwbzdoRzZzS2NGbi1PNFV3aHBxRHhsUTkyeFdXdDZKS1QxV2RKdThyU2JGS1E4amZXN05CYjZFS1BpRXAwX0hmcXVVLTgwc2RqUkJFeFlKQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>Mosaic avalia entrada no mercado de terras raras com projeto em Uberaba - CNN Brasil</t>
+          <t>TERRAS RARAS | Mosaic e Rainbow planejam projeto conjunto em Minas Gerais - Brasil Mineral</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -8728,19 +8728,19 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOaDhHU1U4Z1ZUcDhvSzBheGZqQUxjOXFvZFpKQWI5Q0pTdG4yMkMxbGtoS0JtdDg2Tm5GQ0VRMC1NZ2tBRS12RFowanRSZ0V5b2F1R0Z5RGw2NlYwbzdoRzZzS2NGbi1PNFV3aHBxRHhsUTkyeFdXdDZKS1QxV2RKdThyU2JGS1E4amZXN05CYjZFS1BpRXAwX0hmcXVVLTgwc2RqUkJFeFlKQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQbWZYenFKcUV3ejJVdWJLTDYwY0duaXVYY1VhRzZ2UlNuXzh5OTZ6T19QRktEemp4WWI5S2ZqSWlWMVNRQ1FIeGhmVEtWTENVTFRYNWZobDB3blBuc3RTUUFQWnFMaVpLT01YOUhFQXg2UksyUEZMUmpVeUpGdFUtYzc2YnkwRjZDOHJGVlAwclk0cS1fOFJvRS1LN2gzZVR1NGc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>calcario agricola</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>Guerra no Oriente Médio faz preço da ureia subir e eleva custos de produção, aponta Imea - Canal Rural</t>
+          <t>Agricultores de Corupá já podem solicitar calcário gratuito pelo programa Terra Boa; veja detalhes - JDV - Jornal do Vale</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -8750,19 +8750,19 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQMjNJY202OXBERXA4andGUzdVTnZ4ODdOWnZOVU1xUFBIVDR1Tjh2RmhZdlR6VlRvVmc5Q05BSS04Nm9DSzlkQ2NHT0FVc0RCYU5uTDlkbVBfc2ZiV2FFRncxYVBEUHdBWGFMcFQ0bjQ2OFlETDdGR1ctTXlkbkZaUEt1bDNPYlZ1d3RibF9KaEFQMldpeW1rckFyWjBtX0kyTU1LemJtVE9sN3Bla0tiVDl4ZlV3UENHOWU3b09nS0tSOG5OQkE4MGdR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBoVzBPSUx1aFltY2FyUnN2Ym1qNExJZkxKckl1bnpsdGwzT2hZdF9PaDN1SHhFV1pQRTNmTWM1TXMtakYyUERmcmRwaVpLRk5kb2JUZ1NobzJVblFVWEp2c0xvVVh2ZDg1WEE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>calcario agricola</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>Agricultores de Corupá já podem solicitar calcário gratuito pelo programa Terra Boa; veja detalhes - JDV - Jornal do Vale</t>
+          <t>Guerra no Oriente Médio faz preço da ureia subir e eleva custos de produção, aponta Imea - Canal Rural</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -8772,19 +8772,19 @@
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFBoVzBPSUx1aFltY2FyUnN2Ym1qNExJZkxKckl1bnpsdGwzT2hZdF9PaDN1SHhFV1pQRTNmTWM1TXMtakYyUERmcmRwaVpLRk5kb2JUZ1NobzJVblFVWEp2c0xvVVh2ZDg1WEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQMjNJY202OXBERXA4andGUzdVTnZ4ODdOWnZOVU1xUFBIVDR1Tjh2RmhZdlR6VlRvVmc5Q05BSS04Nm9DSzlkQ2NHT0FVc0RCYU5uTDlkbVBfc2ZiV2FFRncxYVBEUHdBWGFMcFQ0bjQ2OFlETDdGR1ctTXlkbkZaUEt1bDNPYlZ1d3RibF9KaEFQMldpeW1rckFyWjBtX0kyTU1LemJtVE9sN3Bla0tiVDl4ZlV3UENHOWU3b09nS0tSOG5OQkE4MGdR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>Mosaic</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>TERRAS RARAS | Mosaic e Rainbow planejam projeto conjunto em Minas Gerais - Brasil Mineral</t>
+          <t>Conflito no Oriente Médio eleva preço da ureia e pressiona custo da safra em Mato Grosso, aponta Imea - Notícias Agrícolas</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -8794,7 +8794,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQbWZYenFKcUV3ejJVdWJLTDYwY0duaXVYY1VhRzZ2UlNuXzh5OTZ6T19QRktEemp4WWI5S2ZqSWlWMVNRQ1FIeGhmVEtWTENVTFRYNWZobDB3blBuc3RTUUFQWnFMaVpLT01YOUhFQXg2UksyUEZMUmpVeUpGdFUtYzc2YnkwRjZDOHJGVlAwclk0cS1fOFJvRS1LN2gzZVR1NGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxOTnZoc1RsVHBacHBYSTJrZFhacUlvY2h1emtmRktiU3ROajdCX1pHcy04VDJXUndNUWkzMXNfVlJia1p2YVFlbmg1dUd2S2pobG5yOVMyTHR0eWhoU1J1SGt3NlNUUmdUN0JIVjFPV042UDBpT1dDYjFTOTVkVmRLa1Q4anphUWpKQ2J2SUI5R1M3aFpiTmVOVk1wQVhCSFNUM1N5S3RqM0lmWGNXU0RJeUdQbGRQNldncEJid2V6UlVIMmhsUGNmbG1KTlctT3NSOVlnOHRLeW10XzA1OEJYQkhIOHdDV203U0lvWEZIcDQzU3A5Vno3SDFnQW4zWU3SAYQCQVVfeXFMT3NyRl9SQTFZeERRb0w4Sms4dkJNaXlIRVd4eXduNFdPVlgtbkh5ZE5NVUdHU3lEUExlNXdxQi1vMi1ESzQxaVoyRHpTRlBobWlUalRvdVJCNVp4Xy1sSWZzcE1penBXWDRocjFxSjUtVmNGbDkxcTFLOGRGMHROaDU5VVl6TFBLbXJwNl9lZFhDNkdsc21qQkF6WWxEV1dDTC1raEpEZmlHZzVvY1NkbWRBTC11eTdFME83VjBoM1pQRmFFRE5NWDRQQXBGSDFUODR2UFdtTG96V05FX25WTk92ZEU5a2p5ZmN2eW9hME1INzlyMWhWak5tdlZUQkdDaFVWUHo?oc=5</t>
         </is>
       </c>
     </row>
@@ -8823,12 +8823,12 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>calcario agricola</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Prefeitura de Santa Cruz abre inscrições para distribuição gratuita de calcário a produtores rurais - Portal Arauto</t>
+          <t>Agricultores de Corupá já podem solicitar calcário pelo programa Terra Boa - OCP News</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPZjd1TFdpbmV2Ui03ajM5WE9GaWNPUFZ3bVJJd3h3Q2JOdU05Q3Q2c0V1Y1FObVJFXzRTbWg3RVZXVzd5YUd6bXltMGEteUZ0WG5aUzZVckhwVVBBX3ppbDZ3S1NCZ1pnM1hHQlZwcDAxQ1pfa0FjNlFHOHRocHlvdzdvaTlON2lVdjJtaHRfRnpiRkFhcElYYmMtc1ZQTVlTQ3hFMnRLNTRlU0w1VjE2UW9ZUXpzcy02SHRDUGNLZDRhSDRqV3kyRUlPVWRKRjQwaFpnVHZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOemxVOFYzVUJ5cXJKbGM5eVZQUkpkdEVXdk5DcVlpcnFMYWNYOXdNRzdUdTd0ZGFTeDNjNXZHOFUxemZXMUlKYmNJcHowaktZOFgxYmUyYjliQ1Nsc2ZMUVZ2VW5QU284VUI5bi1QdXpnRGg2aDJtSmZTNGFfa0V6Y2VOQnppSndEMW9UQWNERWdaVnJCb01lQ1dxOWd3UnFNaFE?oc=5</t>
         </is>
       </c>
     </row>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Conflito no Oriente Médio dispara preço da ureia e afeta agro do Nordeste - Movimento Econômico</t>
+          <t>Conflito no Oriente Médio dispara preço da ureia e afeta agro do Nordeste - Visão Agro</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -8860,7 +8860,7 @@
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQanphVHkycWR3c05tQ1VBYkl5b3pncV9sRGlGVmJvLVpOUUZRcWRvOFdXc1hhSVFqbDBZMlFNSEdVcnNCVGppQ2ZGMVl5WFN5SUJNWS1FLUVuRUpPRFh3VFZHdk54TndBaU4yZW0zQ3dVeWN3MWpFZTVpRUZudm81MlZTa1NoV2hxSWNxLWltS1piVXJwU3QzdXd2emZWa0RHeDVSV0FNWWhIbzdFeGFycTJjdXIwVm1hZkw5ZGNsazczaURkV0cxek9aQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQb3lyUUdackIxVkRzVVZNbTc2WlpjbEtYclNqdS00cTM5U212T05Jb0FGN0dWcHFqeXc4WkRqR1hUdU1NT2wwSjZ3bUhXamZTSHFwMUNYWC1PTkRjQ3Q5UkVGVG5mSWlJOG8tcWxfNzZjRUZfNEd1N1drYkYtTFZ1YUxMMkZyZzRqSnk0c19na252TWJYZEFoVjQxcjk1SjFs?oc=5</t>
         </is>
       </c>
     </row>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Conflito no Oriente Médio dispara preço da ureia e afeta agro do Nordeste - Visão Agro</t>
+          <t>Conflito no Oriente Médio dispara preço da ureia e afeta agro do Nordeste - Movimento Econômico</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -8904,19 +8904,19 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQb3lyUUdackIxVkRzVVZNbTc2WlpjbEtYclNqdS00cTM5U212T05Jb0FGN0dWcHFqeXc4WkRqR1hUdU1NT2wwSjZ3bUhXamZTSHFwMUNYWC1PTkRjQ3Q5UkVGVG5mSWlJOG8tcWxfNzZjRUZfNEd1N1drYkYtTFZ1YUxMMkZyZzRqSnk0c19na252TWJYZEFoVjQxcjk1SjFs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQanphVHkycWR3c05tQ1VBYkl5b3pncV9sRGlGVmJvLVpOUUZRcWRvOFdXc1hhSVFqbDBZMlFNSEdVcnNCVGppQ2ZGMVl5WFN5SUJNWS1FLUVuRUpPRFh3VFZHdk54TndBaU4yZW0zQ3dVeWN3MWpFZTVpRUZudm81MlZTa1NoV2hxSWNxLWltS1piVXJwU3QzdXd2emZWa0RHeDVSV0FNWWhIbzdFeGFycTJjdXIwVm1hZkw5ZGNsazczaURkV0cxek9aQQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>calcario agricola</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Agricultores de Corupá já podem solicitar calcário pelo programa Terra Boa - OCP News</t>
+          <t>Prefeitura de Santa Cruz abre inscrições para distribuição gratuita de calcário a produtores rurais - Portal Arauto</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -8926,7 +8926,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOemxVOFYzVUJ5cXJKbGM5eVZQUkpkdEVXdk5DcVlpcnFMYWNYOXdNRzdUdTd0ZGFTeDNjNXZHOFUxemZXMUlKYmNJcHowaktZOFgxYmUyYjliQ1Nsc2ZMUVZ2VW5QU284VUI5bi1QdXpnRGg2aDJtSmZTNGFfa0V6Y2VOQnppSndEMW9UQWNERWdaVnJCb01lQ1dxOWd3UnFNaFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPZjd1TFdpbmV2Ui03ajM5WE9GaWNPUFZ3bVJJd3h3Q2JOdU05Q3Q2c0V1Y1FObVJFXzRTbWg3RVZXVzd5YUd6bXltMGEteUZ0WG5aUzZVckhwVVBBX3ppbDZ3S1NCZ1pnM1hHQlZwcDAxQ1pfa0FjNlFHOHRocHlvdzdvaTlON2lVdjJtaHRfRnpiRkFhcElYYmMtc1ZQTVlTQ3hFMnRLNTRlU0w1VjE2UW9ZUXpzcy02SHRDUGNLZDRhSDRqV3kyRUlPVWRKRjQwaFpnVHZR?oc=5</t>
         </is>
       </c>
     </row>
@@ -9043,12 +9043,12 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>Enxofre</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Justiça da Bahia suspende venda bilionária de mina de ouro entre canadenses e chineses - BPMoney</t>
+          <t>Fertilizantes puxam alta de preços de outros produtos químicos para indústria, diz IBGE - Valor Econômico</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -9058,7 +9058,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOV0F3R0dXNDk1eVUxZDJ3SF9QQUE0anFSeEkxOEp1a0dfMXRGZ2lRNTgwbDJsSlhJcjljMVJXS3ZxRDFEaUFUWFpYdmFXTE51YllrZDZSY2JMaGRWTTM2eFRxamhkd0hRbUFCVXY1LWpKbnJzXzNtN3JOMHB3dGdZU1Jicl9mTFdVN242eFl1OS1MLVVvdGtyN0tqU19iSHpmdzdKeDROMVltV0tzS0RfcjhFNVVqT1df?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOWjd4MFdUanZwVU1jUGhrbTVtempwWEFlRWt3RWZNWlNyQVp2RnRNY2lNTGtYTWFNbGRibVVObUlEVGZXNnZqN1pwYnN5Ul9DSlBjSTgyYmlzV3VseFVFbjlwdjRCM0UzekVyNVF2LUY0ZEpxanE2aFdWdnBuRWJDYTJYUnJjYVFyaUo3dUFtZ0tTS3Awd3BLTjBEcVZfNFpXVlpMSTdCSnc5YW9GNjNTT1poT1RteF9NMVNZUzRzUXdsSXlGX0JYZ0o0R2RDYWZZcXVRVnk3RXV1d9IB6AFBVV95cUxOc1gzenZmMHEwTzFZWkprT2FDd0hTT29qUmZrNFdpd2pxWC1hTXlCZ0YxZkNZdm1sR3E1LTdkWm44Vy1XZHZYT3lRaG5ZY01OdkVyUzZSUEczSFNpSk00YmlCM0N3ZUVvOHNZcy1rMExWNlZlM2VPUTZSRFc5QXhvY1dIdDhBSC1FOVdQUlVTa282Um94ZWtHRGF6SHNVcm1vSGl5NENxSy1TTTdTNkRqcUNKS1QzZTZtOVJtZ24xSDBEUFlibnY4WWtQN0d2aDNpZUJ5TDFpMVBrRHFOZTdPOXE0U1pITlpo?oc=5</t>
         </is>
       </c>
     </row>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>JUSTIÇA DA BAHIA SUSPENDE VENDA BILIONÁRIA DE MINA DE OURO - - Bahia Economica</t>
+          <t>Justiça da Bahia suspende venda bilionária de mina de ouro entre canadenses e chineses - BPMoney</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -9080,19 +9080,19 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVGFROXRCUlk3alljZnJUbDU2VnJqS1Y2ZHhheEM0UUV6bERYLWtHYmV2OUpMdF9MUGtDUlljUHg3eVBnamFZUk1GUEk2NTRfOV9YOFM5QndQcm5FTDh0NVlXNGVOVjR2S0kyaEMxTjI2RnBQZWtUMzlvdGlKRUs2QU1HR1pjQmFhYi1xV2hVZUg0bVpqNE54aDE5NGdNcWtDcWYySnRR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOV0F3R0dXNDk1eVUxZDJ3SF9QQUE0anFSeEkxOEp1a0dfMXRGZ2lRNTgwbDJsSlhJcjljMVJXS3ZxRDFEaUFUWFpYdmFXTE51YllrZDZSY2JMaGRWTTM2eFRxamhkd0hRbUFCVXY1LWpKbnJzXzNtN3JOMHB3dGdZU1Jicl9mTFdVN242eFl1OS1MLVVvdGtyN0tqU19iSHpmdzdKeDROMVltV0tzS0RfcjhFNVVqT1df?oc=5</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>Enxofre</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Fertilizantes puxam alta de preços de outros produtos químicos para indústria, diz IBGE - Valor Econômico</t>
+          <t>JUSTIÇA DA BAHIA SUSPENDE VENDA BILIONÁRIA DE MINA DE OURO - - Bahia Economica</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -9102,7 +9102,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOWjd4MFdUanZwVU1jUGhrbTVtempwWEFlRWt3RWZNWlNyQVp2RnRNY2lNTGtYTWFNbGRibVVObUlEVGZXNnZqN1pwYnN5Ul9DSlBjSTgyYmlzV3VseFVFbjlwdjRCM0UzekVyNVF2LUY0ZEpxanE2aFdWdnBuRWJDYTJYUnJjYVFyaUo3dUFtZ0tTS3Awd3BLTjBEcVZfNFpXVlpMSTdCSnc5YW9GNjNTT1poT1RteF9NMVNZUzRzUXdsSXlGX0JYZ0o0R2RDYWZZcXVRVnk3RXV1d9IB6AFBVV95cUxOc1gzenZmMHEwTzFZWkprT2FDd0hTT29qUmZrNFdpd2pxWC1hTXlCZ0YxZkNZdm1sR3E1LTdkWm44Vy1XZHZYT3lRaG5ZY01OdkVyUzZSUEczSFNpSk00YmlCM0N3ZUVvOHNZcy1rMExWNlZlM2VPUTZSRFc5QXhvY1dIdDhBSC1FOVdQUlVTa282Um94ZWtHRGF6SHNVcm1vSGl5NENxSy1TTTdTNkRqcUNKS1QzZTZtOVJtZ24xSDBEUFlibnY4WWtQN0d2aDNpZUJ5TDFpMVBrRHFOZTdPOXE0U1pITlpo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVGFROXRCUlk3alljZnJUbDU2VnJqS1Y2ZHhheEM0UUV6bERYLWtHYmV2OUpMdF9MUGtDUlljUHg3eVBnamFZUk1GUEk2NTRfOV9YOFM5QndQcm5FTDh0NVlXNGVOVjR2S0kyaEMxTjI2RnBQZWtUMzlvdGlKRUs2QU1HR1pjQmFhYi1xV2hVZUg0bVpqNE54aDE5NGdNcWtDcWYySnRR?oc=5</t>
         </is>
       </c>
     </row>
@@ -9175,12 +9175,12 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>Ureia</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Justiça da Bahia suspende negócio bilionário de minas de ouro entre canadenses e chineses - Folha de S.Paulo</t>
+          <t>Ureia dispara e mercado reduz negociações em meio à guerra do Irã - CNN Brasil</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -9190,19 +9190,19 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQYWNULVM2dHlzUUd3UDNyYUp6SDZrdGs4VjJSdUllMlJYQWFMdkJJblVjaUxfSGpTNXJ6S3gxOENtQTl3clNIeG56VVpVZkdWNWs5a05DWE04N3ZyZWJySzFRZEZESVhiVEcyMHZSWUVETVRaOUtnWlMwLWNjUXY0Ti11ZjF0UXJ0ODNXcG5lYldORXJuU2JQX0xaTHJBRGxKVWk5QmFwbVd2cUc5Z2wtSk5oNC1vV3F1U0U1WkJGMEhDRHNWVVpBNmltMVBzUTdnV0Rqbm8tcFTSAd4BQVVfeXFMTlE5cnFkMU1MWjZsaHVCdkxKM3JmOURJV25ZSUh3LU1xc2RsYmZhTzNOaEZjRGlBeTg5RFRndzE5X2h2cGxLb3BQYXY0aEc4b0dkbjh4VzdLbmRudXlYUEhwU1pnZVRGODRvY0ltTEsxWkE3OW15ZmZNOTZYdHRuWXN0ZzJMMnppM3h1WnBHSW5XM09QVVdBWlRBZFdzc0o3eDhvc3BUdW05VmhIRWl2RVVaUFRtRGVCWG1iSlFTTkpBTGwyS2RRc1Q4aDdjSFEwbzBsOTJTbU5lN3g3SGd3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYi1XSk5GWVlFUFlZVzR2UXlURVpUajhfTjd5c0tBUUVqVUkxQy1OVFNfc3M3eDJWdndqSzJSZEJYRTdlTXI2ejdGbmlYQ1pGUmlkMVlJRGtIbmVZeDdNLXM2YS0xajQxc0p1b2pKYjJmT2Z4TGxBU0VoUTAxRlFuYkZNUWVGZWsybUdXLUxrQzNvcFRnZnNLQkxjQTBLTW5mMmc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>Ureia</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Ureia dispara e mercado reduz negociações em meio à guerra do Irã - CNN Brasil</t>
+          <t>Justiça da Bahia suspende negócio bilionário de minas de ouro entre canadenses e chineses - Folha de S.Paulo</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -9212,7 +9212,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNYi1XSk5GWVlFUFlZVzR2UXlURVpUajhfTjd5c0tBUUVqVUkxQy1OVFNfc3M3eDJWdndqSzJSZEJYRTdlTXI2ejdGbmlYQ1pGUmlkMVlJRGtIbmVZeDdNLXM2YS0xajQxc0p1b2pKYjJmT2Z4TGxBU0VoUTAxRlFuYkZNUWVGZWsybUdXLUxrQzNvcFRnZnNLQkxjQTBLTW5mMmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQYWNULVM2dHlzUUd3UDNyYUp6SDZrdGs4VjJSdUllMlJYQWFMdkJJblVjaUxfSGpTNXJ6S3gxOENtQTl3clNIeG56VVpVZkdWNWs5a05DWE04N3ZyZWJySzFRZEZESVhiVEcyMHZSWUVETVRaOUtnWlMwLWNjUXY0Ti11ZjF0UXJ0ODNXcG5lYldORXJuU2JQX0xaTHJBRGxKVWk5QmFwbVd2cUc5Z2wtSk5oNC1vV3F1U0U1WkJGMEhDRHNWVVpBNmltMVBzUTdnV0Rqbm8tcFTSAd4BQVVfeXFMTlE5cnFkMU1MWjZsaHVCdkxKM3JmOURJV25ZSUh3LU1xc2RsYmZhTzNOaEZjRGlBeTg5RFRndzE5X2h2cGxLb3BQYXY0aEc4b0dkbjh4VzdLbmRudXlYUEhwU1pnZVRGODRvY0ltTEsxWkE3OW15ZmZNOTZYdHRuWXN0ZzJMMnppM3h1WnBHSW5XM09QVVdBWlRBZFdzc0o3eDhvc3BUdW05VmhIRWl2RVVaUFRtRGVCWG1iSlFTTkpBTGwyS2RRc1Q4aDdjSFEwbzBsOTJTbU5lN3g3SGd3?oc=5</t>
         </is>
       </c>
     </row>
@@ -9329,12 +9329,12 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>corretivo de solo</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>CBPM contesta venda de ativo de metais preciosos da Equinox na Bahia para chinesa CMOC - Bloomberg Línea Brasil</t>
+          <t>Custos da safra 2026/27 variam em MT; algodão e soja recuam, milho sobe 7,19% - Nativa News</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -9344,19 +9344,19 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPWXgwYnhxbzhZaGZOZHd3bkxXbUhQa1lOZWxiVFBfVWp2QjZWMW5UVnB3U2d1ZDZfSlRpSG9MSVJlODlhX3VjZ3NERE42OVpnSG9WdHhXdE95Umh0YjBhekpSTkppQ21oWjNEeWFUUkhaRVlIN01HekxWM1RpbWc0dDBjeUxHQU9GZnRTVl9COHFIWE1CRlkzMnFCYTNvRU9BR1NYSGptRzRHVEc2akd2Tkk1UmdiTklhX3p0UEFCOUsxYlhSMkNwWnlR0gHeAUFVX3lxTE1zOExaOFF5OWI5VUdVQXFXZG04cDVEd0NVS1B0ejh0R1UwTFQ2QUwtRDdfR2RjblhBREhmbFFYTVFQLW9zT3R0SXJyVmZXZkl4X1h1bUk3TlBhMTlCNzlIQUJEODhBc2RZeEx1cXBKR2xEeHl4TlN4Z3FnLTVSSG96b0lqbF8zRU9yVlROZ3JwR0F3UUlrMlpiUlNaRTdLWE1jZTJ6N3JyTDBMN3E0cmJlMzNxZi1rbGlBbzBPQkFhczdFRWtXZGRaWllFQ281YWZOWkxYMlpHU3FzSHpvUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWnBBY2Uwc2FseU4zdDQ2aVhkdWdVNXJGRDZJR0tTZ0Y1UWZSREc2ZDVySi1rMndqSkMyWEgyVzVQTGlOSmhKTEgzWXRfNm5zd280WW5BUFhwdFNYemdvc1dqX095TG9kQ3dNSmU3VmdnNFJkMjNBeHZSZEprSzBOVHhLSWEzbDcyZUNnbnY1U0xpLVZTNVBHdEVFMDRVMVlySU1XNHJZQWdwbVJ3QkVuZ2lMWQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>calcario agricola</t>
+          <t>Ical</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>CRA vai analisar redução de alíquota sobre o calcário de uso agrícola - Senado Federal</t>
+          <t>Um dia após ser nomeado, presidente interino do Peru é intimado por 'apropriação indébita' - Opera Mundi</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -9366,19 +9366,19 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNeWVQYnFWb2NCX2FFS3ltNHh0enBBZFVrS0tCSVJJb3ZBQ1FldnRaUVNQNF91WXN1V0ZNd1JENkVjVzBmVUNwS2RDTTZ1eW53WndKTDdHVWtUUmE1UDktTUsxSjdYMzBiMzJkV3B1aWY0d2VmczFJeUl6ZlpjRXd0VlFZUTlIN2tHQnlrRXlYNzZ4Rk5ZNThGWGtaZV9BSVV5SUVFNS1yREwweS1aQVMwOS1yZm5yQThBaDNVSnZKb1VWV1dO?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPay1sZXVrRnVUZlJFNWU0cGtSb1lULVI5R3FFQWhXdTJhblFWS1NwcHh2aFdRX1lYV2pfakFlU0FyTTVqZE15TmRHcGZPYmJJLXZOSHRmR2lCM282NWM5WEhqR2ppRE1kMHhELVRmX0lZb1FXeHlIRFFRT1VXSnM4NjVfNkEzV1MxMlJaZTVNYTA4NmhnZkFBbTJiODNxWVFRYjhFa1ZGamhVV2oxdzhyendSZVRUd0VoeXFOemZOX2RpSHVIbHlJVDliTmJlQQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>corretivo de solo</t>
+          <t>calcario agricola</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Custos da safra 2026/27 variam em MT; algodão e soja recuam, milho sobe 7,19% - Nativa News</t>
+          <t>CRA vai analisar redução de alíquota sobre o calcário de uso agrícola - Senado Federal</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -9388,7 +9388,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWnBBY2Uwc2FseU4zdDQ2aVhkdWdVNXJGRDZJR0tTZ0Y1UWZSREc2ZDVySi1rMndqSkMyWEgyVzVQTGlOSmhKTEgzWXRfNm5zd280WW5BUFhwdFNYemdvc1dqX095TG9kQ3dNSmU3VmdnNFJkMjNBeHZSZEprSzBOVHhLSWEzbDcyZUNnbnY1U0xpLVZTNVBHdEVFMDRVMVlySU1XNHJZQWdwbVJ3QkVuZ2lMWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNeWVQYnFWb2NCX2FFS3ltNHh0enBBZFVrS0tCSVJJb3ZBQ1FldnRaUVNQNF91WXN1V0ZNd1JENkVjVzBmVUNwS2RDTTZ1eW53WndKTDdHVWtUUmE1UDktTUsxSjdYMzBiMzJkV3B1aWY0d2VmczFJeUl6ZlpjRXd0VlFZUTlIN2tHQnlrRXlYNzZ4Rk5ZNThGWGtaZV9BSVV5SUVFNS1yREwweS1aQVMwOS1yZm5yQThBaDNVSnZKb1VWV1dO?oc=5</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Um dia após ser nomeado, presidente interino do Peru é intimado por 'apropriação indébita' - Opera Mundi</t>
+          <t>Novo presidente de esquerda do Peru será julgado por corrupção - Gazeta do Povo</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -9410,19 +9410,19 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPay1sZXVrRnVUZlJFNWU0cGtSb1lULVI5R3FFQWhXdTJhblFWS1NwcHh2aFdRX1lYV2pfakFlU0FyTTVqZE15TmRHcGZPYmJJLXZOSHRmR2lCM282NWM5WEhqR2ppRE1kMHhELVRmX0lZb1FXeHlIRFFRT1VXSnM4NjVfNkEzV1MxMlJaZTVNYTA4NmhnZkFBbTJiODNxWVFRYjhFa1ZGamhVV2oxdzhyendSZVRUd0VoeXFOemZOX2RpSHVIbHlJVDliTmJlQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOWGxsYkZLamdUbENJS0dQVjF2T18xODhVYWNfcHFNZGpJOVE1Q3BWSER5V1R0NXRvalpObHdzcmF0TEMteFJpRjNrV2gxeUVPU2NkSUpjS3Rta2xfNkxkZURnSnhOeDJvY0Q1Q0c1Z1JEZVRwc1RhS1RDX1pLUWVVZEhpSXVRQzR3X2xETHVTVEZvQnZmV3JNblBJYmVHNDgzV1J3VndMUjlPSFdnc1Y2T1RaRGU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>Ical</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Novo presidente de esquerda do Peru será julgado por corrupção - Gazeta do Povo</t>
+          <t>CBPM contesta venda de ativo de metais preciosos da Equinox na Bahia para chinesa CMOC - Bloomberg Línea Brasil</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOWGxsYkZLamdUbENJS0dQVjF2T18xODhVYWNfcHFNZGpJOVE1Q3BWSER5V1R0NXRvalpObHdzcmF0TEMteFJpRjNrV2gxeUVPU2NkSUpjS3Rta2xfNkxkZURnSnhOeDJvY0Q1Q0c1Z1JEZVRwc1RhS1RDX1pLUWVVZEhpSXVRQzR3X2xETHVTVEZvQnZmV3JNblBJYmVHNDgzV1J3VndMUjlPSFdnc1Y2T1RaRGU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPWXgwYnhxbzhZaGZOZHd3bkxXbUhQa1lOZWxiVFBfVWp2QjZWMW5UVnB3U2d1ZDZfSlRpSG9MSVJlODlhX3VjZ3NERE42OVpnSG9WdHhXdE95Umh0YjBhekpSTkppQ21oWjNEeWFUUkhaRVlIN01HekxWM1RpbWc0dDBjeUxHQU9GZnRTVl9COHFIWE1CRlkzMnFCYTNvRU9BR1NYSGptRzRHVEc2akd2Tkk1UmdiTklhX3p0UEFCOUsxYlhSMkNwWnlR0gHeAUFVX3lxTE1zOExaOFF5OWI5VUdVQXFXZG04cDVEd0NVS1B0ejh0R1UwTFQ2QUwtRDdfR2RjblhBREhmbFFYTVFQLW9zT3R0SXJyVmZXZkl4X1h1bUk3TlBhMTlCNzlIQUJEODhBc2RZeEx1cXBKR2xEeHl4TlN4Z3FnLTVSSG96b0lqbF8zRU9yVlROZ3JwR0F3UUlrMlpiUlNaRTdLWE1jZTJ6N3JyTDBMN3E0cmJlMzNxZi1rbGlBbzBPQkFhczdFRWtXZGRaWllFQ281YWZOWkxYMlpHU3FzSHpvUQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Negócio bilionário de ouro vira alvo de disputa entre estatal baiana e mineradoras internacionais - G1</t>
+          <t>Estatal da Bahia tenta anular negócio bilionário de ouro entre canadenses e chineses - Folha de S.Paulo</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -9630,7 +9630,7 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNalRrbEVWVGYxMWtjSUJVREZfM254QjYwM3BSLUdlaWlhb2QyMERZcHBrajRVLUtlYmZieXJiUnRpM1NENTdtS0ZKc3R0am45SmNkSTNfVjJ5akMyM00xdC1TYTlULXYyVFEzMF9OSWFNRF9yM0cwVGoyaFdZcmI2QnA1MTRoeE5OeU9pSXNlY2JhLUhXQnMzUzMtY3dmQdIBrAFBVV95cUxOYy1aYldiLVZyWVd0Q1ZMS05VR1pHZVJLb1NqZUFDa1dQR3NRZ2x6WEtSX3dFbUlQalBBa0FmWkNrUVZHQ2lxVUR3T2pSa2s5WVBOQjhFNEMtTW43MmxjM3FoaUxLak5yY2EzaTk1aXBWOVhBUjNLRjY1M2d0U19sekxZQzJLcnlnbDBzd2M5TXdzY2tnYkJYLWxIem5keG4yVzNHcDVDZHdyaGcx?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPVUlXUktSbEdjOC1NTzE1d0ZIVmNad0RVMDE5VlpBWGh0X0VkZkZqSTFuR2EwNVBpNHVnOEtuUWdaTF9DeGRIV0FYNW01M3E5c1ViZVgtT1h1VnVhVFRoZnVRNDNNbm9fVG5FMmVGQTZiU2w4UmlOTXVwRnZIaWhzNjNXTXpEcHRRMGZ3ZmYxazByT01MZXJiRjhLajh6X1VEdjhILUtaZllZa3BRZUZVcGJXTmFCRjF4bDRWWE5FeUQxYlNabF9mMnlvMER1akRaclHSAdcBQVVfeXFMTmFLYWxidHM1czVENlhQTzdaSlZmSUZmT3M4LXZtV2k3ZXBranlIb2F3clBQQ3lIaWpIVC1mNXoxZUYzaVc1cDFLbUR2R0VydTNsZUktcWVKRkZqeGp1TEhKUTN1Z3JpeG9wZjItdzJyanlUTW14WE1yVnE5VmNUa3FVWXNudnNzeEdyUEIxbklVSldyRzVoR2tMcTVIQXEyTm41ZVRMOUpsVmJfdVBLc1RscS1zY1JPYW8tTUlmODdRbm8xMmF5NWV3clZqdURDTTMzVURncGM?oc=5</t>
         </is>
       </c>
     </row>
@@ -9642,7 +9642,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Estatal da Bahia tenta anular negócio bilionário de ouro entre canadenses e chineses - Folha de S.Paulo</t>
+          <t>Negócio bilionário de ouro vira alvo de disputa entre estatal baiana e mineradoras internacionais - G1</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -9652,7 +9652,7 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPVUlXUktSbEdjOC1NTzE1d0ZIVmNad0RVMDE5VlpBWGh0X0VkZkZqSTFuR2EwNVBpNHVnOEtuUWdaTF9DeGRIV0FYNW01M3E5c1ViZVgtT1h1VnVhVFRoZnVRNDNNbm9fVG5FMmVGQTZiU2w4UmlOTXVwRnZIaWhzNjNXTXpEcHRRMGZ3ZmYxazByT01MZXJiRjhLajh6X1VEdjhILUtaZllZa3BRZUZVcGJXTmFCRjF4bDRWWE5FeUQxYlNabF9mMnlvMER1akRaclHSAdcBQVVfeXFMTmFLYWxidHM1czVENlhQTzdaSlZmSUZmT3M4LXZtV2k3ZXBranlIb2F3clBQQ3lIaWpIVC1mNXoxZUYzaVc1cDFLbUR2R0VydTNsZUktcWVKRkZqeGp1TEhKUTN1Z3JpeG9wZjItdzJyanlUTW14WE1yVnE5VmNUa3FVWXNudnNzeEdyUEIxbklVSldyRzVoR2tMcTVIQXEyTm41ZVRMOUpsVmJfdVBLc1RscS1zY1JPYW8tTUlmODdRbm8xMmF5NWV3clZqdURDTTMzVURncGM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNalRrbEVWVGYxMWtjSUJVREZfM254QjYwM3BSLUdlaWlhb2QyMERZcHBrajRVLUtlYmZieXJiUnRpM1NENTdtS0ZKc3R0am45SmNkSTNfVjJ5akMyM00xdC1TYTlULXYyVFEzMF9OSWFNRF9yM0cwVGoyaFdZcmI2QnA1MTRoeE5OeU9pSXNlY2JhLUhXQnMzUzMtY3dmQdIBrAFBVV95cUxOYy1aYldiLVZyWVd0Q1ZMS05VR1pHZVJLb1NqZUFDa1dQR3NRZ2x6WEtSX3dFbUlQalBBa0FmWkNrUVZHQ2lxVUR3T2pSa2s5WVBOQjhFNEMtTW43MmxjM3FoaUxLak5yY2EzaTk1aXBWOVhBUjNLRjY1M2d0U19sekxZQzJLcnlnbDBzd2M5TXdzY2tnYkJYLWxIem5keG4yVzNHcDVDZHdyaGcx?oc=5</t>
         </is>
       </c>
     </row>
@@ -9681,12 +9681,12 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>calcario</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>CRA deve votar redução de alíquota sobre calcário nesta quarta - Senado Federal</t>
+          <t>CBPM barra venda de US$ 1 bi da Equinox Gold - BPMoney</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -9696,19 +9696,19 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOeTNjVGxONFNqaV92QmFjbHM5a2VHMHgwNE9sNkV1MzNBNnowdjFiNjhjdm9oeFFsNWdxX3p0Y0xRMDRJMmNRdDV6eEtZOFNwU3V2RURWc2VsMTlVMEZLcXN1aGJ6ZlNMa0hxTDF3ZDhlMTdMSXNCTmw2bGNtZVBEakhuY0NBZjVrUEdUNXFfUk1TZjM1U2hERkl1Y1BaSlZ0QmJVdnY1V1pVSXd2NGFSbnR1ZkdaUDBWREtN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFBWblRQRGhkRGVieU40amJOckdTQncyS21zQno3b0hlNmQxQU5ZTkRMTDc2clI3SEs0ckFJT3BMeFY3M09Zd0hNb0hMU2tOWjlMSldqTzJ3cmR2a1VlZHNsMHBEYUZwWWkxbnRsUFVZVWJsOURCMjZTUHdHaUJEZ0k?oc=5</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>calcario</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>CBPM barra venda de US$ 1 bi da Equinox Gold - BPMoney</t>
+          <t>CRA deve votar redução de alíquota sobre calcário nesta quarta - Senado Federal</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFBWblRQRGhkRGVieU40amJOckdTQncyS21zQno3b0hlNmQxQU5ZTkRMTDc2clI3SEs0ckFJT3BMeFY3M09Zd0hNb0hMU2tOWjlMSldqTzJ3cmR2a1VlZHNsMHBEYUZwWWkxbnRsUFVZVWJsOURCMjZTUHdHaUJEZ0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOeTNjVGxONFNqaV92QmFjbHM5a2VHMHgwNE9sNkV1MzNBNnowdjFiNjhjdm9oeFFsNWdxX3p0Y0xRMDRJMmNRdDV6eEtZOFNwU3V2RURWc2VsMTlVMEZLcXN1aGJ6ZlNMa0hxTDF3ZDhlMTdMSXNCTmw2bGNtZVBEakhuY0NBZjVrUEdUNXFfUk1TZjM1U2hERkl1Y1BaSlZ0QmJVdnY1V1pVSXd2NGFSbnR1ZkdaUDBWREtN?oc=5</t>
         </is>
       </c>
     </row>
@@ -10143,12 +10143,12 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>corretivo de solo</t>
+          <t>Cal Cruzeiro</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>CSN testa aplicação agrícola de agregado siderúrgico em lavouras de café em Minas Gerais - A Voz da Cidade</t>
+          <t>Saída de Gabigol do Cruzeiro é consenso; destino passa a ser a dúvida - DeFato.com</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -10158,19 +10158,19 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNUF9QWHBiMF9mc2pNUU1Vb2xxdEJrZmlvdGRiUlJWWXFEY0U4M3p4YWlCT1ZxeEhOY0trQ0RXcXk1NFg4SlJNSjFwQWNneFhjeWV2dkVIMlZZeVVGQ2xqaTFZT0VBdWJRaWxPOURBczU3NUFpNFV4RVJXTXRKLWRELXhoLVVkbE1pNklBVWZwTkJFbGJLVVlKN1hNS2xrU2RZMmxBUHd0Z240SmVCaldtWjEwTmh5QTli?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNa2tNM01IRUF0a3VjME5PaDlsRWd5cW5OVW90a1J1SmxVZm5sbC1fdDZkVjZRcm1TYTdhRWs1RTJuSzJhUEhPYXpvWmhqcUExdGV5VkNPaXZLQmVvdzh0VTFraG9QbmZsZ3VlbFpXSThWWTNLLTdsZkNQNEFSLVhUcjQ5U1VIQ1BGSXZYd2tTLWV4SS1SWEl4bGdLal8tc0lz?oc=5</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>Cal Cruzeiro</t>
+          <t>corretivo de solo</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>Saída de Gabigol do Cruzeiro é consenso; destino passa a ser a dúvida - DeFato.com</t>
+          <t>CSN testa aplicação agrícola de agregado siderúrgico em lavouras de café em Minas Gerais - A Voz da Cidade</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
@@ -10180,7 +10180,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNa2tNM01IRUF0a3VjME5PaDlsRWd5cW5OVW90a1J1SmxVZm5sbC1fdDZkVjZRcm1TYTdhRWs1RTJuSzJhUEhPYXpvWmhqcUExdGV5VkNPaXZLQmVvdzh0VTFraG9QbmZsZ3VlbFpXSThWWTNLLTdsZkNQNEFSLVhUcjQ5U1VIQ1BGSXZYd2tTLWV4SS1SWEl4bGdLal8tc0lz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNUF9QWHBiMF9mc2pNUU1Vb2xxdEJrZmlvdGRiUlJWWXFEY0U4M3p4YWlCT1ZxeEhOY0trQ0RXcXk1NFg4SlJNSjFwQWNneFhjeWV2dkVIMlZZeVVGQ2xqaTFZT0VBdWJRaWxPOURBczU3NUFpNFV4RVJXTXRKLWRELXhoLVVkbE1pNklBVWZwTkJFbGJLVVlKN1hNS2xrU2RZMmxBUHd0Z240SmVCaldtWjEwTmh5QTli?oc=5</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>EMPRESA CHINESA COMPRA MINAS DE OURO NO BRASIL E VAI ASSUMIR A MINERAÇÃO DE OURO NA BAHIA - - Bahia Economica</t>
+          <t>CMOC entra no ouro no Brasil e compra minas da Equinox por até US$ 1,015 bi - Estado de Minas</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNZXVMTUFYSkUwMnlmS3lpZlU2VkczaWFyX1JuRy1FSGhFUVkzb2lpU0I2b19LM0VMSHBDelUwbU14Uk5lVVRSVGFhUGxOSGhZbEtyMG40NUZ5dndaelVvZTZiUktxb2taa2M0czRmRllWTWZ0djYzSDMxa1JZR3FCMlN0N2RsNEdBSl9oeTZ5STVENTVzY2ZSdGtIeU1Fb3o0VWFuNksxV3Y1UWE5b3VwWkEwUWZjdHBJS1BVNGJMVmpLbUItWU1ZcFdFYnczM25QZ1lj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNYmxtd1NMbXd3d3lRSnhVZF9GLXd3a0JfMHJhel81U1BQTFV0bl9JUTBPMFdCVVNFZFF4TjN4NWEwa254cV9pdFl0M1Y1UGt3VHhrLXBxTy1od29NaTZUc2ZvdkZva3YwVklDdmFxcVdyXzU1Yy0wT2Jkb3B6cTFIdFplZTBNLXpvLVJSSll2cFBoelpUUlFjNDc5WWc1WnI4ZUdjVWlKcWhLOWctM1JtMlA5QXIyWDllY0RScDJOYV8zYzBvdW5rVVNRalg5YldIOGdz0gHYAUFVX3lxTFBCd3RLUWlLUm4wZnlCUFVMdE05RXUzcVNXTXlEYnZIem9wbG5TaWJPVmJjem5kNUtQSFpjWFRfdm1jRHdVMUlhb1p0Z0NHeE9yVnA2SjdaOWtGRjNWVENxbEZQcWtQVFZHUmpadUg4VVZiUlUyOEQ0NDhqaXZZSi1LWGM5TG5OaEhGcExFQkdtQTA5b1AwdDZTbW9SM1ZyZzN3UU1YWUJTUDhTaW5HMlJ6clloeUthcnJ5dDRjUXJITXNSUXR1VzVBdm5XS1VQX0lPQk11eGU4QQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>NEGÓCIOS | A incursão chinesa no setor mineral brasileiro e os desafios do capital nacional - Brasil Mineral</t>
+          <t>Equinox Gold vende minas no Brasil à chinesa CMOC por US$ 1 bilhão - Jornal Portuário</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -10224,7 +10224,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNeEczVHluQ0N4cDRucDc3SWpBNzV1SGdHdUJ0RUg1ZFdCQlYzZGlIM0RZaXd6bHJ3b2tUZjgzWll1dGRiOFN3S09kM3Z3aFItTmkyR0YyRkMtRUZyMGFENUxXOGpCbEdURHlPNVM2d0NJendkdXd1aWtpVUZPSVhtMFFxWEJWMlRzQkx5LW4zUEF3ajRUVU1QVEYtSUFxOHdXa0dLeE1yb18yNnlRYzRwNlBNOXBmdk5vd3B3Rmx5VQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOejlYQmU1SzhnRGtFMFJKWU9sNFZmM01temlpNFdjTVRTQzdqeFFwM0hZUzlIVlJZa2pGaGo1UVdmTXd0dGRtX041d1ptUVdvUmNfTnNlM2ppdmFEMUtlMlZVNzBvWlZyaVlGZUpOV19CR0FKeXFKU21yWEo4Q0RoMnEzdHV2Zk1ZR0prQzRnQzNzOGR1OGwwQkFYM2hwemo0emFXQ0tkUmR6a3NnYWc?oc=5</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>CMOC entra no ouro no Brasil e compra minas da Equinox por até US$ 1,015 bi - Estado de Minas</t>
+          <t>NEGÓCIOS | A incursão chinesa no setor mineral brasileiro e os desafios do capital nacional - Brasil Mineral</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNYmxtd1NMbXd3d3lRSnhVZF9GLXd3a0JfMHJhel81U1BQTFV0bl9JUTBPMFdCVVNFZFF4TjN4NWEwa254cV9pdFl0M1Y1UGt3VHhrLXBxTy1od29NaTZUc2ZvdkZva3YwVklDdmFxcVdyXzU1Yy0wT2Jkb3B6cTFIdFplZTBNLXpvLVJSSll2cFBoelpUUlFjNDc5WWc1WnI4ZUdjVWlKcWhLOWctM1JtMlA5QXIyWDllY0RScDJOYV8zYzBvdW5rVVNRalg5YldIOGdz0gHYAUFVX3lxTFBCd3RLUWlLUm4wZnlCUFVMdE05RXUzcVNXTXlEYnZIem9wbG5TaWJPVmJjem5kNUtQSFpjWFRfdm1jRHdVMUlhb1p0Z0NHeE9yVnA2SjdaOWtGRjNWVENxbEZQcWtQVFZHUmpadUg4VVZiUlUyOEQ0NDhqaXZZSi1LWGM5TG5OaEhGcExFQkdtQTA5b1AwdDZTbW9SM1ZyZzN3UU1YWUJTUDhTaW5HMlJ6clloeUthcnJ5dDRjUXJITXNSUXR1VzVBdm5XS1VQX0lPQk11eGU4QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNeEczVHluQ0N4cDRucDc3SWpBNzV1SGdHdUJ0RUg1ZFdCQlYzZGlIM0RZaXd6bHJ3b2tUZjgzWll1dGRiOFN3S09kM3Z3aFItTmkyR0YyRkMtRUZyMGFENUxXOGpCbEdURHlPNVM2d0NJendkdXd1aWtpVUZPSVhtMFFxWEJWMlRzQkx5LW4zUEF3ajRUVU1QVEYtSUFxOHdXa0dLeE1yb18yNnlRYzRwNlBNOXBmdk5vd3B3Rmx5VQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10280,7 +10280,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>Equinox Gold vende minas no Brasil à chinesa CMOC por US$ 1 bilhão - Jornal Portuário</t>
+          <t>EMPRESA CHINESA COMPRA MINAS DE OURO NO BRASIL E VAI ASSUMIR A MINERAÇÃO DE OURO NA BAHIA - - Bahia Economica</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -10290,7 +10290,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOejlYQmU1SzhnRGtFMFJKWU9sNFZmM01temlpNFdjTVRTQzdqeFFwM0hZUzlIVlJZa2pGaGo1UVdmTXd0dGRtX041d1ptUVdvUmNfTnNlM2ppdmFEMUtlMlZVNzBvWlZyaVlGZUpOV19CR0FKeXFKU21yWEo4Q0RoMnEzdHV2Zk1ZR0prQzRnQzNzOGR1OGwwQkFYM2hwemo0emFXQ0tkUmR6a3NnYWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNZXVMTUFYSkUwMnlmS3lpZlU2VkczaWFyX1JuRy1FSGhFUVkzb2lpU0I2b19LM0VMSHBDelUwbU14Uk5lVVRSVGFhUGxOSGhZbEtyMG40NUZ5dndaelVvZTZiUktxb2taa2M0czRmRllWTWZ0djYzSDMxa1JZR3FCMlN0N2RsNEdBSl9oeTZ5STVENTVzY2ZSdGtIeU1Fb3o0VWFuNksxV3Y1UWE5b3VwWkEwUWZjdHBJS1BVNGJMVmpLbUItWU1ZcFdFYnczM25QZ1lj?oc=5</t>
         </is>
       </c>
     </row>
@@ -10302,7 +10302,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>Equinox Gold vende minas de ouro no Brasil para CMOC, da China, por US$ 1 bilhão - Estadão</t>
+          <t>Chinesa CMOC compra operações da Equinox e produzirá ouro no Brasil - Valor Econômico</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -10312,7 +10312,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOb1F1OGg3dHNSNEkwNU5vZG44NVpRZThWZG9MVXpkbU5HUFJnSFJsVFhYdndGOTYtRDVaWV9pcTdFUExMLTRqWlhsNXI5OFBPdEJBWE9EZ3NNaDctVUhRaUNpcWhrMWVxM3dOTWdQSTYxODRQTllKMjF2b0s2QzJhWDhERUFTTEFjWnFEdkVKcnVvQmFxNWhlbFF5aF9LY2hWVWlLTFo2aUlMUUttQnRqaWd1WmVhenp2M2fSAb8BQVVfeXFMUHAwZnJHMlZkOXpSbkRRTVlfejYwRExQeVMxZHlxWmRRRGNOOFdrTXFWNkZKLTJ1bXlVV0N6Z0xhMHR6dUVocHF2Z0tLQ3YxVENvR3VacGhpQUlXbDJqRlM1VldCcTdNWHItSDB2cXJhblhBM29zcjdQZlZnOVNCd0RYQmZ5MHhtS0xEY2ZTSjBCS05RTm1kQWl6MWw4QTU2RnhLZm5WTWtFVkg5UFh1OGdZdDNIVWE5ejRCQ3dNeUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxNdjJLdXR0TWF1WVRBWGpwZW5vUlAtZk9scmFlMUxKbWxpcUVKZ2ZkNGJqZXhCVENIRVpaRlBPWE9ycnJteDJnbW1WcmZUVjVJOG9DTjF0andnXzMweFV0anRSLXdjVUllZ3JvYUNLU1U3SnFoRWx4Z21OVnFNQ05nWDZaVVRBQnoxMFVSYm5PQ3AyZlVqdmpabzNCY25qZVE0VkI4NGlKVGEzd3RncWNtX0swakhzYjh5WUktLUx2bjdrQkHSAdIBQVVfeXFMTndraVAxVThDT0d6d0xTbVdRa25WdENfanhibkVOamNHaVFMR3VJQWp4b1RiVmFaRXFGQmIwLUZHVTlTdHcxWnZhZERhRWRyRmhBUFlmakVxRHYtZVJNNW5OS1JuZ0xyVXdWVFVSdDU3NmN5MWt4Zmw2R01fR2ZMNG5fVDB0LVNtRENfdlNZS2hmSGg0a2xES1p4aDdzMk1RODRWaHBjVVE0MXNLcWRfMGJuSHZ2SVhZcHcyZnQ5eVN6UXhkd2ZhZGdzeDc0UzRFUkln?oc=5</t>
         </is>
       </c>
     </row>
@@ -10324,7 +10324,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>China CMOC compra quatro minas de ouro no Brasil por 863 milhões de euros - RTP</t>
+          <t>Equinox Gold vende minas de ouro no Brasil para CMOC, da China, por US$ 1 bilhão - Estadão</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQV0FjeGVtTGVqd2VhNU5fanJxQVlOSWI5ckFnZTFhLVgtdjZQNXlzUUFIYVJhS285THFzZjRiNUw4QnJJcENRVmtQT3l0NUVzR3c0UzlnT3I0anItNXprX0Qzd1R2b000V3Bya3NsSVVtMi16U2JQaERkcFZQRVFxalA1cTByWEVjTzZKQjc5RHZrdWdncy1zWEh6ZURSTFJXWG1HdlE1cV9iLXpMRG1sVWl4R0ltNDF5VHVJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOb1F1OGg3dHNSNEkwNU5vZG44NVpRZThWZG9MVXpkbU5HUFJnSFJsVFhYdndGOTYtRDVaWV9pcTdFUExMLTRqWlhsNXI5OFBPdEJBWE9EZ3NNaDctVUhRaUNpcWhrMWVxM3dOTWdQSTYxODRQTllKMjF2b0s2QzJhWDhERUFTTEFjWnFEdkVKcnVvQmFxNWhlbFF5aF9LY2hWVWlLTFo2aUlMUUttQnRqaWd1WmVhenp2M2fSAb8BQVVfeXFMUHAwZnJHMlZkOXpSbkRRTVlfejYwRExQeVMxZHlxWmRRRGNOOFdrTXFWNkZKLTJ1bXlVV0N6Z0xhMHR6dUVocHF2Z0tLQ3YxVENvR3VacGhpQUlXbDJqRlM1VldCcTdNWHItSDB2cXJhblhBM29zcjdQZlZnOVNCd0RYQmZ5MHhtS0xEY2ZTSjBCS05RTm1kQWl6MWw4QTU2RnhLZm5WTWtFVkg5UFh1OGdZdDNIVWE5ejRCQ3dNeUE?oc=5</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>Chinesa CMOC compra operações da Equinox e produzirá ouro no Brasil - Valor Econômico</t>
+          <t>China CMOC compra quatro minas de ouro no Brasil por 863 milhões de euros - RTP</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxNdjJLdXR0TWF1WVRBWGpwZW5vUlAtZk9scmFlMUxKbWxpcUVKZ2ZkNGJqZXhCVENIRVpaRlBPWE9ycnJteDJnbW1WcmZUVjVJOG9DTjF0andnXzMweFV0anRSLXdjVUllZ3JvYUNLU1U3SnFoRWx4Z21OVnFNQ05nWDZaVVRBQnoxMFVSYm5PQ3AyZlVqdmpabzNCY25qZVE0VkI4NGlKVGEzd3RncWNtX0swakhzYjh5WUktLUx2bjdrQkHSAdIBQVVfeXFMTndraVAxVThDT0d6d0xTbVdRa25WdENfanhibkVOamNHaVFMR3VJQWp4b1RiVmFaRXFGQmIwLUZHVTlTdHcxWnZhZERhRWRyRmhBUFlmakVxRHYtZVJNNW5OS1JuZ0xyVXdWVFVSdDU3NmN5MWt4Zmw2R01fR2ZMNG5fVDB0LVNtRENfdlNZS2hmSGg0a2xES1p4aDdzMk1RODRWaHBjVVE0MXNLcWRfMGJuSHZ2SVhZcHcyZnQ5eVN6UXhkd2ZhZGdzeDc0UzRFUkln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQV0FjeGVtTGVqd2VhNU5fanJxQVlOSWI5ckFnZTFhLVgtdjZQNXlzUUFIYVJhS285THFzZjRiNUw4QnJJcENRVmtQT3l0NUVzR3c0UzlnT3I0anItNXprX0Qzd1R2b000V3Bya3NsSVVtMi16U2JQaERkcFZQRVFxalA1cTByWEVjTzZKQjc5RHZrdWdncy1zWEh6ZURSTFJXWG1HdlE1cV9iLXpMRG1sVWl4R0ltNDF5VHVJ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>Chinesa CMOC fecha compra de minas de ouro brasileiras da Equinox Gold por US$ 1 bilhão - InvestNews - InvestNews</t>
+          <t>Agência de Comunicação - Equinox Gold vende operações no Brasil para chinesa CMOC por US$ 1,015 bilhão - Estadão Blue Studio</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPS0o5bC02RWVGMFNDRlFMV2huMEcyaGwwdTVPdjRUWEVwSk1RZGJGbWR5NG5aVnRGSzFzQTVJZUsxdHRvMVh1dU9zRTVvYVVmb0dzU2dkZUtuMzRFMXlmc2NEaEo3aFBQdy05RVpmNmd6dmpMQWctTERZNmVvYThyX3VaNTdGWTNZMlpKNk9HbXFXd3N3QzJFM2VfS3NvWklUQ21LbXBNR3NqdUtMcnhSdnhJR3lHVjdS0gG-AUFVX3lxTFBsRW5abk9ZQlFxd2dvV3ZhbFByOVFqNFBQWmROcEFfMGFHaWhrdkgxYmUzbGJPbmtFQXdTMzNINlJsNUNRTm1TZ3FyVXlURDRHT1hpakVxSXZqV3V3OEVEMUpwdFF1a2R3bXdKcEk4Zi1QUFJUcHQtcmQ5SUpOVkVYRVVtT1hMTDQyQmN3SDZfRDQ3c2ZEMGNHYWR3ajRWdDF3YlZNQjRGV2tpM3dORUNHeFNxcm1oOUFia1NQeUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTDRHMUtOeFVXOTk1NlEzYnRSVU04ZUltZW5TVWQybFZQdmFwdGV0YkdqMVk0VXQ5YXJHQmpXelZyUDlUcTZLNFA1NnlXS3NLX1pSYXlUaV8xbkdxSktMcHlma3VWMXRFSWZMbGRobU1NX1pyeGRSd0d6VXZvS0N6azZ0NklzWnloN0w2ZnFod045RFRfWloxa3Z4QlhFTE5YQTR4WnpnRUNBUTBtZWFRRW5IRk9MVDA?oc=5</t>
         </is>
       </c>
     </row>
@@ -10390,7 +10390,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>Equinox vende minas de ouro no Brasil por US$ 1 bilhão para focar na América do Norte - Times Brasil | CNBC</t>
+          <t>Empresa chinesa compra minas de ouro no Brasil e amplia presença global - Revista Oeste</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
@@ -10400,7 +10400,7 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNR28ySFpHMzJDeW0xM3dXcXktU19yeVBESW1qVXF3dDA0dThMVkZ2WXFiT2J5ak5ZUjdzQW16Q0Z3dE5PZm9MVEkyb3F0MndOSDZTM2RhUFlBX2VTdVozR0ZaTHc2Y3d5M3JWdF9vNjJ6aGJXNko5RThyZjByeWtlSFRNdE1JZFdhVUUzVVBoUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQNzRxZEFqRTNNS3dablR5U2liLVhrbUZOVThwYUhwUGFrdWR1eWcwWHJGckxoWG5JNHY3V3hDZjhaRTRvX2wtaFRkdnJjdFUyZ1BlRjdCV2oxMTA1ZUxlYnlXOHY4ZjFxMGl2ODZDaUM2VWJhcWVjbE4wUWxPLVRxejFzaWduNnlGUFUzOGEzSE9CckhDUFBhTG5xNjJZSGR5OU1UUmtHblAtUQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10412,7 +10412,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>Grupo chinês CMOC fecha compra bilionária de minas de ouro no Brasil - Claudio Dantas</t>
+          <t>Chinesa CMOC fecha compra de minas de ouro brasileiras da Equinox Gold por US$ 1 bilhão - InvestNews - InvestNews</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE9ZTnZqV1dXYWtXTm9wUHlLcGVQVDdSdjdmU0lvOEFFakVKSTZLWnBRQ3gxdUpVSkMzOS1SbU5HM1lJOW9yRXFlYXhSUlJPZnNOVWJuY2hBQjFmN2E1VkRnV0pvcG8tX3hIeFZTWTRJR2NBUnk1S0p3Ul92LVFnQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPS0o5bC02RWVGMFNDRlFMV2huMEcyaGwwdTVPdjRUWEVwSk1RZGJGbWR5NG5aVnRGSzFzQTVJZUsxdHRvMVh1dU9zRTVvYVVmb0dzU2dkZUtuMzRFMXlmc2NEaEo3aFBQdy05RVpmNmd6dmpMQWctTERZNmVvYThyX3VaNTdGWTNZMlpKNk9HbXFXd3N3QzJFM2VfS3NvWklUQ21LbXBNR3NqdUtMcnhSdnhJR3lHVjdS0gG-AUFVX3lxTFBsRW5abk9ZQlFxd2dvV3ZhbFByOVFqNFBQWmROcEFfMGFHaWhrdkgxYmUzbGJPbmtFQXdTMzNINlJsNUNRTm1TZ3FyVXlURDRHT1hpakVxSXZqV3V3OEVEMUpwdFF1a2R3bXdKcEk4Zi1QUFJUcHQtcmQ5SUpOVkVYRVVtT1hMTDQyQmN3SDZfRDQ3c2ZEMGNHYWR3ajRWdDF3YlZNQjRGV2tpM3dORUNHeFNxcm1oOUFia1NQeUE?oc=5</t>
         </is>
       </c>
     </row>
@@ -10434,7 +10434,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>Gigante chinesa CMOC gasta US$ 1 bilhão para abocanhar minas de ouro no Brasil, derruba concorrentes, turbina produção a 8 toneladas por ano e avança pesado no controle de metais preciosos na América do Sul - CPG Click Petróleo e Gás</t>
+          <t>Equinox vende minas de ouro no Brasil por US$ 1 bilhão para focar na América do Norte - Times Brasil | CNBC</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
@@ -10444,7 +10444,7 @@
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxNWGl1NS0wZzJVbG9BZ2ozUlFlOHNnejMwdXNFNFFnQm5majZCLWFkQ3ROc1JSX0hJaUdBbzhPUFJTalpCYTBKZkNjY25Sa0Y1OW9zcUkzY3ROZW4zYVRnMHJ0THlMYVJRUEt1ajBaMGwySm4xVkNlakw5ZW8yUER0MFBjcnhJazF2ZnNxVFVvamJGcHI1QWpscVAxS0x1M0I4OXYxUFhxaWpZX2RSVDZ4aXFBMXRScmV6cmNqbU5UMFlQRTJfMHBKS1RHWC03LW1IZkhvSFNQUWlpR0QxdzduRHFEZFlvNTJBTzJqUjZ0cmFLenZ1MWE2Yy1FX0NTS1VIcFVNU01QZEc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNR28ySFpHMzJDeW0xM3dXcXktU19yeVBESW1qVXF3dDA0dThMVkZ2WXFiT2J5ak5ZUjdzQW16Q0Z3dE5PZm9MVEkyb3F0MndOSDZTM2RhUFlBX2VTdVozR0ZaTHc2Y3d5M3JWdF9vNjJ6aGJXNko5RThyZjByeWtlSFRNdE1JZFdhVUUzVVBoUQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10456,7 +10456,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>Empresa chinesa compra minas de ouro no Brasil e amplia presença global - Revista Oeste</t>
+          <t>Grupo chinês CMOC fecha compra bilionária de minas de ouro no Brasil - Claudio Dantas</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQNzRxZEFqRTNNS3dablR5U2liLVhrbUZOVThwYUhwUGFrdWR1eWcwWHJGckxoWG5JNHY3V3hDZjhaRTRvX2wtaFRkdnJjdFUyZ1BlRjdCV2oxMTA1ZUxlYnlXOHY4ZjFxMGl2ODZDaUM2VWJhcWVjbE4wUWxPLVRxejFzaWduNnlGUFUzOGEzSE9CckhDUFBhTG5xNjJZSGR5OU1UUmtHblAtUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE9ZTnZqV1dXYWtXTm9wUHlLcGVQVDdSdjdmU0lvOEFFakVKSTZLWnBRQ3gxdUpVSkMzOS1SbU5HM1lJOW9yRXFlYXhSUlJPZnNOVWJuY2hBQjFmN2E1VkRnV0pvcG8tX3hIeFZTWTRJR2NBUnk1S0p3Ul92LVFnQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>Agência de Comunicação - Equinox Gold vende operações no Brasil para chinesa CMOC por US$ 1,015 bilhão - Estadão Blue Studio</t>
+          <t>Gigante chinesa CMOC gasta US$ 1 bilhão para abocanhar minas de ouro no Brasil, derruba concorrentes, turbina produção a 8 toneladas por ano e avança pesado no controle de metais preciosos na América do Sul - CPG Click Petróleo e Gás</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTDRHMUtOeFVXOTk1NlEzYnRSVU04ZUltZW5TVWQybFZQdmFwdGV0YkdqMVk0VXQ5YXJHQmpXelZyUDlUcTZLNFA1NnlXS3NLX1pSYXlUaV8xbkdxSktMcHlma3VWMXRFSWZMbGRobU1NX1pyeGRSd0d6VXZvS0N6azZ0NklzWnloN0w2ZnFod045RFRfWloxa3Z4QlhFTE5YQTR4WnpnRUNBUTBtZWFRRW5IRk9MVDA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxNWGl1NS0wZzJVbG9BZ2ozUlFlOHNnejMwdXNFNFFnQm5majZCLWFkQ3ROc1JSX0hJaUdBbzhPUFJTalpCYTBKZkNjY25Sa0Y1OW9zcUkzY3ROZW4zYVRnMHJ0THlMYVJRUEt1ajBaMGwySm4xVkNlakw5ZW8yUER0MFBjcnhJazF2ZnNxVFVvamJGcHI1QWpscVAxS0x1M0I4OXYxUFhxaWpZX2RSVDZ4aXFBMXRScmV6cmNqbU5UMFlQRTJfMHBKS1RHWC03LW1IZkhvSFNQUWlpR0QxdzduRHFEZFlvNTJBTzJqUjZ0cmFLenZ1MWE2Yy1FX0NTS1VIcFVNU01QZEc?oc=5</t>
         </is>
       </c>
     </row>
@@ -10539,12 +10539,12 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>CMOC</t>
+          <t>Cal Cruzeiro</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>OURO | Equinox Gold vende operações brasileiras para CMOC por US$ 1,015 bilhão - Brasil Mineral</t>
+          <t>E se for para os pênaltis? Quem leva vantagem entre Hugo Souza e Cássio em Corinthians x Cruzeiro na Copa do Brasil - ESPN Brasil</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -10554,7 +10554,7 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPRVJxVWY5aVdLMG85emtjZ04xVG10c3JUSkdSVjdhQko5UUU4S2gtRXdzang5ckZmOHFoYUlqR2huemllR0lOMUQxYVFDWjAwbkIxSUx2ZjhFa1dQbTkyVGh0MlZlb3BWbWMwN2p3TEplUzM4UEpTQWxFckJsMVU0ckJmZXAwbEh6Vm9WbjRyNWhRZGdMRHJBT3ROZ1ZvcWFJYUVGMEVpekZQck9idWlmRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPOWs4S016VVRvTnBGOURieGlCNWlNZjIyX21jOV9HYjlMZGpyLS1LMUx3Nkt0Wm5rc21aMkpSZTlxdHEzLWpRV05XLTRReVFzQTVEazNEb19QSW9PemJwWjhMYWstVkYwVmhzZ1RRMjk5MWtJa2FnUzNzd096MWFHRFZTM013YlNqaXpPUWdEZjlHMGowaW92Qk5RUXZTWUdKbWtuMDg2cTU0eEVmYkNGNnctc2doX09vaFhqejNLNW9CSkt3czBFRFVSam1QdnJUMmcyd290SzgtRW9OY05hdDlacm11LVAx?oc=5</t>
         </is>
       </c>
     </row>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>E se for para os pênaltis? Quem leva vantagem entre Hugo Souza e Cássio em Corinthians x Cruzeiro na Copa do Brasil - ESPN Brasil</t>
+          <t>Cássio iguala Dida em pênaltis defendidos; veja ranking - band.com.br</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPOWs4S016VVRvTnBGOURieGlCNWlNZjIyX21jOV9HYjlMZGpyLS1LMUx3Nkt0Wm5rc21aMkpSZTlxdHEzLWpRV05XLTRReVFzQTVEazNEb19QSW9PemJwWjhMYWstVkYwVmhzZ1RRMjk5MWtJa2FnUzNzd096MWFHRFZTM013YlNqaXpPUWdEZjlHMGowaW92Qk5RUXZTWUdKbWtuMDg2cTU0eEVmYkNGNnctc2doX09vaFhqejNLNW9CSkt3czBFRFVSam1QdnJUMmcyd290SzgtRW9OY05hdDlacm11LVAx?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNMFU4a0ZjNk5fVWV1eGpWbDJ2UjRTUW1rS1RZZWFVVThzMm1nQVFYbDB0dDhHblE4d2R0di1ac3dJUjhBZWlWbTI2d3FsWU15emhnbExQSU54VFprZjJKNE1mWTN3dmlEby1qTnY2dWxvdmlmak9HUU5pajVrVE5yRjRVRm5Ock5Rdnd0b0dxNnk1U2k5RnNGb29DUkhYemRsRFE?oc=5</t>
         </is>
       </c>
     </row>
@@ -10588,7 +10588,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>Chinesa CMOC fecha compra de minas de ouro no Brasil por US$ 1 bilhão - O GLOBO</t>
+          <t>OURO | Equinox Gold vende operações brasileiras para CMOC por US$ 1,015 bilhão - Brasil Mineral</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
@@ -10598,19 +10598,19 @@
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQWGs3cTNKQ1ZUQkw2M1FhQUtBRWVXRENXQlcxTlZZWVQxR3JwakE3VHhLSk85VHJZNW9FRlNZdTJxYWJod1JpZHNzQU5FZmQ4NTBlSHRzYWR2cGdmNUJBbjBfc2g4Z0xCeDhZS2lQUDNkZVM2YlNKUmRsaGRSUXlzaFhVc1VCUjdqdGJ4MVczTDdiXzBJdGY0MGxuRFNPanpMVkNmWllPd1Fubk9Fb3VVVUlQYmtHa05ZZGEzT3hMZFdhZU9YUVHSAdQBQVVfeXFMTnhIOF9JRDZ2d1VLU3lpT050cHpXdkNxTjIxUGJHNFlTbk9zLTRHeWZ2dWZLOVRXNVI4YVNPMVNOelZURVdSMTl5RVRfTU1GdTlZRkl0Y2hsQ1Bzd21yZzRPZ0RtMlZlNlhuRE1TbkdDczVIRTRpdWpfYzh1ZlloTVItWnJXVzN4TnBibDFweERzVDh0anhkajlTT0wyUkRxSWJUckhpSHlpTjY3ejNFRTlEcm4yWWZFM1FxQXRmQkJpVVN2T1JoZXl0WXVwRjlFM0d4QXM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPRVJxVWY5aVdLMG85emtjZ04xVG10c3JUSkdSVjdhQko5UUU4S2gtRXdzang5ckZmOHFoYUlqR2huemllR0lOMUQxYVFDWjAwbkIxSUx2ZjhFa1dQbTkyVGh0MlZlb3BWbWMwN2p3TEplUzM4UEpTQWxFckJsMVU0ckJmZXAwbEh6Vm9WbjRyNWhRZGdMRHJBT3ROZ1ZvcWFJYUVGMEVpekZQck9idWlmRQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>Cal Cruzeiro</t>
+          <t>CMOC</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>Corinthians elimina Cruzeiro pela 3ª vez na história da Copa do Brasil - CNN Brasil</t>
+          <t>Chinesa CMOC fecha compra de minas de ouro no Brasil por US$ 1 bilhão - O GLOBO</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
@@ -10620,7 +10620,7 @@
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQQ1AzUm1KNUYtMGxCaEFfQ05zUzNnemhZblotcVNfdlY2RU9Hd0M3UThGX3JEdHFoRVdFa1BncW9PanJUVHVZSEVzZk8xbmxGRkZqa2lPZWJXQjBQZjhJN04weV96TGFqS0dNNEtUZW9RQWlvNS1UUkpGYmU2ckl0S0RwaEpHR1BCaWFBeUYyeXhXdlhTQkZKRVNRUUg3OVRwTGNYUGtRbmFOVUtpQlBpWk1naHhHSTRNM2V1ZWVtV2xLQ1N3bnRnU1ZoMjA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQWGs3cTNKQ1ZUQkw2M1FhQUtBRWVXRENXQlcxTlZZWVQxR3JwakE3VHhLSk85VHJZNW9FRlNZdTJxYWJod1JpZHNzQU5FZmQ4NTBlSHRzYWR2cGdmNUJBbjBfc2g4Z0xCeDhZS2lQUDNkZVM2YlNKUmRsaGRSUXlzaFhVc1VCUjdqdGJ4MVczTDdiXzBJdGY0MGxuRFNPanpMVkNmWllPd1Fubk9Fb3VVVUlQYmtHa05ZZGEzT3hMZFdhZU9YUVHSAdQBQVVfeXFMTnhIOF9JRDZ2d1VLU3lpT050cHpXdkNxTjIxUGJHNFlTbk9zLTRHeWZ2dWZLOVRXNVI4YVNPMVNOelZURVdSMTl5RVRfTU1GdTlZRkl0Y2hsQ1Bzd21yZzRPZ0RtMlZlNlhuRE1TbkdDczVIRTRpdWpfYzh1ZlloTVItWnJXVzN4TnBibDFweERzVDh0anhkajlTT0wyUkRxSWJUckhpSHlpTjY3ejNFRTlEcm4yWWZFM1FxQXRmQkJpVVN2T1JoZXl0WXVwRjlFM0d4QXM?oc=5</t>
         </is>
       </c>
     </row>
@@ -10632,7 +10632,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>Hugo Souza gigante, Corinthians elimina o Cruzeiro nos pênaltis e está na final da Copa do Brasil - capitalnews.com.br</t>
+          <t>Corinthians elimina Cruzeiro pela 3ª vez na história da Copa do Brasil - CNN Brasil</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
@@ -10642,7 +10642,7 @@
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxQMlJiZVMtX3NqVlBzYzBDUnJPVk5ZWkRYcmszc2FVY2dMTWVkRG8yTDhCU1pxcl9jR0dIN0tKUHFVRVlOblVuOTdpdXlYR2lZSjhSQkpZZ25CSE5VX3Y1bThsa2dnMkpOUEtwVmF2ek5OZXFhZm1CRGF5elZQNW5SV2VjYy0wV1ZTU3hQRmswT1Z1OFRHRG5ydHlvRlEyb2oyekhBbG1uOWdpM1dIZkVXUWNMVy1Rdm9wa3dMMlZyeDZ3SENla2VjR0xqdGt0b3NnTWc2T0hQb2hWc1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQQ1AzUm1KNUYtMGxCaEFfQ05zUzNnemhZblotcVNfdlY2RU9Hd0M3UThGX3JEdHFoRVdFa1BncW9PanJUVHVZSEVzZk8xbmxGRkZqa2lPZWJXQjBQZjhJN04weV96TGFqS0dNNEtUZW9RQWlvNS1UUkpGYmU2ckl0S0RwaEpHR1BCaWFBeUYyeXhXdlhTQkZKRVNRUUg3OVRwTGNYUGtRbmFOVUtpQlBpWk1naHhHSTRNM2V1ZWVtV2xLQ1N3bnRnU1ZoMjA?oc=5</t>
         </is>
       </c>
     </row>
@@ -10654,7 +10654,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>Corinthians vence o Cruzeiro nos pênaltis e vai à final da Copa do Brasil - band.com.br</t>
+          <t>Hugo Souza gigante, Corinthians elimina o Cruzeiro nos pênaltis e está na final da Copa do Brasil - capitalnews.com.br</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPV1d5dEFNd0t1ME9tQWJSWWRzLWtuckNpd25abG9vcUJ3czlmcl9xLTQxQmE4Ni1udEFTRDBFZUd3VWFMMU5McWlELUtoTG50dTZTeXY2SmtJMXdObllneDBuV1JLbXdscG1NTzhRLTJMSExGQjNxSkF3WjBuS0dkaXBYdTR0WW1DeDBQdVBvUzlmZ1JQM2pSVDhqdEFCdXlXWjZqSlhoT3ZjeVNMZGtobGdsTlBoWUpZVGlv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxQMlJiZVMtX3NqVlBzYzBDUnJPVk5ZWkRYcmszc2FVY2dMTWVkRG8yTDhCU1pxcl9jR0dIN0tKUHFVRVlOblVuOTdpdXlYR2lZSjhSQkpZZ25CSE5VX3Y1bThsa2dnMkpOUEtwVmF2ek5OZXFhZm1CRGF5elZQNW5SV2VjYy0wV1ZTU3hQRmswT1Z1OFRHRG5ydHlvRlEyb2oyekhBbG1uOWdpM1dIZkVXUWNMVy1Rdm9wa3dMMlZyeDZ3SENla2VjR0xqdGt0b3NnTWc2T0hQb2hWc1E?oc=5</t>
         </is>
       </c>
     </row>
@@ -10676,7 +10676,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>Cássio iguala Dida em pênaltis defendidos; veja ranking - band.com.br</t>
+          <t>Corinthians vence o Cruzeiro nos pênaltis e vai à final da Copa do Brasil - band.com.br</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
@@ -10686,7 +10686,7 @@
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNMFU4a0ZjNk5fVWV1eGpWbDJ2UjRTUW1rS1RZZWFVVThzMm1nQVFYbDB0dDhHblE4d2R0di1ac3dJUjhBZWlWbTI2d3FsWU15emhnbExQSU54VFprZjJKNE1mWTN3dmlEby1qTnY2dWxvdmlmak9HUU5pajVrVE5yRjRVRm5Ock5Rdnd0b0dxNnk1U2k5RnNGb29DUkhYemRsRFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPV1d5dEFNd0t1ME9tQWJSWWRzLWtuckNpd25abG9vcUJ3czlmcl9xLTQxQmE4Ni1udEFTRDBFZUd3VWFMMU5McWlELUtoTG50dTZTeXY2SmtJMXdObllneDBuV1JLbXdscG1NTzhRLTJMSExGQjNxSkF3WjBuS0dkaXBYdTR0WW1DeDBQdVBvUzlmZ1JQM2pSVDhqdEFCdXlXWjZqSlhoT3ZjeVNMZGtobGdsTlBoWUpZVGlv?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>